<commit_message>
FIX: Corrected RGB FPGA comparison csv and png.
</commit_message>
<xml_diff>
--- a/FPGA_Performance_Comparison_RGB.xlsx
+++ b/FPGA_Performance_Comparison_RGB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/DanielBiswas/Desktop/Documents/University/Year 5/Semester 1/AMME4112/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2BD9A6D-4DEA-504C-9F59-5EA9C97352DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17FD29B5-04C4-9C4B-A111-4375D66E1867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10500" yWindow="-28200" windowWidth="51200" windowHeight="28200" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17840" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -325,19 +325,19 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -685,28 +685,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
+      <c r="B1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
       <c r="E1" s="6"/>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G1" s="9"/>
+      <c r="G1" s="10"/>
       <c r="H1" s="6"/>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="9"/>
+      <c r="J1" s="10"/>
       <c r="K1" s="6"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="10"/>
+      <c r="A2" s="13"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1699,22 +1699,22 @@
       <c r="B33" s="1">
         <v>36.935268000000001</v>
       </c>
-      <c r="C33" s="9">
+      <c r="C33" s="10">
         <v>35.655293</v>
       </c>
-      <c r="D33" s="9"/>
+      <c r="D33" s="10"/>
       <c r="E33" s="6"/>
-      <c r="F33" s="9">
+      <c r="F33" s="10">
         <f>C33-B33</f>
         <v>-1.2799750000000003</v>
       </c>
-      <c r="G33" s="9"/>
+      <c r="G33" s="10"/>
       <c r="H33" s="6"/>
-      <c r="I33" s="11">
+      <c r="I33" s="9">
         <f>F33/B33</f>
         <v>-3.4654547518106552E-2</v>
       </c>
-      <c r="J33" s="11"/>
+      <c r="J33" s="9"/>
       <c r="K33" s="6"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
@@ -1724,22 +1724,22 @@
       <c r="B34" s="1">
         <v>4.1183040000000002</v>
       </c>
-      <c r="C34" s="9">
+      <c r="C34" s="10">
         <v>4.0647320000000002</v>
       </c>
-      <c r="D34" s="9"/>
+      <c r="D34" s="10"/>
       <c r="E34" s="6"/>
-      <c r="F34" s="9">
+      <c r="F34" s="10">
         <f t="shared" ref="F34:F44" si="8">C34-B34</f>
         <v>-5.3571999999999953E-2</v>
       </c>
-      <c r="G34" s="9"/>
+      <c r="G34" s="10"/>
       <c r="H34" s="6"/>
-      <c r="I34" s="11">
+      <c r="I34" s="9">
         <f t="shared" ref="I34:I44" si="9">F34/B34</f>
         <v>-1.300826748098245E-2</v>
       </c>
-      <c r="J34" s="11"/>
+      <c r="J34" s="9"/>
       <c r="K34" s="6"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
@@ -1749,22 +1749,22 @@
       <c r="B35" s="1">
         <v>2</v>
       </c>
-      <c r="C35" s="9">
+      <c r="C35" s="10">
         <v>2</v>
       </c>
-      <c r="D35" s="9"/>
+      <c r="D35" s="10"/>
       <c r="E35" s="6"/>
-      <c r="F35" s="9">
+      <c r="F35" s="10">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G35" s="9"/>
+      <c r="G35" s="10"/>
       <c r="H35" s="6"/>
-      <c r="I35" s="11">
+      <c r="I35" s="9">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J35" s="11"/>
+      <c r="J35" s="9"/>
       <c r="K35" s="6"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
@@ -1774,22 +1774,22 @@
       <c r="B36" s="1">
         <v>2</v>
       </c>
-      <c r="C36" s="9">
+      <c r="C36" s="10">
         <v>2</v>
       </c>
-      <c r="D36" s="9"/>
+      <c r="D36" s="10"/>
       <c r="E36" s="6"/>
-      <c r="F36" s="9">
+      <c r="F36" s="10">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G36" s="9"/>
+      <c r="G36" s="10"/>
       <c r="H36" s="6"/>
-      <c r="I36" s="11">
+      <c r="I36" s="9">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J36" s="11"/>
+      <c r="J36" s="9"/>
       <c r="K36" s="6"/>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
@@ -1799,21 +1799,21 @@
       <c r="B37" s="1">
         <v>0</v>
       </c>
-      <c r="C37" s="9">
-        <v>0</v>
-      </c>
-      <c r="D37" s="9"/>
+      <c r="C37" s="10">
+        <v>0</v>
+      </c>
+      <c r="D37" s="10"/>
       <c r="E37" s="6"/>
-      <c r="F37" s="9">
+      <c r="F37" s="10">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G37" s="9"/>
+      <c r="G37" s="10"/>
       <c r="H37" s="6"/>
-      <c r="I37" s="11" t="s">
+      <c r="I37" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="J37" s="11"/>
+      <c r="J37" s="9"/>
       <c r="K37" s="6"/>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
@@ -1823,22 +1823,22 @@
       <c r="B38" s="1">
         <v>23</v>
       </c>
-      <c r="C38" s="9">
+      <c r="C38" s="10">
         <v>23</v>
       </c>
-      <c r="D38" s="9"/>
+      <c r="D38" s="10"/>
       <c r="E38" s="6"/>
-      <c r="F38" s="9">
+      <c r="F38" s="10">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G38" s="9"/>
+      <c r="G38" s="10"/>
       <c r="H38" s="6"/>
-      <c r="I38" s="11">
+      <c r="I38" s="9">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J38" s="11"/>
+      <c r="J38" s="9"/>
       <c r="K38" s="6"/>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
@@ -1848,22 +1848,22 @@
       <c r="B39" s="1">
         <v>6.6195789999999999</v>
       </c>
-      <c r="C39" s="9">
+      <c r="C39" s="10">
         <v>6.6183040000000002</v>
       </c>
-      <c r="D39" s="9"/>
+      <c r="D39" s="10"/>
       <c r="E39" s="6"/>
-      <c r="F39" s="9">
+      <c r="F39" s="10">
         <f t="shared" si="8"/>
         <v>-1.274999999999693E-3</v>
       </c>
-      <c r="G39" s="9"/>
+      <c r="G39" s="10"/>
       <c r="H39" s="6"/>
-      <c r="I39" s="11">
+      <c r="I39" s="9">
         <f t="shared" si="9"/>
         <v>-1.9261043640383973E-4</v>
       </c>
-      <c r="J39" s="11"/>
+      <c r="J39" s="9"/>
       <c r="K39" s="6"/>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
@@ -1873,22 +1873,22 @@
       <c r="B40" s="1">
         <v>7</v>
       </c>
-      <c r="C40" s="9">
+      <c r="C40" s="10">
         <v>7</v>
       </c>
-      <c r="D40" s="9"/>
+      <c r="D40" s="10"/>
       <c r="E40" s="6"/>
-      <c r="F40" s="9">
+      <c r="F40" s="10">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G40" s="9"/>
+      <c r="G40" s="10"/>
       <c r="H40" s="6"/>
-      <c r="I40" s="11">
+      <c r="I40" s="9">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J40" s="11"/>
+      <c r="J40" s="9"/>
       <c r="K40" s="6"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
@@ -1898,22 +1898,22 @@
       <c r="B41" s="1">
         <v>8</v>
       </c>
-      <c r="C41" s="9">
+      <c r="C41" s="10">
         <v>8</v>
       </c>
-      <c r="D41" s="9"/>
+      <c r="D41" s="10"/>
       <c r="E41" s="6"/>
-      <c r="F41" s="9">
+      <c r="F41" s="10">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G41" s="9"/>
+      <c r="G41" s="10"/>
       <c r="H41" s="6"/>
-      <c r="I41" s="11">
+      <c r="I41" s="9">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J41" s="11"/>
+      <c r="J41" s="9"/>
       <c r="K41" s="6"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
@@ -1923,22 +1923,22 @@
       <c r="B42" s="1">
         <v>3</v>
       </c>
-      <c r="C42" s="9">
+      <c r="C42" s="10">
         <v>3</v>
       </c>
-      <c r="D42" s="9"/>
+      <c r="D42" s="10"/>
       <c r="E42" s="6"/>
-      <c r="F42" s="9">
+      <c r="F42" s="10">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G42" s="9"/>
+      <c r="G42" s="10"/>
       <c r="H42" s="6"/>
-      <c r="I42" s="11">
+      <c r="I42" s="9">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J42" s="11"/>
+      <c r="J42" s="9"/>
       <c r="K42" s="6"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
@@ -1948,22 +1948,22 @@
       <c r="B43" s="1">
         <v>471</v>
       </c>
-      <c r="C43" s="9">
+      <c r="C43" s="10">
         <v>455</v>
       </c>
-      <c r="D43" s="9"/>
+      <c r="D43" s="10"/>
       <c r="E43" s="6"/>
-      <c r="F43" s="9">
+      <c r="F43" s="10">
         <f t="shared" si="8"/>
         <v>-16</v>
       </c>
-      <c r="G43" s="9"/>
+      <c r="G43" s="10"/>
       <c r="H43" s="6"/>
-      <c r="I43" s="11">
+      <c r="I43" s="9">
         <f t="shared" si="9"/>
         <v>-3.3970276008492568E-2</v>
       </c>
-      <c r="J43" s="11"/>
+      <c r="J43" s="9"/>
       <c r="K43" s="6"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
@@ -1973,22 +1973,22 @@
       <c r="B44" s="5">
         <v>0.15019133000000001</v>
       </c>
-      <c r="C44" s="13">
+      <c r="C44" s="12">
         <v>0.14508929000000001</v>
       </c>
-      <c r="D44" s="13"/>
+      <c r="D44" s="12"/>
       <c r="E44" s="6"/>
-      <c r="F44" s="9">
+      <c r="F44" s="10">
         <f t="shared" si="8"/>
         <v>-5.1020400000000021E-3</v>
       </c>
-      <c r="G44" s="9"/>
+      <c r="G44" s="10"/>
       <c r="H44" s="6"/>
-      <c r="I44" s="11">
+      <c r="I44" s="9">
         <f t="shared" si="9"/>
         <v>-3.3970269788542402E-2</v>
       </c>
-      <c r="J44" s="11"/>
+      <c r="J44" s="9"/>
       <c r="K44" s="6"/>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
@@ -2011,22 +2011,22 @@
       <c r="B46" s="1">
         <v>3.401786</v>
       </c>
-      <c r="C46" s="9">
+      <c r="C46" s="10">
         <v>3.4068879999999999</v>
       </c>
-      <c r="D46" s="9"/>
+      <c r="D46" s="10"/>
       <c r="E46" s="6"/>
-      <c r="F46" s="9">
+      <c r="F46" s="10">
         <f>C46-B46</f>
         <v>5.1019999999999399E-3</v>
       </c>
-      <c r="G46" s="9"/>
+      <c r="G46" s="10"/>
       <c r="H46" s="6"/>
-      <c r="I46" s="11">
+      <c r="I46" s="9">
         <f t="shared" ref="I46" si="10">F46/B46</f>
         <v>1.4998003989668779E-3</v>
       </c>
-      <c r="J46" s="11"/>
+      <c r="J46" s="9"/>
       <c r="K46" s="6"/>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
@@ -2036,22 +2036,22 @@
       <c r="B47" s="1">
         <v>1.770408</v>
       </c>
-      <c r="C47" s="9">
+      <c r="C47" s="10">
         <v>1.772321</v>
       </c>
-      <c r="D47" s="9"/>
+      <c r="D47" s="10"/>
       <c r="E47" s="6"/>
-      <c r="F47" s="9">
+      <c r="F47" s="10">
         <f t="shared" ref="F47:F57" si="11">C47-B47</f>
         <v>1.9130000000000535E-3</v>
       </c>
-      <c r="G47" s="9"/>
+      <c r="G47" s="10"/>
       <c r="H47" s="6"/>
-      <c r="I47" s="11">
+      <c r="I47" s="9">
         <f t="shared" ref="I47:I57" si="12">F47/B47</f>
         <v>1.0805418863900601E-3</v>
       </c>
-      <c r="J47" s="11"/>
+      <c r="J47" s="9"/>
       <c r="K47" s="6"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
@@ -2061,22 +2061,22 @@
       <c r="B48" s="1">
         <v>2</v>
       </c>
-      <c r="C48" s="9">
+      <c r="C48" s="10">
         <v>2</v>
       </c>
-      <c r="D48" s="9"/>
+      <c r="D48" s="10"/>
       <c r="E48" s="6"/>
-      <c r="F48" s="9">
+      <c r="F48" s="10">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G48" s="9"/>
+      <c r="G48" s="10"/>
       <c r="H48" s="6"/>
-      <c r="I48" s="11">
+      <c r="I48" s="9">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J48" s="11"/>
+      <c r="J48" s="9"/>
       <c r="K48" s="6"/>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
@@ -2086,22 +2086,22 @@
       <c r="B49" s="1">
         <v>-2</v>
       </c>
-      <c r="C49" s="9">
+      <c r="C49" s="10">
         <v>-2</v>
       </c>
-      <c r="D49" s="9"/>
+      <c r="D49" s="10"/>
       <c r="E49" s="6"/>
-      <c r="F49" s="9">
+      <c r="F49" s="10">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G49" s="9"/>
+      <c r="G49" s="10"/>
       <c r="H49" s="6"/>
-      <c r="I49" s="11">
+      <c r="I49" s="9">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J49" s="11"/>
+      <c r="J49" s="9"/>
       <c r="K49" s="6"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.2">
@@ -2111,22 +2111,22 @@
       <c r="B50" s="1">
         <v>-3</v>
       </c>
-      <c r="C50" s="9">
+      <c r="C50" s="10">
         <v>-3</v>
       </c>
-      <c r="D50" s="9"/>
+      <c r="D50" s="10"/>
       <c r="E50" s="6"/>
-      <c r="F50" s="9">
+      <c r="F50" s="10">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G50" s="9"/>
+      <c r="G50" s="10"/>
       <c r="H50" s="6"/>
-      <c r="I50" s="11">
+      <c r="I50" s="9">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J50" s="11"/>
+      <c r="J50" s="9"/>
       <c r="K50" s="6"/>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.2">
@@ -2136,22 +2136,22 @@
       <c r="B51" s="1">
         <v>2</v>
       </c>
-      <c r="C51" s="9">
+      <c r="C51" s="10">
         <v>2</v>
       </c>
-      <c r="D51" s="9"/>
+      <c r="D51" s="10"/>
       <c r="E51" s="6"/>
-      <c r="F51" s="9">
+      <c r="F51" s="10">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G51" s="9"/>
+      <c r="G51" s="10"/>
       <c r="H51" s="6"/>
-      <c r="I51" s="11">
+      <c r="I51" s="9">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J51" s="11"/>
+      <c r="J51" s="9"/>
       <c r="K51" s="6"/>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
@@ -2161,22 +2161,22 @@
       <c r="B52" s="1">
         <v>6.7904970000000002</v>
       </c>
-      <c r="C52" s="9">
+      <c r="C52" s="10">
         <v>6.78986</v>
       </c>
-      <c r="D52" s="9"/>
+      <c r="D52" s="10"/>
       <c r="E52" s="6"/>
-      <c r="F52" s="9">
+      <c r="F52" s="10">
         <f t="shared" si="11"/>
         <v>-6.3700000000022072E-4</v>
       </c>
-      <c r="G52" s="9"/>
+      <c r="G52" s="10"/>
       <c r="H52" s="6"/>
-      <c r="I52" s="11">
+      <c r="I52" s="9">
         <f t="shared" si="12"/>
         <v>-9.3807566662678849E-5</v>
       </c>
-      <c r="J52" s="11"/>
+      <c r="J52" s="9"/>
       <c r="K52" s="6"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.2">
@@ -2186,22 +2186,22 @@
       <c r="B53" s="1">
         <v>7</v>
       </c>
-      <c r="C53" s="9">
+      <c r="C53" s="10">
         <v>7</v>
       </c>
-      <c r="D53" s="9"/>
+      <c r="D53" s="10"/>
       <c r="E53" s="6"/>
-      <c r="F53" s="9">
+      <c r="F53" s="10">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G53" s="9"/>
+      <c r="G53" s="10"/>
       <c r="H53" s="6"/>
-      <c r="I53" s="11">
+      <c r="I53" s="9">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J53" s="11"/>
+      <c r="J53" s="9"/>
       <c r="K53" s="6"/>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.2">
@@ -2211,22 +2211,22 @@
       <c r="B54" s="1">
         <v>8</v>
       </c>
-      <c r="C54" s="9">
+      <c r="C54" s="10">
         <v>8</v>
       </c>
-      <c r="D54" s="9"/>
+      <c r="D54" s="10"/>
       <c r="E54" s="6"/>
-      <c r="F54" s="9">
+      <c r="F54" s="10">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G54" s="9"/>
+      <c r="G54" s="10"/>
       <c r="H54" s="6"/>
-      <c r="I54" s="11">
+      <c r="I54" s="9">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J54" s="11"/>
+      <c r="J54" s="9"/>
       <c r="K54" s="6"/>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.2">
@@ -2236,22 +2236,22 @@
       <c r="B55" s="1">
         <v>5</v>
       </c>
-      <c r="C55" s="9">
+      <c r="C55" s="10">
         <v>5</v>
       </c>
-      <c r="D55" s="9"/>
+      <c r="D55" s="10"/>
       <c r="E55" s="6"/>
-      <c r="F55" s="9">
+      <c r="F55" s="10">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G55" s="9"/>
+      <c r="G55" s="10"/>
       <c r="H55" s="6"/>
-      <c r="I55" s="11">
+      <c r="I55" s="9">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J55" s="11"/>
+      <c r="J55" s="9"/>
       <c r="K55" s="6"/>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.2">
@@ -2261,22 +2261,22 @@
       <c r="B56" s="1">
         <v>61</v>
       </c>
-      <c r="C56" s="9">
+      <c r="C56" s="10">
         <v>60</v>
       </c>
-      <c r="D56" s="9"/>
+      <c r="D56" s="10"/>
       <c r="E56" s="6"/>
-      <c r="F56" s="9">
+      <c r="F56" s="10">
         <f t="shared" si="11"/>
         <v>-1</v>
       </c>
-      <c r="G56" s="9"/>
+      <c r="G56" s="10"/>
       <c r="H56" s="6"/>
-      <c r="I56" s="11">
+      <c r="I56" s="9">
         <f t="shared" si="12"/>
         <v>-1.6393442622950821E-2</v>
       </c>
-      <c r="J56" s="11"/>
+      <c r="J56" s="9"/>
       <c r="K56" s="6"/>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.2">
@@ -2286,22 +2286,22 @@
       <c r="B57" s="5">
         <v>1.9451530000000002E-2</v>
       </c>
-      <c r="C57" s="11">
+      <c r="C57" s="9">
         <v>1.9132650000000001E-2</v>
       </c>
-      <c r="D57" s="11"/>
+      <c r="D57" s="9"/>
       <c r="E57" s="6"/>
-      <c r="F57" s="9">
+      <c r="F57" s="10">
         <f t="shared" si="11"/>
         <v>-3.1888000000000055E-4</v>
       </c>
-      <c r="G57" s="9"/>
+      <c r="G57" s="10"/>
       <c r="H57" s="6"/>
-      <c r="I57" s="11">
+      <c r="I57" s="9">
         <f t="shared" si="12"/>
         <v>-1.6393569040584494E-2</v>
       </c>
-      <c r="J57" s="11"/>
+      <c r="J57" s="9"/>
       <c r="K57" s="6"/>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.2">
@@ -2321,143 +2321,143 @@
       <c r="A59" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B59" s="9" t="s">
+      <c r="B59" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="C59" s="9"/>
-      <c r="D59" s="9"/>
+      <c r="C59" s="10"/>
+      <c r="D59" s="10"/>
       <c r="E59" s="6"/>
-      <c r="F59" s="9">
-        <v>0</v>
-      </c>
-      <c r="G59" s="9"/>
+      <c r="F59" s="10">
+        <v>0</v>
+      </c>
+      <c r="G59" s="10"/>
       <c r="H59" s="6"/>
-      <c r="I59" s="12">
-        <v>0</v>
-      </c>
-      <c r="J59" s="12"/>
+      <c r="I59" s="11">
+        <v>0</v>
+      </c>
+      <c r="J59" s="11"/>
       <c r="K59" s="6"/>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="9">
+      <c r="B60" s="10">
         <v>1</v>
       </c>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="10"/>
       <c r="E60" s="6"/>
-      <c r="F60" s="9">
-        <v>0</v>
-      </c>
-      <c r="G60" s="9"/>
+      <c r="F60" s="10">
+        <v>0</v>
+      </c>
+      <c r="G60" s="10"/>
       <c r="H60" s="6"/>
-      <c r="I60" s="11">
+      <c r="I60" s="9">
         <f t="shared" ref="I60:I68" si="13">F60/B60</f>
         <v>0</v>
       </c>
-      <c r="J60" s="11"/>
+      <c r="J60" s="9"/>
       <c r="K60" s="6"/>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="9">
+      <c r="B61" s="10">
         <v>69633</v>
       </c>
-      <c r="C61" s="9"/>
-      <c r="D61" s="9"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="10"/>
       <c r="E61" s="6"/>
-      <c r="F61" s="9">
-        <v>0</v>
-      </c>
-      <c r="G61" s="9"/>
+      <c r="F61" s="10">
+        <v>0</v>
+      </c>
+      <c r="G61" s="10"/>
       <c r="H61" s="6"/>
-      <c r="I61" s="11">
+      <c r="I61" s="9">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J61" s="11"/>
+      <c r="J61" s="9"/>
       <c r="K61" s="6"/>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B62" s="9">
+      <c r="B62" s="10">
         <v>70352</v>
       </c>
-      <c r="C62" s="9"/>
-      <c r="D62" s="9"/>
+      <c r="C62" s="10"/>
+      <c r="D62" s="10"/>
       <c r="E62" s="6"/>
-      <c r="F62" s="9">
-        <v>0</v>
-      </c>
-      <c r="G62" s="9"/>
+      <c r="F62" s="10">
+        <v>0</v>
+      </c>
+      <c r="G62" s="10"/>
       <c r="H62" s="6"/>
-      <c r="I62" s="11">
+      <c r="I62" s="9">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J62" s="11"/>
+      <c r="J62" s="9"/>
       <c r="K62" s="6"/>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B63" s="9">
+      <c r="B63" s="10">
         <v>73927</v>
       </c>
-      <c r="C63" s="9"/>
-      <c r="D63" s="9"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="10"/>
       <c r="E63" s="6"/>
-      <c r="F63" s="9">
-        <v>0</v>
-      </c>
-      <c r="G63" s="9"/>
+      <c r="F63" s="10">
+        <v>0</v>
+      </c>
+      <c r="G63" s="10"/>
       <c r="H63" s="6"/>
-      <c r="I63" s="11">
+      <c r="I63" s="9">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J63" s="11"/>
+      <c r="J63" s="9"/>
       <c r="K63" s="6"/>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B64" s="9">
+      <c r="B64" s="10">
         <f>B63-B60</f>
         <v>73926</v>
       </c>
-      <c r="C64" s="9"/>
-      <c r="D64" s="9"/>
+      <c r="C64" s="10"/>
+      <c r="D64" s="10"/>
       <c r="E64" s="6"/>
-      <c r="F64" s="9">
-        <v>0</v>
-      </c>
-      <c r="G64" s="9"/>
+      <c r="F64" s="10">
+        <v>0</v>
+      </c>
+      <c r="G64" s="10"/>
       <c r="H64" s="6"/>
-      <c r="I64" s="11">
+      <c r="I64" s="9">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J64" s="11"/>
+      <c r="J64" s="9"/>
       <c r="K64" s="6"/>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B65" s="9">
+      <c r="B65" s="10">
         <f>B64/(B3*10^3)</f>
         <v>0.98568</v>
       </c>
-      <c r="C65" s="9"/>
+      <c r="C65" s="10"/>
       <c r="D65" s="1">
         <f>B64/(D3*10^3)</f>
         <v>0.37910769230769231</v>
@@ -2467,7 +2467,7 @@
         <v>0</v>
       </c>
       <c r="G65" s="1">
-        <f t="shared" ref="G60:G68" si="14">D65-B65</f>
+        <f t="shared" ref="G65:G68" si="14">D65-B65</f>
         <v>-0.60657230769230774</v>
       </c>
       <c r="H65" s="6"/>
@@ -2475,7 +2475,7 @@
         <v>0</v>
       </c>
       <c r="J65" s="5">
-        <f t="shared" ref="J60:J68" si="15">G65/B65</f>
+        <f t="shared" ref="J65:J68" si="15">G65/B65</f>
         <v>-0.61538461538461542</v>
       </c>
       <c r="K65" s="6"/>
@@ -2484,34 +2484,34 @@
       <c r="A66" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B66" s="9">
+      <c r="B66" s="10">
         <f>B63-B61</f>
         <v>4294</v>
       </c>
-      <c r="C66" s="9"/>
-      <c r="D66" s="9"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="10"/>
       <c r="E66" s="6"/>
-      <c r="F66" s="9">
-        <v>0</v>
-      </c>
-      <c r="G66" s="9"/>
+      <c r="F66" s="10">
+        <v>0</v>
+      </c>
+      <c r="G66" s="10"/>
       <c r="H66" s="6"/>
-      <c r="I66" s="11">
+      <c r="I66" s="9">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J66" s="11"/>
+      <c r="J66" s="9"/>
       <c r="K66" s="6"/>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B67" s="9">
+      <c r="B67" s="10">
         <f>B66/B3</f>
         <v>57.25333333333333</v>
       </c>
-      <c r="C67" s="9"/>
+      <c r="C67" s="10"/>
       <c r="D67" s="1">
         <f>B66/D3</f>
         <v>22.02051282051282</v>
@@ -2543,8 +2543,8 @@
         <v>954.97606800000005</v>
       </c>
       <c r="C68" s="1">
-        <f t="shared" ref="C68:D68" si="16">C12*C65</f>
-        <v>0</v>
+        <f>C12*B65</f>
+        <v>946.92306239999994</v>
       </c>
       <c r="D68" s="1">
         <f>D12*D65</f>
@@ -2552,8 +2552,8 @@
       </c>
       <c r="E68" s="6"/>
       <c r="F68" s="1">
-        <f t="shared" ref="F60:F68" si="17">C68-B68</f>
-        <v>-954.97606800000005</v>
+        <f t="shared" ref="F68" si="16">C68-B68</f>
+        <v>-8.0530056000001196</v>
       </c>
       <c r="G68" s="1">
         <f t="shared" si="14"/>
@@ -2562,7 +2562,7 @@
       <c r="H68" s="6"/>
       <c r="I68" s="5">
         <f t="shared" si="13"/>
-        <v>-1</v>
+        <v>-8.4326779171183582E-3</v>
       </c>
       <c r="J68" s="5">
         <f t="shared" si="15"/>
@@ -2585,30 +2585,65 @@
     </row>
   </sheetData>
   <mergeCells count="99">
-    <mergeCell ref="I54:J54"/>
-    <mergeCell ref="I55:J55"/>
-    <mergeCell ref="I56:J56"/>
-    <mergeCell ref="I57:J57"/>
-    <mergeCell ref="I49:J49"/>
-    <mergeCell ref="I50:J50"/>
-    <mergeCell ref="I51:J51"/>
-    <mergeCell ref="I52:J52"/>
-    <mergeCell ref="I53:J53"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="F61:G61"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="F64:G64"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="I66:J66"/>
+    <mergeCell ref="I64:J64"/>
+    <mergeCell ref="I63:J63"/>
+    <mergeCell ref="I62:J62"/>
+    <mergeCell ref="I61:J61"/>
+    <mergeCell ref="I60:J60"/>
+    <mergeCell ref="I59:J59"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="C53:D53"/>
+    <mergeCell ref="C54:D54"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="C49:D49"/>
     <mergeCell ref="C55:D55"/>
     <mergeCell ref="C56:D56"/>
     <mergeCell ref="C57:D57"/>
@@ -2625,65 +2660,30 @@
     <mergeCell ref="F56:G56"/>
     <mergeCell ref="F57:G57"/>
     <mergeCell ref="C50:D50"/>
-    <mergeCell ref="C51:D51"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="C53:D53"/>
-    <mergeCell ref="C54:D54"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="C48:D48"/>
-    <mergeCell ref="C49:D49"/>
-    <mergeCell ref="I60:J60"/>
-    <mergeCell ref="I59:J59"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="I66:J66"/>
-    <mergeCell ref="I64:J64"/>
-    <mergeCell ref="I63:J63"/>
-    <mergeCell ref="I62:J62"/>
-    <mergeCell ref="I61:J61"/>
-    <mergeCell ref="B66:D66"/>
-    <mergeCell ref="F59:G59"/>
-    <mergeCell ref="F60:G60"/>
-    <mergeCell ref="F61:G61"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="F64:G64"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="B60:D60"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="B62:D62"/>
-    <mergeCell ref="B63:D63"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="I54:J54"/>
+    <mergeCell ref="I55:J55"/>
+    <mergeCell ref="I56:J56"/>
+    <mergeCell ref="I57:J57"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="I51:J51"/>
+    <mergeCell ref="I52:J52"/>
+    <mergeCell ref="I53:J53"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
UPDATE: Added information and corrected excel spreadsheets.
</commit_message>
<xml_diff>
--- a/FPGA_Performance_Comparison_RGB.xlsx
+++ b/FPGA_Performance_Comparison_RGB.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/DanielBiswas/Desktop/Documents/University/Year 5/Semester 1/AMME4112/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17FD29B5-04C4-9C4B-A111-4375D66E1867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B67F714D-CC8B-214D-8923-062CFC2C5C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17840" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17760" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="71">
   <si>
     <t>FPGA Implementation</t>
   </si>
@@ -246,6 +246,9 @@
   </si>
   <si>
     <t>Light Field Dimensions (Sub-Apertures, Length, Width)</t>
+  </si>
+  <si>
+    <t>Max Throughput (FPS)</t>
   </si>
 </sst>
 </file>
@@ -325,19 +328,19 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -675,7 +678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A45085A3-2BCA-FA4F-9A9B-A0D6975F9A68}">
-  <dimension ref="A1:K69"/>
+  <dimension ref="A1:K70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="50.83203125" style="3" customWidth="1"/>
@@ -685,28 +688,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
       <c r="E1" s="6"/>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G1" s="10"/>
+      <c r="G1" s="9"/>
       <c r="H1" s="6"/>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="10"/>
+      <c r="J1" s="9"/>
       <c r="K1" s="6"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="13"/>
+      <c r="A2" s="10"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1699,22 +1702,22 @@
       <c r="B33" s="1">
         <v>36.935268000000001</v>
       </c>
-      <c r="C33" s="10">
+      <c r="C33" s="9">
         <v>35.655293</v>
       </c>
-      <c r="D33" s="10"/>
+      <c r="D33" s="9"/>
       <c r="E33" s="6"/>
-      <c r="F33" s="10">
+      <c r="F33" s="9">
         <f>C33-B33</f>
         <v>-1.2799750000000003</v>
       </c>
-      <c r="G33" s="10"/>
+      <c r="G33" s="9"/>
       <c r="H33" s="6"/>
-      <c r="I33" s="9">
+      <c r="I33" s="11">
         <f>F33/B33</f>
         <v>-3.4654547518106552E-2</v>
       </c>
-      <c r="J33" s="9"/>
+      <c r="J33" s="11"/>
       <c r="K33" s="6"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
@@ -1724,22 +1727,22 @@
       <c r="B34" s="1">
         <v>4.1183040000000002</v>
       </c>
-      <c r="C34" s="10">
+      <c r="C34" s="9">
         <v>4.0647320000000002</v>
       </c>
-      <c r="D34" s="10"/>
+      <c r="D34" s="9"/>
       <c r="E34" s="6"/>
-      <c r="F34" s="10">
+      <c r="F34" s="9">
         <f t="shared" ref="F34:F44" si="8">C34-B34</f>
         <v>-5.3571999999999953E-2</v>
       </c>
-      <c r="G34" s="10"/>
+      <c r="G34" s="9"/>
       <c r="H34" s="6"/>
-      <c r="I34" s="9">
+      <c r="I34" s="11">
         <f t="shared" ref="I34:I44" si="9">F34/B34</f>
         <v>-1.300826748098245E-2</v>
       </c>
-      <c r="J34" s="9"/>
+      <c r="J34" s="11"/>
       <c r="K34" s="6"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
@@ -1749,22 +1752,22 @@
       <c r="B35" s="1">
         <v>2</v>
       </c>
-      <c r="C35" s="10">
+      <c r="C35" s="9">
         <v>2</v>
       </c>
-      <c r="D35" s="10"/>
+      <c r="D35" s="9"/>
       <c r="E35" s="6"/>
-      <c r="F35" s="10">
+      <c r="F35" s="9">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G35" s="10"/>
+      <c r="G35" s="9"/>
       <c r="H35" s="6"/>
-      <c r="I35" s="9">
+      <c r="I35" s="11">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J35" s="9"/>
+      <c r="J35" s="11"/>
       <c r="K35" s="6"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
@@ -1774,22 +1777,22 @@
       <c r="B36" s="1">
         <v>2</v>
       </c>
-      <c r="C36" s="10">
+      <c r="C36" s="9">
         <v>2</v>
       </c>
-      <c r="D36" s="10"/>
+      <c r="D36" s="9"/>
       <c r="E36" s="6"/>
-      <c r="F36" s="10">
+      <c r="F36" s="9">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G36" s="10"/>
+      <c r="G36" s="9"/>
       <c r="H36" s="6"/>
-      <c r="I36" s="9">
+      <c r="I36" s="11">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J36" s="9"/>
+      <c r="J36" s="11"/>
       <c r="K36" s="6"/>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
@@ -1799,21 +1802,21 @@
       <c r="B37" s="1">
         <v>0</v>
       </c>
-      <c r="C37" s="10">
-        <v>0</v>
-      </c>
-      <c r="D37" s="10"/>
+      <c r="C37" s="9">
+        <v>0</v>
+      </c>
+      <c r="D37" s="9"/>
       <c r="E37" s="6"/>
-      <c r="F37" s="10">
+      <c r="F37" s="9">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G37" s="10"/>
+      <c r="G37" s="9"/>
       <c r="H37" s="6"/>
-      <c r="I37" s="9" t="s">
+      <c r="I37" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="J37" s="9"/>
+      <c r="J37" s="11"/>
       <c r="K37" s="6"/>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
@@ -1823,22 +1826,22 @@
       <c r="B38" s="1">
         <v>23</v>
       </c>
-      <c r="C38" s="10">
+      <c r="C38" s="9">
         <v>23</v>
       </c>
-      <c r="D38" s="10"/>
+      <c r="D38" s="9"/>
       <c r="E38" s="6"/>
-      <c r="F38" s="10">
+      <c r="F38" s="9">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G38" s="10"/>
+      <c r="G38" s="9"/>
       <c r="H38" s="6"/>
-      <c r="I38" s="9">
+      <c r="I38" s="11">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J38" s="9"/>
+      <c r="J38" s="11"/>
       <c r="K38" s="6"/>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
@@ -1848,22 +1851,22 @@
       <c r="B39" s="1">
         <v>6.6195789999999999</v>
       </c>
-      <c r="C39" s="10">
+      <c r="C39" s="9">
         <v>6.6183040000000002</v>
       </c>
-      <c r="D39" s="10"/>
+      <c r="D39" s="9"/>
       <c r="E39" s="6"/>
-      <c r="F39" s="10">
+      <c r="F39" s="9">
         <f t="shared" si="8"/>
         <v>-1.274999999999693E-3</v>
       </c>
-      <c r="G39" s="10"/>
+      <c r="G39" s="9"/>
       <c r="H39" s="6"/>
-      <c r="I39" s="9">
+      <c r="I39" s="11">
         <f t="shared" si="9"/>
         <v>-1.9261043640383973E-4</v>
       </c>
-      <c r="J39" s="9"/>
+      <c r="J39" s="11"/>
       <c r="K39" s="6"/>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
@@ -1873,22 +1876,22 @@
       <c r="B40" s="1">
         <v>7</v>
       </c>
-      <c r="C40" s="10">
+      <c r="C40" s="9">
         <v>7</v>
       </c>
-      <c r="D40" s="10"/>
+      <c r="D40" s="9"/>
       <c r="E40" s="6"/>
-      <c r="F40" s="10">
+      <c r="F40" s="9">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G40" s="10"/>
+      <c r="G40" s="9"/>
       <c r="H40" s="6"/>
-      <c r="I40" s="9">
+      <c r="I40" s="11">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J40" s="9"/>
+      <c r="J40" s="11"/>
       <c r="K40" s="6"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
@@ -1898,22 +1901,22 @@
       <c r="B41" s="1">
         <v>8</v>
       </c>
-      <c r="C41" s="10">
+      <c r="C41" s="9">
         <v>8</v>
       </c>
-      <c r="D41" s="10"/>
+      <c r="D41" s="9"/>
       <c r="E41" s="6"/>
-      <c r="F41" s="10">
+      <c r="F41" s="9">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G41" s="10"/>
+      <c r="G41" s="9"/>
       <c r="H41" s="6"/>
-      <c r="I41" s="9">
+      <c r="I41" s="11">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J41" s="9"/>
+      <c r="J41" s="11"/>
       <c r="K41" s="6"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
@@ -1923,22 +1926,22 @@
       <c r="B42" s="1">
         <v>3</v>
       </c>
-      <c r="C42" s="10">
+      <c r="C42" s="9">
         <v>3</v>
       </c>
-      <c r="D42" s="10"/>
+      <c r="D42" s="9"/>
       <c r="E42" s="6"/>
-      <c r="F42" s="10">
+      <c r="F42" s="9">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G42" s="10"/>
+      <c r="G42" s="9"/>
       <c r="H42" s="6"/>
-      <c r="I42" s="9">
+      <c r="I42" s="11">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="J42" s="9"/>
+      <c r="J42" s="11"/>
       <c r="K42" s="6"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
@@ -1948,22 +1951,22 @@
       <c r="B43" s="1">
         <v>471</v>
       </c>
-      <c r="C43" s="10">
+      <c r="C43" s="9">
         <v>455</v>
       </c>
-      <c r="D43" s="10"/>
+      <c r="D43" s="9"/>
       <c r="E43" s="6"/>
-      <c r="F43" s="10">
+      <c r="F43" s="9">
         <f t="shared" si="8"/>
         <v>-16</v>
       </c>
-      <c r="G43" s="10"/>
+      <c r="G43" s="9"/>
       <c r="H43" s="6"/>
-      <c r="I43" s="9">
+      <c r="I43" s="11">
         <f t="shared" si="9"/>
         <v>-3.3970276008492568E-2</v>
       </c>
-      <c r="J43" s="9"/>
+      <c r="J43" s="11"/>
       <c r="K43" s="6"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
@@ -1973,22 +1976,22 @@
       <c r="B44" s="5">
         <v>0.15019133000000001</v>
       </c>
-      <c r="C44" s="12">
+      <c r="C44" s="13">
         <v>0.14508929000000001</v>
       </c>
-      <c r="D44" s="12"/>
+      <c r="D44" s="13"/>
       <c r="E44" s="6"/>
-      <c r="F44" s="10">
+      <c r="F44" s="9">
         <f t="shared" si="8"/>
         <v>-5.1020400000000021E-3</v>
       </c>
-      <c r="G44" s="10"/>
+      <c r="G44" s="9"/>
       <c r="H44" s="6"/>
-      <c r="I44" s="9">
+      <c r="I44" s="11">
         <f t="shared" si="9"/>
         <v>-3.3970269788542402E-2</v>
       </c>
-      <c r="J44" s="9"/>
+      <c r="J44" s="11"/>
       <c r="K44" s="6"/>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
@@ -2011,22 +2014,22 @@
       <c r="B46" s="1">
         <v>3.401786</v>
       </c>
-      <c r="C46" s="10">
+      <c r="C46" s="9">
         <v>3.4068879999999999</v>
       </c>
-      <c r="D46" s="10"/>
+      <c r="D46" s="9"/>
       <c r="E46" s="6"/>
-      <c r="F46" s="10">
+      <c r="F46" s="9">
         <f>C46-B46</f>
         <v>5.1019999999999399E-3</v>
       </c>
-      <c r="G46" s="10"/>
+      <c r="G46" s="9"/>
       <c r="H46" s="6"/>
-      <c r="I46" s="9">
+      <c r="I46" s="11">
         <f t="shared" ref="I46" si="10">F46/B46</f>
         <v>1.4998003989668779E-3</v>
       </c>
-      <c r="J46" s="9"/>
+      <c r="J46" s="11"/>
       <c r="K46" s="6"/>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
@@ -2036,22 +2039,22 @@
       <c r="B47" s="1">
         <v>1.770408</v>
       </c>
-      <c r="C47" s="10">
+      <c r="C47" s="9">
         <v>1.772321</v>
       </c>
-      <c r="D47" s="10"/>
+      <c r="D47" s="9"/>
       <c r="E47" s="6"/>
-      <c r="F47" s="10">
+      <c r="F47" s="9">
         <f t="shared" ref="F47:F57" si="11">C47-B47</f>
         <v>1.9130000000000535E-3</v>
       </c>
-      <c r="G47" s="10"/>
+      <c r="G47" s="9"/>
       <c r="H47" s="6"/>
-      <c r="I47" s="9">
+      <c r="I47" s="11">
         <f t="shared" ref="I47:I57" si="12">F47/B47</f>
         <v>1.0805418863900601E-3</v>
       </c>
-      <c r="J47" s="9"/>
+      <c r="J47" s="11"/>
       <c r="K47" s="6"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
@@ -2061,22 +2064,22 @@
       <c r="B48" s="1">
         <v>2</v>
       </c>
-      <c r="C48" s="10">
+      <c r="C48" s="9">
         <v>2</v>
       </c>
-      <c r="D48" s="10"/>
+      <c r="D48" s="9"/>
       <c r="E48" s="6"/>
-      <c r="F48" s="10">
+      <c r="F48" s="9">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G48" s="10"/>
+      <c r="G48" s="9"/>
       <c r="H48" s="6"/>
-      <c r="I48" s="9">
+      <c r="I48" s="11">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J48" s="9"/>
+      <c r="J48" s="11"/>
       <c r="K48" s="6"/>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
@@ -2086,22 +2089,22 @@
       <c r="B49" s="1">
         <v>-2</v>
       </c>
-      <c r="C49" s="10">
+      <c r="C49" s="9">
         <v>-2</v>
       </c>
-      <c r="D49" s="10"/>
+      <c r="D49" s="9"/>
       <c r="E49" s="6"/>
-      <c r="F49" s="10">
+      <c r="F49" s="9">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G49" s="10"/>
+      <c r="G49" s="9"/>
       <c r="H49" s="6"/>
-      <c r="I49" s="9">
+      <c r="I49" s="11">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J49" s="9"/>
+      <c r="J49" s="11"/>
       <c r="K49" s="6"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.2">
@@ -2111,22 +2114,22 @@
       <c r="B50" s="1">
         <v>-3</v>
       </c>
-      <c r="C50" s="10">
+      <c r="C50" s="9">
         <v>-3</v>
       </c>
-      <c r="D50" s="10"/>
+      <c r="D50" s="9"/>
       <c r="E50" s="6"/>
-      <c r="F50" s="10">
+      <c r="F50" s="9">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G50" s="10"/>
+      <c r="G50" s="9"/>
       <c r="H50" s="6"/>
-      <c r="I50" s="9">
+      <c r="I50" s="11">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J50" s="9"/>
+      <c r="J50" s="11"/>
       <c r="K50" s="6"/>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.2">
@@ -2136,22 +2139,22 @@
       <c r="B51" s="1">
         <v>2</v>
       </c>
-      <c r="C51" s="10">
+      <c r="C51" s="9">
         <v>2</v>
       </c>
-      <c r="D51" s="10"/>
+      <c r="D51" s="9"/>
       <c r="E51" s="6"/>
-      <c r="F51" s="10">
+      <c r="F51" s="9">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G51" s="10"/>
+      <c r="G51" s="9"/>
       <c r="H51" s="6"/>
-      <c r="I51" s="9">
+      <c r="I51" s="11">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J51" s="9"/>
+      <c r="J51" s="11"/>
       <c r="K51" s="6"/>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
@@ -2161,22 +2164,22 @@
       <c r="B52" s="1">
         <v>6.7904970000000002</v>
       </c>
-      <c r="C52" s="10">
+      <c r="C52" s="9">
         <v>6.78986</v>
       </c>
-      <c r="D52" s="10"/>
+      <c r="D52" s="9"/>
       <c r="E52" s="6"/>
-      <c r="F52" s="10">
+      <c r="F52" s="9">
         <f t="shared" si="11"/>
         <v>-6.3700000000022072E-4</v>
       </c>
-      <c r="G52" s="10"/>
+      <c r="G52" s="9"/>
       <c r="H52" s="6"/>
-      <c r="I52" s="9">
+      <c r="I52" s="11">
         <f t="shared" si="12"/>
         <v>-9.3807566662678849E-5</v>
       </c>
-      <c r="J52" s="9"/>
+      <c r="J52" s="11"/>
       <c r="K52" s="6"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.2">
@@ -2186,22 +2189,22 @@
       <c r="B53" s="1">
         <v>7</v>
       </c>
-      <c r="C53" s="10">
+      <c r="C53" s="9">
         <v>7</v>
       </c>
-      <c r="D53" s="10"/>
+      <c r="D53" s="9"/>
       <c r="E53" s="6"/>
-      <c r="F53" s="10">
+      <c r="F53" s="9">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G53" s="10"/>
+      <c r="G53" s="9"/>
       <c r="H53" s="6"/>
-      <c r="I53" s="9">
+      <c r="I53" s="11">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J53" s="9"/>
+      <c r="J53" s="11"/>
       <c r="K53" s="6"/>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.2">
@@ -2211,22 +2214,22 @@
       <c r="B54" s="1">
         <v>8</v>
       </c>
-      <c r="C54" s="10">
+      <c r="C54" s="9">
         <v>8</v>
       </c>
-      <c r="D54" s="10"/>
+      <c r="D54" s="9"/>
       <c r="E54" s="6"/>
-      <c r="F54" s="10">
+      <c r="F54" s="9">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G54" s="10"/>
+      <c r="G54" s="9"/>
       <c r="H54" s="6"/>
-      <c r="I54" s="9">
+      <c r="I54" s="11">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J54" s="9"/>
+      <c r="J54" s="11"/>
       <c r="K54" s="6"/>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.2">
@@ -2236,22 +2239,22 @@
       <c r="B55" s="1">
         <v>5</v>
       </c>
-      <c r="C55" s="10">
+      <c r="C55" s="9">
         <v>5</v>
       </c>
-      <c r="D55" s="10"/>
+      <c r="D55" s="9"/>
       <c r="E55" s="6"/>
-      <c r="F55" s="10">
+      <c r="F55" s="9">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="G55" s="10"/>
+      <c r="G55" s="9"/>
       <c r="H55" s="6"/>
-      <c r="I55" s="9">
+      <c r="I55" s="11">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J55" s="9"/>
+      <c r="J55" s="11"/>
       <c r="K55" s="6"/>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.2">
@@ -2261,22 +2264,22 @@
       <c r="B56" s="1">
         <v>61</v>
       </c>
-      <c r="C56" s="10">
+      <c r="C56" s="9">
         <v>60</v>
       </c>
-      <c r="D56" s="10"/>
+      <c r="D56" s="9"/>
       <c r="E56" s="6"/>
-      <c r="F56" s="10">
+      <c r="F56" s="9">
         <f t="shared" si="11"/>
         <v>-1</v>
       </c>
-      <c r="G56" s="10"/>
+      <c r="G56" s="9"/>
       <c r="H56" s="6"/>
-      <c r="I56" s="9">
+      <c r="I56" s="11">
         <f t="shared" si="12"/>
         <v>-1.6393442622950821E-2</v>
       </c>
-      <c r="J56" s="9"/>
+      <c r="J56" s="11"/>
       <c r="K56" s="6"/>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.2">
@@ -2286,22 +2289,22 @@
       <c r="B57" s="5">
         <v>1.9451530000000002E-2</v>
       </c>
-      <c r="C57" s="9">
+      <c r="C57" s="11">
         <v>1.9132650000000001E-2</v>
       </c>
-      <c r="D57" s="9"/>
+      <c r="D57" s="11"/>
       <c r="E57" s="6"/>
-      <c r="F57" s="10">
+      <c r="F57" s="9">
         <f t="shared" si="11"/>
         <v>-3.1888000000000055E-4</v>
       </c>
-      <c r="G57" s="10"/>
+      <c r="G57" s="9"/>
       <c r="H57" s="6"/>
-      <c r="I57" s="9">
+      <c r="I57" s="11">
         <f t="shared" si="12"/>
         <v>-1.6393569040584494E-2</v>
       </c>
-      <c r="J57" s="9"/>
+      <c r="J57" s="11"/>
       <c r="K57" s="6"/>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.2">
@@ -2321,143 +2324,143 @@
       <c r="A59" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B59" s="10" t="s">
+      <c r="B59" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C59" s="10"/>
-      <c r="D59" s="10"/>
+      <c r="C59" s="9"/>
+      <c r="D59" s="9"/>
       <c r="E59" s="6"/>
-      <c r="F59" s="10">
-        <v>0</v>
-      </c>
-      <c r="G59" s="10"/>
+      <c r="F59" s="9">
+        <v>0</v>
+      </c>
+      <c r="G59" s="9"/>
       <c r="H59" s="6"/>
-      <c r="I59" s="11">
-        <v>0</v>
-      </c>
-      <c r="J59" s="11"/>
+      <c r="I59" s="12">
+        <v>0</v>
+      </c>
+      <c r="J59" s="12"/>
       <c r="K59" s="6"/>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="10">
+      <c r="B60" s="9">
         <v>1</v>
       </c>
-      <c r="C60" s="10"/>
-      <c r="D60" s="10"/>
+      <c r="C60" s="9"/>
+      <c r="D60" s="9"/>
       <c r="E60" s="6"/>
-      <c r="F60" s="10">
-        <v>0</v>
-      </c>
-      <c r="G60" s="10"/>
+      <c r="F60" s="9">
+        <v>0</v>
+      </c>
+      <c r="G60" s="9"/>
       <c r="H60" s="6"/>
-      <c r="I60" s="9">
+      <c r="I60" s="11">
         <f t="shared" ref="I60:I68" si="13">F60/B60</f>
         <v>0</v>
       </c>
-      <c r="J60" s="9"/>
+      <c r="J60" s="11"/>
       <c r="K60" s="6"/>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="10">
+      <c r="B61" s="9">
         <v>69633</v>
       </c>
-      <c r="C61" s="10"/>
-      <c r="D61" s="10"/>
+      <c r="C61" s="9"/>
+      <c r="D61" s="9"/>
       <c r="E61" s="6"/>
-      <c r="F61" s="10">
-        <v>0</v>
-      </c>
-      <c r="G61" s="10"/>
+      <c r="F61" s="9">
+        <v>0</v>
+      </c>
+      <c r="G61" s="9"/>
       <c r="H61" s="6"/>
-      <c r="I61" s="9">
+      <c r="I61" s="11">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J61" s="9"/>
+      <c r="J61" s="11"/>
       <c r="K61" s="6"/>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B62" s="10">
+      <c r="B62" s="9">
         <v>70352</v>
       </c>
-      <c r="C62" s="10"/>
-      <c r="D62" s="10"/>
+      <c r="C62" s="9"/>
+      <c r="D62" s="9"/>
       <c r="E62" s="6"/>
-      <c r="F62" s="10">
-        <v>0</v>
-      </c>
-      <c r="G62" s="10"/>
+      <c r="F62" s="9">
+        <v>0</v>
+      </c>
+      <c r="G62" s="9"/>
       <c r="H62" s="6"/>
-      <c r="I62" s="9">
+      <c r="I62" s="11">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J62" s="9"/>
+      <c r="J62" s="11"/>
       <c r="K62" s="6"/>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B63" s="10">
+      <c r="B63" s="9">
         <v>73927</v>
       </c>
-      <c r="C63" s="10"/>
-      <c r="D63" s="10"/>
+      <c r="C63" s="9"/>
+      <c r="D63" s="9"/>
       <c r="E63" s="6"/>
-      <c r="F63" s="10">
-        <v>0</v>
-      </c>
-      <c r="G63" s="10"/>
+      <c r="F63" s="9">
+        <v>0</v>
+      </c>
+      <c r="G63" s="9"/>
       <c r="H63" s="6"/>
-      <c r="I63" s="9">
+      <c r="I63" s="11">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J63" s="9"/>
+      <c r="J63" s="11"/>
       <c r="K63" s="6"/>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B64" s="10">
+      <c r="B64" s="9">
         <f>B63-B60</f>
         <v>73926</v>
       </c>
-      <c r="C64" s="10"/>
-      <c r="D64" s="10"/>
+      <c r="C64" s="9"/>
+      <c r="D64" s="9"/>
       <c r="E64" s="6"/>
-      <c r="F64" s="10">
-        <v>0</v>
-      </c>
-      <c r="G64" s="10"/>
+      <c r="F64" s="9">
+        <v>0</v>
+      </c>
+      <c r="G64" s="9"/>
       <c r="H64" s="6"/>
-      <c r="I64" s="9">
+      <c r="I64" s="11">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J64" s="9"/>
+      <c r="J64" s="11"/>
       <c r="K64" s="6"/>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B65" s="10">
+      <c r="B65" s="9">
         <f>B64/(B3*10^3)</f>
         <v>0.98568</v>
       </c>
-      <c r="C65" s="10"/>
+      <c r="C65" s="9"/>
       <c r="D65" s="1">
         <f>B64/(D3*10^3)</f>
         <v>0.37910769230769231</v>
@@ -2467,7 +2470,7 @@
         <v>0</v>
       </c>
       <c r="G65" s="1">
-        <f t="shared" ref="G65:G68" si="14">D65-B65</f>
+        <f t="shared" ref="G65:G69" si="14">D65-B65</f>
         <v>-0.60657230769230774</v>
       </c>
       <c r="H65" s="6"/>
@@ -2475,7 +2478,7 @@
         <v>0</v>
       </c>
       <c r="J65" s="5">
-        <f t="shared" ref="J65:J68" si="15">G65/B65</f>
+        <f t="shared" ref="J65:J69" si="15">G65/B65</f>
         <v>-0.61538461538461542</v>
       </c>
       <c r="K65" s="6"/>
@@ -2484,34 +2487,34 @@
       <c r="A66" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B66" s="10">
+      <c r="B66" s="9">
         <f>B63-B61</f>
         <v>4294</v>
       </c>
-      <c r="C66" s="10"/>
-      <c r="D66" s="10"/>
+      <c r="C66" s="9"/>
+      <c r="D66" s="9"/>
       <c r="E66" s="6"/>
-      <c r="F66" s="10">
-        <v>0</v>
-      </c>
-      <c r="G66" s="10"/>
+      <c r="F66" s="9">
+        <v>0</v>
+      </c>
+      <c r="G66" s="9"/>
       <c r="H66" s="6"/>
-      <c r="I66" s="9">
+      <c r="I66" s="11">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="J66" s="9"/>
+      <c r="J66" s="11"/>
       <c r="K66" s="6"/>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B67" s="10">
+      <c r="B67" s="9">
         <f>B66/B3</f>
         <v>57.25333333333333</v>
       </c>
-      <c r="C67" s="10"/>
+      <c r="C67" s="9"/>
       <c r="D67" s="1">
         <f>B66/D3</f>
         <v>22.02051282051282</v>
@@ -2571,55 +2574,91 @@
       <c r="K68" s="6"/>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A69" s="7"/>
-      <c r="B69" s="8"/>
-      <c r="C69" s="8"/>
-      <c r="D69" s="8"/>
+      <c r="A69" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B69" s="9">
+        <f>1/(B65/1000)</f>
+        <v>1014.5280415550685</v>
+      </c>
+      <c r="C69" s="9"/>
+      <c r="D69" s="1">
+        <f>1/(D65/1000)</f>
+        <v>2637.7729080431786</v>
+      </c>
       <c r="E69" s="6"/>
-      <c r="F69" s="8"/>
-      <c r="G69" s="8"/>
+      <c r="F69" s="1">
+        <v>0</v>
+      </c>
+      <c r="G69" s="1">
+        <f t="shared" si="14"/>
+        <v>1623.2448664881101</v>
+      </c>
       <c r="H69" s="6"/>
-      <c r="I69" s="8"/>
-      <c r="J69" s="8"/>
+      <c r="I69" s="5">
+        <v>0</v>
+      </c>
+      <c r="J69" s="5">
+        <f t="shared" si="15"/>
+        <v>1.6000000000000005</v>
+      </c>
       <c r="K69" s="6"/>
     </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A70" s="7"/>
+      <c r="B70" s="8"/>
+      <c r="C70" s="8"/>
+      <c r="D70" s="8"/>
+      <c r="E70" s="6"/>
+      <c r="F70" s="8"/>
+      <c r="G70" s="8"/>
+      <c r="H70" s="6"/>
+      <c r="I70" s="8"/>
+      <c r="J70" s="8"/>
+      <c r="K70" s="6"/>
+    </row>
   </sheetData>
-  <mergeCells count="99">
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="B66:D66"/>
-    <mergeCell ref="F59:G59"/>
-    <mergeCell ref="F60:G60"/>
-    <mergeCell ref="F61:G61"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="F64:G64"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="B60:D60"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="B62:D62"/>
-    <mergeCell ref="B63:D63"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="I66:J66"/>
-    <mergeCell ref="I64:J64"/>
-    <mergeCell ref="I63:J63"/>
-    <mergeCell ref="I62:J62"/>
-    <mergeCell ref="I61:J61"/>
-    <mergeCell ref="I60:J60"/>
+  <mergeCells count="100">
+    <mergeCell ref="I57:J57"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="I51:J51"/>
+    <mergeCell ref="I52:J52"/>
+    <mergeCell ref="I53:J53"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="I54:J54"/>
+    <mergeCell ref="I55:J55"/>
+    <mergeCell ref="I56:J56"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="C55:D55"/>
+    <mergeCell ref="C56:D56"/>
+    <mergeCell ref="C57:D57"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="F54:G54"/>
+    <mergeCell ref="F55:G55"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="F57:G57"/>
+    <mergeCell ref="C50:D50"/>
     <mergeCell ref="I59:J59"/>
     <mergeCell ref="B67:C67"/>
     <mergeCell ref="B65:C65"/>
@@ -2644,46 +2683,42 @@
     <mergeCell ref="C47:D47"/>
     <mergeCell ref="C48:D48"/>
     <mergeCell ref="C49:D49"/>
-    <mergeCell ref="C55:D55"/>
-    <mergeCell ref="C56:D56"/>
-    <mergeCell ref="C57:D57"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="F49:G49"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="F52:G52"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="F54:G54"/>
-    <mergeCell ref="F55:G55"/>
-    <mergeCell ref="F56:G56"/>
-    <mergeCell ref="F57:G57"/>
-    <mergeCell ref="C50:D50"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="I54:J54"/>
-    <mergeCell ref="I55:J55"/>
-    <mergeCell ref="I56:J56"/>
-    <mergeCell ref="I57:J57"/>
-    <mergeCell ref="I49:J49"/>
-    <mergeCell ref="I50:J50"/>
-    <mergeCell ref="I51:J51"/>
-    <mergeCell ref="I52:J52"/>
-    <mergeCell ref="I53:J53"/>
+    <mergeCell ref="F64:G64"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="I66:J66"/>
+    <mergeCell ref="I64:J64"/>
+    <mergeCell ref="I63:J63"/>
+    <mergeCell ref="I62:J62"/>
+    <mergeCell ref="I61:J61"/>
+    <mergeCell ref="I60:J60"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="F61:G61"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="F63:G63"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
UPDATE: WIP - Updated excel.
</commit_message>
<xml_diff>
--- a/FPGA_Performance_Comparison_RGB.xlsx
+++ b/FPGA_Performance_Comparison_RGB.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA795196-7082-C141-AFB9-906B9776AE42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="24100" windowHeight="26900" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="24100" windowHeight="17760" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -332,7 +332,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -365,22 +365,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -728,15 +722,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
+      <c r="B1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
       <c r="F1" s="6"/>
       <c r="G1" s="11" t="s">
         <v>55</v>
@@ -752,7 +746,7 @@
       <c r="N1" s="6"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A2" s="12"/>
+      <c r="A2" s="14"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2024,27 +2018,27 @@
       <c r="N32" s="6"/>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A33" s="15" t="s">
+      <c r="A33" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B33" s="16" t="s">
+      <c r="B33" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11"/>
       <c r="F33" s="6"/>
-      <c r="G33" s="16" t="s">
+      <c r="G33" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="H33" s="16"/>
-      <c r="I33" s="16"/>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11"/>
       <c r="J33" s="6"/>
-      <c r="K33" s="16" t="s">
+      <c r="K33" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="L33" s="16"/>
-      <c r="M33" s="16"/>
+      <c r="L33" s="11"/>
+      <c r="M33" s="11"/>
       <c r="N33" s="6"/>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.2">
@@ -2361,11 +2355,11 @@
       <c r="B45" s="5">
         <v>0.15019133000000001</v>
       </c>
-      <c r="C45" s="14">
+      <c r="C45" s="12">
         <v>0.14508929000000001</v>
       </c>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="12"/>
       <c r="F45" s="6"/>
       <c r="G45" s="11">
         <f t="shared" si="7"/>
@@ -2399,27 +2393,27 @@
       <c r="N46" s="6"/>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A47" s="15" t="s">
+      <c r="A47" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B47" s="16" t="s">
+      <c r="B47" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C47" s="16"/>
-      <c r="D47" s="16"/>
-      <c r="E47" s="16"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="11"/>
       <c r="F47" s="6"/>
-      <c r="G47" s="16" t="s">
+      <c r="G47" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="H47" s="16"/>
-      <c r="I47" s="16"/>
+      <c r="H47" s="11"/>
+      <c r="I47" s="11"/>
       <c r="J47" s="6"/>
-      <c r="K47" s="16" t="s">
+      <c r="K47" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="L47" s="16"/>
-      <c r="M47" s="16"/>
+      <c r="L47" s="11"/>
+      <c r="M47" s="11"/>
       <c r="N47" s="6"/>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.2">
@@ -2775,27 +2769,27 @@
       <c r="N60" s="6"/>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A61" s="15" t="s">
+      <c r="A61" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B61" s="16" t="s">
+      <c r="B61" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="C61" s="16"/>
-      <c r="D61" s="16"/>
-      <c r="E61" s="16"/>
+      <c r="C61" s="11"/>
+      <c r="D61" s="11"/>
+      <c r="E61" s="11"/>
       <c r="F61" s="6"/>
-      <c r="G61" s="16" t="s">
+      <c r="G61" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="H61" s="16"/>
-      <c r="I61" s="16"/>
+      <c r="H61" s="11"/>
+      <c r="I61" s="11"/>
       <c r="J61" s="6"/>
-      <c r="K61" s="16" t="s">
+      <c r="K61" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="L61" s="16"/>
-      <c r="M61" s="16"/>
+      <c r="L61" s="11"/>
+      <c r="M61" s="11"/>
       <c r="N61" s="6"/>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.2">
@@ -3112,11 +3106,11 @@
       <c r="B73" s="5">
         <v>0.15019133000000001</v>
       </c>
-      <c r="C73" s="14">
+      <c r="C73" s="12">
         <v>7.33418E-3</v>
       </c>
-      <c r="D73" s="14"/>
-      <c r="E73" s="14"/>
+      <c r="D73" s="12"/>
+      <c r="E73" s="12"/>
       <c r="F73" s="6"/>
       <c r="G73" s="11">
         <f t="shared" si="11"/>
@@ -3150,27 +3144,27 @@
       <c r="N74" s="6"/>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A75" s="15" t="s">
+      <c r="A75" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B75" s="16" t="s">
+      <c r="B75" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="C75" s="16"/>
-      <c r="D75" s="16"/>
-      <c r="E75" s="16"/>
+      <c r="C75" s="11"/>
+      <c r="D75" s="11"/>
+      <c r="E75" s="11"/>
       <c r="F75" s="6"/>
-      <c r="G75" s="16" t="s">
+      <c r="G75" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="H75" s="16"/>
-      <c r="I75" s="16"/>
+      <c r="H75" s="11"/>
+      <c r="I75" s="11"/>
       <c r="J75" s="6"/>
-      <c r="K75" s="16" t="s">
+      <c r="K75" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="L75" s="16"/>
-      <c r="M75" s="16"/>
+      <c r="L75" s="11"/>
+      <c r="M75" s="11"/>
       <c r="N75" s="6"/>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.2">
@@ -3526,27 +3520,27 @@
       <c r="N88" s="6"/>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A89" s="15" t="s">
+      <c r="A89" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B89" s="16" t="s">
+      <c r="B89" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="C89" s="16"/>
-      <c r="D89" s="16"/>
-      <c r="E89" s="16"/>
+      <c r="C89" s="11"/>
+      <c r="D89" s="11"/>
+      <c r="E89" s="11"/>
       <c r="F89" s="6"/>
-      <c r="G89" s="16" t="s">
+      <c r="G89" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="H89" s="16"/>
-      <c r="I89" s="16"/>
+      <c r="H89" s="11"/>
+      <c r="I89" s="11"/>
       <c r="J89" s="6"/>
-      <c r="K89" s="16" t="s">
+      <c r="K89" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="L89" s="16"/>
-      <c r="M89" s="16"/>
+      <c r="L89" s="11"/>
+      <c r="M89" s="11"/>
       <c r="N89" s="6"/>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.2">
@@ -3863,11 +3857,11 @@
       <c r="B101" s="5">
         <v>0.15019133000000001</v>
       </c>
-      <c r="C101" s="14">
+      <c r="C101" s="12">
         <v>6.1862239999999999E-2</v>
       </c>
-      <c r="D101" s="14"/>
-      <c r="E101" s="14"/>
+      <c r="D101" s="12"/>
+      <c r="E101" s="12"/>
       <c r="F101" s="6"/>
       <c r="G101" s="11">
         <f t="shared" si="15"/>
@@ -3901,27 +3895,27 @@
       <c r="N102" s="6"/>
     </row>
     <row r="103" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A103" s="15" t="s">
+      <c r="A103" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B103" s="16" t="s">
+      <c r="B103" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="C103" s="16"/>
-      <c r="D103" s="16"/>
-      <c r="E103" s="16"/>
+      <c r="C103" s="11"/>
+      <c r="D103" s="11"/>
+      <c r="E103" s="11"/>
       <c r="F103" s="6"/>
-      <c r="G103" s="16" t="s">
+      <c r="G103" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="H103" s="16"/>
-      <c r="I103" s="16"/>
+      <c r="H103" s="11"/>
+      <c r="I103" s="11"/>
       <c r="J103" s="6"/>
-      <c r="K103" s="16" t="s">
+      <c r="K103" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="L103" s="16"/>
-      <c r="M103" s="16"/>
+      <c r="L103" s="11"/>
+      <c r="M103" s="11"/>
       <c r="N103" s="6"/>
     </row>
     <row r="104" spans="1:14" x14ac:dyDescent="0.2">
@@ -4277,27 +4271,27 @@
       <c r="N116" s="6"/>
     </row>
     <row r="117" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A117" s="15" t="s">
+      <c r="A117" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B117" s="16" t="s">
+      <c r="B117" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="C117" s="16"/>
-      <c r="D117" s="16"/>
-      <c r="E117" s="16"/>
+      <c r="C117" s="11"/>
+      <c r="D117" s="11"/>
+      <c r="E117" s="11"/>
       <c r="F117" s="6"/>
-      <c r="G117" s="16" t="s">
+      <c r="G117" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="H117" s="16"/>
-      <c r="I117" s="16"/>
+      <c r="H117" s="11"/>
+      <c r="I117" s="11"/>
       <c r="J117" s="6"/>
-      <c r="K117" s="16" t="s">
+      <c r="K117" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="L117" s="16"/>
-      <c r="M117" s="16"/>
+      <c r="L117" s="11"/>
+      <c r="M117" s="11"/>
       <c r="N117" s="6"/>
     </row>
     <row r="118" spans="1:14" x14ac:dyDescent="0.2">
@@ -4625,7 +4619,7 @@
       <c r="B129" s="5">
         <v>0.15019133000000001</v>
       </c>
-      <c r="C129" s="17">
+      <c r="C129" s="13">
         <f t="shared" si="20"/>
         <v>7.1428570000000011E-2</v>
       </c>
@@ -4664,27 +4658,27 @@
       <c r="N130" s="6"/>
     </row>
     <row r="131" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A131" s="15" t="s">
+      <c r="A131" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B131" s="16" t="s">
+      <c r="B131" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="C131" s="16"/>
-      <c r="D131" s="16"/>
-      <c r="E131" s="16"/>
+      <c r="C131" s="11"/>
+      <c r="D131" s="11"/>
+      <c r="E131" s="11"/>
       <c r="F131" s="6"/>
-      <c r="G131" s="16" t="s">
+      <c r="G131" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="H131" s="16"/>
-      <c r="I131" s="16"/>
+      <c r="H131" s="11"/>
+      <c r="I131" s="11"/>
       <c r="J131" s="6"/>
-      <c r="K131" s="16" t="s">
+      <c r="K131" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="L131" s="16"/>
-      <c r="M131" s="16"/>
+      <c r="L131" s="11"/>
+      <c r="M131" s="11"/>
       <c r="N131" s="6"/>
     </row>
     <row r="132" spans="1:14" x14ac:dyDescent="0.2">
@@ -5013,7 +5007,7 @@
       <c r="B143" s="5">
         <v>1.9451530000000002E-2</v>
       </c>
-      <c r="C143" s="17">
+      <c r="C143" s="13">
         <f t="shared" si="24"/>
         <v>0.66847363999999987</v>
       </c>
@@ -5068,11 +5062,11 @@
       <c r="H145" s="11"/>
       <c r="I145" s="11"/>
       <c r="J145" s="6"/>
-      <c r="K145" s="13">
-        <v>0</v>
-      </c>
-      <c r="L145" s="13"/>
-      <c r="M145" s="13"/>
+      <c r="K145" s="15">
+        <v>0</v>
+      </c>
+      <c r="L145" s="15"/>
+      <c r="M145" s="15"/>
       <c r="N145" s="6"/>
     </row>
     <row r="146" spans="1:14" x14ac:dyDescent="0.2">
@@ -5395,63 +5389,285 @@
     </row>
   </sheetData>
   <mergeCells count="360">
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="G59:I59"/>
-    <mergeCell ref="K59:M59"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="G56:I56"/>
-    <mergeCell ref="K56:M56"/>
-    <mergeCell ref="C57:E57"/>
-    <mergeCell ref="G57:I57"/>
-    <mergeCell ref="K57:M57"/>
-    <mergeCell ref="C58:E58"/>
-    <mergeCell ref="G58:I58"/>
-    <mergeCell ref="K58:M58"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="G53:I53"/>
-    <mergeCell ref="K53:M53"/>
-    <mergeCell ref="C54:E54"/>
-    <mergeCell ref="G54:I54"/>
-    <mergeCell ref="K54:M54"/>
-    <mergeCell ref="C55:E55"/>
-    <mergeCell ref="G55:I55"/>
-    <mergeCell ref="K55:M55"/>
-    <mergeCell ref="C50:E50"/>
-    <mergeCell ref="G50:I50"/>
-    <mergeCell ref="K50:M50"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="G51:I51"/>
-    <mergeCell ref="K51:M51"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="G52:I52"/>
-    <mergeCell ref="K52:M52"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="G47:I47"/>
-    <mergeCell ref="K47:M47"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="G48:I48"/>
-    <mergeCell ref="K48:M48"/>
-    <mergeCell ref="C49:E49"/>
-    <mergeCell ref="G49:I49"/>
-    <mergeCell ref="K49:M49"/>
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="G43:I43"/>
-    <mergeCell ref="K43:M43"/>
-    <mergeCell ref="C44:E44"/>
-    <mergeCell ref="G44:I44"/>
-    <mergeCell ref="K44:M44"/>
-    <mergeCell ref="C45:E45"/>
-    <mergeCell ref="G45:I45"/>
-    <mergeCell ref="K45:M45"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="G40:I40"/>
-    <mergeCell ref="K40:M40"/>
-    <mergeCell ref="C41:E41"/>
-    <mergeCell ref="G41:I41"/>
-    <mergeCell ref="K41:M41"/>
-    <mergeCell ref="C42:E42"/>
-    <mergeCell ref="G42:I42"/>
-    <mergeCell ref="K42:M42"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="G153:H153"/>
+    <mergeCell ref="G155:H155"/>
+    <mergeCell ref="G151:H151"/>
+    <mergeCell ref="K151:L151"/>
+    <mergeCell ref="K153:L153"/>
+    <mergeCell ref="K155:L155"/>
+    <mergeCell ref="K146:M146"/>
+    <mergeCell ref="K152:M152"/>
+    <mergeCell ref="K150:M150"/>
+    <mergeCell ref="K149:M149"/>
+    <mergeCell ref="K148:M148"/>
+    <mergeCell ref="K147:M147"/>
+    <mergeCell ref="K134:M134"/>
+    <mergeCell ref="K140:M140"/>
+    <mergeCell ref="K141:M141"/>
+    <mergeCell ref="K142:M142"/>
+    <mergeCell ref="K118:M118"/>
+    <mergeCell ref="K119:M119"/>
+    <mergeCell ref="K120:M120"/>
+    <mergeCell ref="K121:M121"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="B153:D153"/>
+    <mergeCell ref="B155:D155"/>
+    <mergeCell ref="B151:D151"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="G127:I127"/>
+    <mergeCell ref="G128:I128"/>
+    <mergeCell ref="B152:E152"/>
+    <mergeCell ref="G145:I145"/>
+    <mergeCell ref="G146:I146"/>
+    <mergeCell ref="G147:I147"/>
+    <mergeCell ref="G148:I148"/>
+    <mergeCell ref="G149:I149"/>
+    <mergeCell ref="G150:I150"/>
+    <mergeCell ref="G152:I152"/>
+    <mergeCell ref="B146:E146"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="B145:E145"/>
+    <mergeCell ref="G118:I118"/>
+    <mergeCell ref="G119:I119"/>
+    <mergeCell ref="G120:I120"/>
+    <mergeCell ref="G121:I121"/>
+    <mergeCell ref="G122:I122"/>
+    <mergeCell ref="G123:I123"/>
+    <mergeCell ref="G124:I124"/>
+    <mergeCell ref="G125:I125"/>
+    <mergeCell ref="G126:I126"/>
+    <mergeCell ref="K145:M145"/>
+    <mergeCell ref="C118:E118"/>
+    <mergeCell ref="C119:E119"/>
+    <mergeCell ref="C120:E120"/>
+    <mergeCell ref="C121:E121"/>
+    <mergeCell ref="C122:E122"/>
+    <mergeCell ref="C123:E123"/>
+    <mergeCell ref="C124:E124"/>
+    <mergeCell ref="C125:E125"/>
+    <mergeCell ref="C126:E126"/>
+    <mergeCell ref="B147:E147"/>
+    <mergeCell ref="B148:E148"/>
+    <mergeCell ref="B149:E149"/>
+    <mergeCell ref="B150:E150"/>
+    <mergeCell ref="C138:E138"/>
+    <mergeCell ref="C139:E139"/>
+    <mergeCell ref="C140:E140"/>
+    <mergeCell ref="G129:I129"/>
+    <mergeCell ref="C132:E132"/>
+    <mergeCell ref="C133:E133"/>
+    <mergeCell ref="C134:E134"/>
+    <mergeCell ref="C135:E135"/>
+    <mergeCell ref="C128:E128"/>
+    <mergeCell ref="C129:E129"/>
+    <mergeCell ref="C137:E137"/>
+    <mergeCell ref="C141:E141"/>
+    <mergeCell ref="C142:E142"/>
+    <mergeCell ref="C143:E143"/>
+    <mergeCell ref="G132:I132"/>
+    <mergeCell ref="G133:I133"/>
+    <mergeCell ref="G134:I134"/>
+    <mergeCell ref="G135:I135"/>
+    <mergeCell ref="G136:I136"/>
+    <mergeCell ref="G137:I137"/>
+    <mergeCell ref="G138:I138"/>
+    <mergeCell ref="G139:I139"/>
+    <mergeCell ref="G140:I140"/>
+    <mergeCell ref="G141:I141"/>
+    <mergeCell ref="G142:I142"/>
+    <mergeCell ref="G143:I143"/>
+    <mergeCell ref="C136:E136"/>
+    <mergeCell ref="K133:M133"/>
+    <mergeCell ref="K143:M143"/>
+    <mergeCell ref="K135:M135"/>
+    <mergeCell ref="K136:M136"/>
+    <mergeCell ref="K137:M137"/>
+    <mergeCell ref="K138:M138"/>
+    <mergeCell ref="K139:M139"/>
+    <mergeCell ref="K117:M117"/>
+    <mergeCell ref="G117:I117"/>
+    <mergeCell ref="K122:M122"/>
+    <mergeCell ref="K123:M123"/>
+    <mergeCell ref="K124:M124"/>
+    <mergeCell ref="K125:M125"/>
+    <mergeCell ref="K126:M126"/>
+    <mergeCell ref="K127:M127"/>
+    <mergeCell ref="K128:M128"/>
+    <mergeCell ref="K129:M129"/>
+    <mergeCell ref="K132:M132"/>
+    <mergeCell ref="B117:E117"/>
+    <mergeCell ref="B131:E131"/>
+    <mergeCell ref="G131:I131"/>
+    <mergeCell ref="K131:M131"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="G89:I89"/>
+    <mergeCell ref="K89:M89"/>
+    <mergeCell ref="C90:E90"/>
+    <mergeCell ref="G90:I90"/>
+    <mergeCell ref="K90:M90"/>
+    <mergeCell ref="C91:E91"/>
+    <mergeCell ref="G91:I91"/>
+    <mergeCell ref="K91:M91"/>
+    <mergeCell ref="C92:E92"/>
+    <mergeCell ref="G92:I92"/>
+    <mergeCell ref="K92:M92"/>
+    <mergeCell ref="C93:E93"/>
+    <mergeCell ref="G93:I93"/>
+    <mergeCell ref="K93:M93"/>
+    <mergeCell ref="C94:E94"/>
+    <mergeCell ref="G94:I94"/>
+    <mergeCell ref="K94:M94"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="C127:E127"/>
+    <mergeCell ref="G95:I95"/>
+    <mergeCell ref="K95:M95"/>
+    <mergeCell ref="C96:E96"/>
+    <mergeCell ref="G96:I96"/>
+    <mergeCell ref="K96:M96"/>
+    <mergeCell ref="C97:E97"/>
+    <mergeCell ref="G97:I97"/>
+    <mergeCell ref="K97:M97"/>
+    <mergeCell ref="C98:E98"/>
+    <mergeCell ref="G98:I98"/>
+    <mergeCell ref="K98:M98"/>
+    <mergeCell ref="C99:E99"/>
+    <mergeCell ref="G99:I99"/>
+    <mergeCell ref="K99:M99"/>
+    <mergeCell ref="C100:E100"/>
+    <mergeCell ref="G100:I100"/>
+    <mergeCell ref="K100:M100"/>
+    <mergeCell ref="C101:E101"/>
+    <mergeCell ref="G101:I101"/>
+    <mergeCell ref="K101:M101"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="G103:I103"/>
+    <mergeCell ref="K103:M103"/>
+    <mergeCell ref="C104:E104"/>
+    <mergeCell ref="G104:I104"/>
+    <mergeCell ref="K104:M104"/>
+    <mergeCell ref="C105:E105"/>
+    <mergeCell ref="G105:I105"/>
+    <mergeCell ref="K105:M105"/>
+    <mergeCell ref="C106:E106"/>
+    <mergeCell ref="G106:I106"/>
+    <mergeCell ref="K106:M106"/>
+    <mergeCell ref="C107:E107"/>
+    <mergeCell ref="G107:I107"/>
+    <mergeCell ref="K107:M107"/>
+    <mergeCell ref="C108:E108"/>
+    <mergeCell ref="G108:I108"/>
+    <mergeCell ref="K108:M108"/>
+    <mergeCell ref="C109:E109"/>
+    <mergeCell ref="G109:I109"/>
+    <mergeCell ref="K109:M109"/>
+    <mergeCell ref="C110:E110"/>
+    <mergeCell ref="G110:I110"/>
+    <mergeCell ref="K110:M110"/>
+    <mergeCell ref="C111:E111"/>
+    <mergeCell ref="G111:I111"/>
+    <mergeCell ref="K111:M111"/>
+    <mergeCell ref="C112:E112"/>
+    <mergeCell ref="G112:I112"/>
+    <mergeCell ref="K112:M112"/>
+    <mergeCell ref="C113:E113"/>
+    <mergeCell ref="G113:I113"/>
+    <mergeCell ref="K113:M113"/>
+    <mergeCell ref="C114:E114"/>
+    <mergeCell ref="G114:I114"/>
+    <mergeCell ref="K114:M114"/>
+    <mergeCell ref="C115:E115"/>
+    <mergeCell ref="G115:I115"/>
+    <mergeCell ref="K115:M115"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="G61:I61"/>
+    <mergeCell ref="K61:M61"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="G62:I62"/>
+    <mergeCell ref="K62:M62"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="G63:I63"/>
+    <mergeCell ref="K63:M63"/>
+    <mergeCell ref="C64:E64"/>
+    <mergeCell ref="G64:I64"/>
+    <mergeCell ref="K64:M64"/>
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="G65:I65"/>
+    <mergeCell ref="K65:M65"/>
+    <mergeCell ref="C66:E66"/>
+    <mergeCell ref="G66:I66"/>
+    <mergeCell ref="K66:M66"/>
+    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="G67:I67"/>
+    <mergeCell ref="K67:M67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="G68:I68"/>
+    <mergeCell ref="K68:M68"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="G69:I69"/>
+    <mergeCell ref="K69:M69"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="G70:I70"/>
+    <mergeCell ref="K70:M70"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="G71:I71"/>
+    <mergeCell ref="K71:M71"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="G72:I72"/>
+    <mergeCell ref="K72:M72"/>
+    <mergeCell ref="C73:E73"/>
+    <mergeCell ref="G73:I73"/>
+    <mergeCell ref="K73:M73"/>
+    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="G75:I75"/>
+    <mergeCell ref="K75:M75"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="G76:I76"/>
+    <mergeCell ref="K76:M76"/>
+    <mergeCell ref="C77:E77"/>
+    <mergeCell ref="G77:I77"/>
+    <mergeCell ref="K77:M77"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="G78:I78"/>
+    <mergeCell ref="K78:M78"/>
+    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="G79:I79"/>
+    <mergeCell ref="K79:M79"/>
+    <mergeCell ref="C80:E80"/>
+    <mergeCell ref="G80:I80"/>
+    <mergeCell ref="K80:M80"/>
+    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="G81:I81"/>
+    <mergeCell ref="K81:M81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="G82:I82"/>
+    <mergeCell ref="K82:M82"/>
+    <mergeCell ref="C83:E83"/>
+    <mergeCell ref="G83:I83"/>
+    <mergeCell ref="K83:M83"/>
+    <mergeCell ref="C84:E84"/>
+    <mergeCell ref="G84:I84"/>
+    <mergeCell ref="K84:M84"/>
+    <mergeCell ref="C85:E85"/>
+    <mergeCell ref="G85:I85"/>
+    <mergeCell ref="K85:M85"/>
+    <mergeCell ref="C86:E86"/>
+    <mergeCell ref="G86:I86"/>
+    <mergeCell ref="K86:M86"/>
     <mergeCell ref="C87:E87"/>
     <mergeCell ref="G87:I87"/>
     <mergeCell ref="K87:M87"/>
@@ -5476,285 +5692,63 @@
     <mergeCell ref="C39:E39"/>
     <mergeCell ref="G39:I39"/>
     <mergeCell ref="K39:M39"/>
-    <mergeCell ref="C84:E84"/>
-    <mergeCell ref="G84:I84"/>
-    <mergeCell ref="K84:M84"/>
-    <mergeCell ref="C85:E85"/>
-    <mergeCell ref="G85:I85"/>
-    <mergeCell ref="K85:M85"/>
-    <mergeCell ref="C86:E86"/>
-    <mergeCell ref="G86:I86"/>
-    <mergeCell ref="K86:M86"/>
-    <mergeCell ref="C81:E81"/>
-    <mergeCell ref="G81:I81"/>
-    <mergeCell ref="K81:M81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="G82:I82"/>
-    <mergeCell ref="K82:M82"/>
-    <mergeCell ref="C83:E83"/>
-    <mergeCell ref="G83:I83"/>
-    <mergeCell ref="K83:M83"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="G78:I78"/>
-    <mergeCell ref="K78:M78"/>
-    <mergeCell ref="C79:E79"/>
-    <mergeCell ref="G79:I79"/>
-    <mergeCell ref="K79:M79"/>
-    <mergeCell ref="C80:E80"/>
-    <mergeCell ref="G80:I80"/>
-    <mergeCell ref="K80:M80"/>
-    <mergeCell ref="B75:E75"/>
-    <mergeCell ref="G75:I75"/>
-    <mergeCell ref="K75:M75"/>
-    <mergeCell ref="C76:E76"/>
-    <mergeCell ref="G76:I76"/>
-    <mergeCell ref="K76:M76"/>
-    <mergeCell ref="C77:E77"/>
-    <mergeCell ref="G77:I77"/>
-    <mergeCell ref="K77:M77"/>
-    <mergeCell ref="C71:E71"/>
-    <mergeCell ref="G71:I71"/>
-    <mergeCell ref="K71:M71"/>
-    <mergeCell ref="C72:E72"/>
-    <mergeCell ref="G72:I72"/>
-    <mergeCell ref="K72:M72"/>
-    <mergeCell ref="C73:E73"/>
-    <mergeCell ref="G73:I73"/>
-    <mergeCell ref="K73:M73"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="G68:I68"/>
-    <mergeCell ref="K68:M68"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="G69:I69"/>
-    <mergeCell ref="K69:M69"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="G70:I70"/>
-    <mergeCell ref="K70:M70"/>
-    <mergeCell ref="C115:E115"/>
-    <mergeCell ref="G115:I115"/>
-    <mergeCell ref="K115:M115"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="G61:I61"/>
-    <mergeCell ref="K61:M61"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="G62:I62"/>
-    <mergeCell ref="K62:M62"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="G63:I63"/>
-    <mergeCell ref="K63:M63"/>
-    <mergeCell ref="C64:E64"/>
-    <mergeCell ref="G64:I64"/>
-    <mergeCell ref="K64:M64"/>
-    <mergeCell ref="C65:E65"/>
-    <mergeCell ref="G65:I65"/>
-    <mergeCell ref="K65:M65"/>
-    <mergeCell ref="C66:E66"/>
-    <mergeCell ref="G66:I66"/>
-    <mergeCell ref="K66:M66"/>
-    <mergeCell ref="C67:E67"/>
-    <mergeCell ref="G67:I67"/>
-    <mergeCell ref="K67:M67"/>
-    <mergeCell ref="C112:E112"/>
-    <mergeCell ref="G112:I112"/>
-    <mergeCell ref="K112:M112"/>
-    <mergeCell ref="C113:E113"/>
-    <mergeCell ref="G113:I113"/>
-    <mergeCell ref="K113:M113"/>
-    <mergeCell ref="C114:E114"/>
-    <mergeCell ref="G114:I114"/>
-    <mergeCell ref="K114:M114"/>
-    <mergeCell ref="C109:E109"/>
-    <mergeCell ref="G109:I109"/>
-    <mergeCell ref="K109:M109"/>
-    <mergeCell ref="C110:E110"/>
-    <mergeCell ref="G110:I110"/>
-    <mergeCell ref="K110:M110"/>
-    <mergeCell ref="C111:E111"/>
-    <mergeCell ref="G111:I111"/>
-    <mergeCell ref="K111:M111"/>
-    <mergeCell ref="C106:E106"/>
-    <mergeCell ref="G106:I106"/>
-    <mergeCell ref="K106:M106"/>
-    <mergeCell ref="C107:E107"/>
-    <mergeCell ref="G107:I107"/>
-    <mergeCell ref="K107:M107"/>
-    <mergeCell ref="C108:E108"/>
-    <mergeCell ref="G108:I108"/>
-    <mergeCell ref="K108:M108"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="G103:I103"/>
-    <mergeCell ref="K103:M103"/>
-    <mergeCell ref="C104:E104"/>
-    <mergeCell ref="G104:I104"/>
-    <mergeCell ref="K104:M104"/>
-    <mergeCell ref="C105:E105"/>
-    <mergeCell ref="G105:I105"/>
-    <mergeCell ref="K105:M105"/>
-    <mergeCell ref="C99:E99"/>
-    <mergeCell ref="G99:I99"/>
-    <mergeCell ref="K99:M99"/>
-    <mergeCell ref="C100:E100"/>
-    <mergeCell ref="G100:I100"/>
-    <mergeCell ref="K100:M100"/>
-    <mergeCell ref="C101:E101"/>
-    <mergeCell ref="G101:I101"/>
-    <mergeCell ref="K101:M101"/>
-    <mergeCell ref="G95:I95"/>
-    <mergeCell ref="K95:M95"/>
-    <mergeCell ref="C96:E96"/>
-    <mergeCell ref="G96:I96"/>
-    <mergeCell ref="K96:M96"/>
-    <mergeCell ref="C97:E97"/>
-    <mergeCell ref="G97:I97"/>
-    <mergeCell ref="K97:M97"/>
-    <mergeCell ref="C98:E98"/>
-    <mergeCell ref="G98:I98"/>
-    <mergeCell ref="K98:M98"/>
-    <mergeCell ref="B117:E117"/>
-    <mergeCell ref="B131:E131"/>
-    <mergeCell ref="G131:I131"/>
-    <mergeCell ref="K131:M131"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="G89:I89"/>
-    <mergeCell ref="K89:M89"/>
-    <mergeCell ref="C90:E90"/>
-    <mergeCell ref="G90:I90"/>
-    <mergeCell ref="K90:M90"/>
-    <mergeCell ref="C91:E91"/>
-    <mergeCell ref="G91:I91"/>
-    <mergeCell ref="K91:M91"/>
-    <mergeCell ref="C92:E92"/>
-    <mergeCell ref="G92:I92"/>
-    <mergeCell ref="K92:M92"/>
-    <mergeCell ref="C93:E93"/>
-    <mergeCell ref="G93:I93"/>
-    <mergeCell ref="K93:M93"/>
-    <mergeCell ref="C94:E94"/>
-    <mergeCell ref="G94:I94"/>
-    <mergeCell ref="K94:M94"/>
-    <mergeCell ref="C95:E95"/>
-    <mergeCell ref="K133:M133"/>
-    <mergeCell ref="K143:M143"/>
-    <mergeCell ref="K135:M135"/>
-    <mergeCell ref="K136:M136"/>
-    <mergeCell ref="K137:M137"/>
-    <mergeCell ref="K138:M138"/>
-    <mergeCell ref="K139:M139"/>
-    <mergeCell ref="K117:M117"/>
-    <mergeCell ref="G117:I117"/>
-    <mergeCell ref="K122:M122"/>
-    <mergeCell ref="K123:M123"/>
-    <mergeCell ref="K124:M124"/>
-    <mergeCell ref="K125:M125"/>
-    <mergeCell ref="K126:M126"/>
-    <mergeCell ref="K127:M127"/>
-    <mergeCell ref="K128:M128"/>
-    <mergeCell ref="K129:M129"/>
-    <mergeCell ref="K132:M132"/>
-    <mergeCell ref="C127:E127"/>
-    <mergeCell ref="C128:E128"/>
-    <mergeCell ref="C129:E129"/>
-    <mergeCell ref="C137:E137"/>
-    <mergeCell ref="C141:E141"/>
-    <mergeCell ref="C142:E142"/>
-    <mergeCell ref="C143:E143"/>
-    <mergeCell ref="G132:I132"/>
-    <mergeCell ref="G133:I133"/>
-    <mergeCell ref="G134:I134"/>
-    <mergeCell ref="G135:I135"/>
-    <mergeCell ref="G136:I136"/>
-    <mergeCell ref="G137:I137"/>
-    <mergeCell ref="G138:I138"/>
-    <mergeCell ref="G139:I139"/>
-    <mergeCell ref="G140:I140"/>
-    <mergeCell ref="G141:I141"/>
-    <mergeCell ref="G142:I142"/>
-    <mergeCell ref="G143:I143"/>
-    <mergeCell ref="C136:E136"/>
-    <mergeCell ref="B147:E147"/>
-    <mergeCell ref="B148:E148"/>
-    <mergeCell ref="B149:E149"/>
-    <mergeCell ref="B150:E150"/>
-    <mergeCell ref="C138:E138"/>
-    <mergeCell ref="C139:E139"/>
-    <mergeCell ref="C140:E140"/>
-    <mergeCell ref="G129:I129"/>
-    <mergeCell ref="C132:E132"/>
-    <mergeCell ref="C133:E133"/>
-    <mergeCell ref="C134:E134"/>
-    <mergeCell ref="C135:E135"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="B145:E145"/>
-    <mergeCell ref="G118:I118"/>
-    <mergeCell ref="G119:I119"/>
-    <mergeCell ref="G120:I120"/>
-    <mergeCell ref="G121:I121"/>
-    <mergeCell ref="G122:I122"/>
-    <mergeCell ref="G123:I123"/>
-    <mergeCell ref="G124:I124"/>
-    <mergeCell ref="G125:I125"/>
-    <mergeCell ref="G126:I126"/>
-    <mergeCell ref="K145:M145"/>
-    <mergeCell ref="C118:E118"/>
-    <mergeCell ref="C119:E119"/>
-    <mergeCell ref="C120:E120"/>
-    <mergeCell ref="C121:E121"/>
-    <mergeCell ref="C122:E122"/>
-    <mergeCell ref="C123:E123"/>
-    <mergeCell ref="C124:E124"/>
-    <mergeCell ref="C125:E125"/>
-    <mergeCell ref="C126:E126"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="B153:D153"/>
-    <mergeCell ref="B155:D155"/>
-    <mergeCell ref="B151:D151"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="G127:I127"/>
-    <mergeCell ref="G128:I128"/>
-    <mergeCell ref="B152:E152"/>
-    <mergeCell ref="G145:I145"/>
-    <mergeCell ref="G146:I146"/>
-    <mergeCell ref="G147:I147"/>
-    <mergeCell ref="G148:I148"/>
-    <mergeCell ref="G149:I149"/>
-    <mergeCell ref="G150:I150"/>
-    <mergeCell ref="G152:I152"/>
-    <mergeCell ref="B146:E146"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="G153:H153"/>
-    <mergeCell ref="G155:H155"/>
-    <mergeCell ref="G151:H151"/>
-    <mergeCell ref="K151:L151"/>
-    <mergeCell ref="K153:L153"/>
-    <mergeCell ref="K155:L155"/>
-    <mergeCell ref="K146:M146"/>
-    <mergeCell ref="K152:M152"/>
-    <mergeCell ref="K150:M150"/>
-    <mergeCell ref="K149:M149"/>
-    <mergeCell ref="K148:M148"/>
-    <mergeCell ref="K147:M147"/>
-    <mergeCell ref="K134:M134"/>
-    <mergeCell ref="K140:M140"/>
-    <mergeCell ref="K141:M141"/>
-    <mergeCell ref="K142:M142"/>
-    <mergeCell ref="K118:M118"/>
-    <mergeCell ref="K119:M119"/>
-    <mergeCell ref="K120:M120"/>
-    <mergeCell ref="K121:M121"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="G40:I40"/>
+    <mergeCell ref="K40:M40"/>
+    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="G41:I41"/>
+    <mergeCell ref="K41:M41"/>
+    <mergeCell ref="C42:E42"/>
+    <mergeCell ref="G42:I42"/>
+    <mergeCell ref="K42:M42"/>
+    <mergeCell ref="C43:E43"/>
+    <mergeCell ref="G43:I43"/>
+    <mergeCell ref="K43:M43"/>
+    <mergeCell ref="C44:E44"/>
+    <mergeCell ref="G44:I44"/>
+    <mergeCell ref="K44:M44"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="G45:I45"/>
+    <mergeCell ref="K45:M45"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="G47:I47"/>
+    <mergeCell ref="K47:M47"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="G48:I48"/>
+    <mergeCell ref="K48:M48"/>
+    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="G49:I49"/>
+    <mergeCell ref="K49:M49"/>
+    <mergeCell ref="C50:E50"/>
+    <mergeCell ref="G50:I50"/>
+    <mergeCell ref="K50:M50"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="G51:I51"/>
+    <mergeCell ref="K51:M51"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="G52:I52"/>
+    <mergeCell ref="K52:M52"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="G53:I53"/>
+    <mergeCell ref="K53:M53"/>
+    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="G54:I54"/>
+    <mergeCell ref="K54:M54"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="G55:I55"/>
+    <mergeCell ref="K55:M55"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="G59:I59"/>
+    <mergeCell ref="K59:M59"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="G56:I56"/>
+    <mergeCell ref="K56:M56"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="G57:I57"/>
+    <mergeCell ref="K57:M57"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="G58:I58"/>
+    <mergeCell ref="K58:M58"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
DONE: Finalised excel files.
TODO: Compare FPGA values to truth disparity.
</commit_message>
<xml_diff>
--- a/FPGA_Performance_Comparison_RGB.xlsx
+++ b/FPGA_Performance_Comparison_RGB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/DanielBiswas/Desktop/Documents/University/Year 5/Semester 1/AMME4112/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA795196-7082-C141-AFB9-906B9776AE42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B736910-53A8-2840-8C5D-D3FB1DFCD8F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="24100" windowHeight="17760" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="18060" windowHeight="17760" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2797,7 +2797,7 @@
         <v>32</v>
       </c>
       <c r="B62" s="1">
-        <v>36.935268000000001</v>
+        <v>128.02455399999999</v>
       </c>
       <c r="C62" s="11">
         <v>124.003508</v>
@@ -2807,14 +2807,14 @@
       <c r="F62" s="6"/>
       <c r="G62" s="11">
         <f t="shared" ref="G62:G73" si="11">C62-B62</f>
-        <v>87.068240000000003</v>
+        <v>-4.0210459999999983</v>
       </c>
       <c r="H62" s="11"/>
       <c r="I62" s="11"/>
       <c r="J62" s="6"/>
       <c r="K62" s="10">
         <f>G62/B62</f>
-        <v>2.3573198385889604</v>
+        <v>-3.140839686112086E-2</v>
       </c>
       <c r="L62" s="10"/>
       <c r="M62" s="10"/>
@@ -2825,7 +2825,7 @@
         <v>33</v>
       </c>
       <c r="B63" s="1">
-        <v>4.1183040000000002</v>
+        <v>9.3899869999999996</v>
       </c>
       <c r="C63" s="11">
         <v>9.2522319999999993</v>
@@ -2835,14 +2835,14 @@
       <c r="F63" s="6"/>
       <c r="G63" s="11">
         <f t="shared" si="11"/>
-        <v>5.1339279999999992</v>
+        <v>-0.13775500000000029</v>
       </c>
       <c r="H63" s="11"/>
       <c r="I63" s="11"/>
       <c r="J63" s="6"/>
       <c r="K63" s="10">
         <f>G63/B63</f>
-        <v>1.2466121976425244</v>
+        <v>-1.4670414346686561E-2</v>
       </c>
       <c r="L63" s="10"/>
       <c r="M63" s="10"/>
@@ -2853,7 +2853,7 @@
         <v>34</v>
       </c>
       <c r="B64" s="1">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C64" s="11">
         <v>8</v>
@@ -2863,14 +2863,14 @@
       <c r="F64" s="6"/>
       <c r="G64" s="11">
         <f t="shared" si="11"/>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H64" s="11"/>
       <c r="I64" s="11"/>
       <c r="J64" s="6"/>
       <c r="K64" s="10">
         <f>G64/B64</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L64" s="10"/>
       <c r="M64" s="10"/>
@@ -2881,7 +2881,7 @@
         <v>35</v>
       </c>
       <c r="B65" s="1">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C65" s="11">
         <v>8</v>
@@ -2891,14 +2891,14 @@
       <c r="F65" s="6"/>
       <c r="G65" s="11">
         <f t="shared" si="11"/>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H65" s="11"/>
       <c r="I65" s="11"/>
       <c r="J65" s="6"/>
       <c r="K65" s="10">
         <f>G65/B65</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L65" s="10"/>
       <c r="M65" s="10"/>
@@ -2936,7 +2936,7 @@
         <v>37</v>
       </c>
       <c r="B67" s="1">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="C67" s="11">
         <v>39</v>
@@ -2946,14 +2946,14 @@
       <c r="F67" s="6"/>
       <c r="G67" s="11">
         <f t="shared" si="11"/>
-        <v>16</v>
+        <v>-1</v>
       </c>
       <c r="H67" s="11"/>
       <c r="I67" s="11"/>
       <c r="J67" s="6"/>
       <c r="K67" s="10">
         <f t="shared" ref="K67:K73" si="12">G67/B67</f>
-        <v>0.69565217391304346</v>
+        <v>-2.5000000000000001E-2</v>
       </c>
       <c r="L67" s="10"/>
       <c r="M67" s="10"/>
@@ -2964,7 +2964,7 @@
         <v>38</v>
       </c>
       <c r="B68" s="1">
-        <v>6.6195789999999999</v>
+        <v>5.8580990000000002</v>
       </c>
       <c r="C68" s="11">
         <v>5.8427930000000003</v>
@@ -2974,14 +2974,14 @@
       <c r="F68" s="6"/>
       <c r="G68" s="11">
         <f t="shared" si="11"/>
-        <v>-0.77678599999999953</v>
+        <v>-1.530599999999982E-2</v>
       </c>
       <c r="H68" s="11"/>
       <c r="I68" s="11"/>
       <c r="J68" s="6"/>
       <c r="K68" s="10">
         <f t="shared" si="12"/>
-        <v>-0.11734673760974823</v>
+        <v>-2.6127929896711919E-3</v>
       </c>
       <c r="L68" s="10"/>
       <c r="M68" s="10"/>
@@ -2992,7 +2992,7 @@
         <v>39</v>
       </c>
       <c r="B69" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C69" s="11">
         <v>6</v>
@@ -3002,14 +3002,14 @@
       <c r="F69" s="6"/>
       <c r="G69" s="11">
         <f t="shared" si="11"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="H69" s="11"/>
       <c r="I69" s="11"/>
       <c r="J69" s="6"/>
       <c r="K69" s="10">
         <f t="shared" si="12"/>
-        <v>-0.14285714285714285</v>
+        <v>0</v>
       </c>
       <c r="L69" s="10"/>
       <c r="M69" s="10"/>
@@ -3076,7 +3076,7 @@
         <v>76</v>
       </c>
       <c r="B72" s="1">
-        <v>471</v>
+        <v>23</v>
       </c>
       <c r="C72" s="11">
         <v>23</v>
@@ -3086,14 +3086,14 @@
       <c r="F72" s="6"/>
       <c r="G72" s="11">
         <f t="shared" si="11"/>
-        <v>-448</v>
+        <v>0</v>
       </c>
       <c r="H72" s="11"/>
       <c r="I72" s="11"/>
       <c r="J72" s="6"/>
       <c r="K72" s="10">
         <f t="shared" si="12"/>
-        <v>-0.95116772823779194</v>
+        <v>0</v>
       </c>
       <c r="L72" s="10"/>
       <c r="M72" s="10"/>
@@ -3104,7 +3104,7 @@
         <v>42</v>
       </c>
       <c r="B73" s="5">
-        <v>0.15019133000000001</v>
+        <v>7.33418E-3</v>
       </c>
       <c r="C73" s="12">
         <v>7.33418E-3</v>
@@ -3114,14 +3114,14 @@
       <c r="F73" s="6"/>
       <c r="G73" s="11">
         <f t="shared" si="11"/>
-        <v>-0.14285715000000002</v>
+        <v>0</v>
       </c>
       <c r="H73" s="11"/>
       <c r="I73" s="11"/>
       <c r="J73" s="6"/>
       <c r="K73" s="10">
         <f t="shared" si="12"/>
-        <v>-0.95116775382440522</v>
+        <v>0</v>
       </c>
       <c r="L73" s="10"/>
       <c r="M73" s="10"/>
@@ -3172,7 +3172,7 @@
         <v>43</v>
       </c>
       <c r="B76" s="1">
-        <v>3.401786</v>
+        <v>0</v>
       </c>
       <c r="C76" s="11">
         <v>0</v>
@@ -3182,14 +3182,14 @@
       <c r="F76" s="6"/>
       <c r="G76" s="11">
         <f t="shared" ref="G76:G87" si="13">C76-B76</f>
-        <v>-3.401786</v>
+        <v>0</v>
       </c>
       <c r="H76" s="11"/>
       <c r="I76" s="11"/>
       <c r="J76" s="6"/>
-      <c r="K76" s="10">
+      <c r="K76" s="10" t="e">
         <f t="shared" ref="K76:K87" si="14">G76/B76</f>
-        <v>-1</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L76" s="10"/>
       <c r="M76" s="10"/>
@@ -3200,7 +3200,7 @@
         <v>44</v>
       </c>
       <c r="B77" s="1">
-        <v>1.770408</v>
+        <v>0</v>
       </c>
       <c r="C77" s="11">
         <v>0</v>
@@ -3210,14 +3210,14 @@
       <c r="F77" s="6"/>
       <c r="G77" s="11">
         <f t="shared" si="13"/>
-        <v>-1.770408</v>
+        <v>0</v>
       </c>
       <c r="H77" s="11"/>
       <c r="I77" s="11"/>
       <c r="J77" s="6"/>
-      <c r="K77" s="10">
+      <c r="K77" s="10" t="e">
         <f t="shared" si="14"/>
-        <v>-1</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L77" s="10"/>
       <c r="M77" s="10"/>
@@ -3228,7 +3228,7 @@
         <v>45</v>
       </c>
       <c r="B78" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C78" s="11">
         <v>0</v>
@@ -3238,14 +3238,14 @@
       <c r="F78" s="6"/>
       <c r="G78" s="11">
         <f t="shared" si="13"/>
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="H78" s="11"/>
       <c r="I78" s="11"/>
       <c r="J78" s="6"/>
-      <c r="K78" s="10">
+      <c r="K78" s="10" t="e">
         <f t="shared" si="14"/>
-        <v>-1</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L78" s="10"/>
       <c r="M78" s="10"/>
@@ -3256,7 +3256,7 @@
         <v>46</v>
       </c>
       <c r="B79" s="1">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="C79" s="11">
         <v>0</v>
@@ -3266,14 +3266,14 @@
       <c r="F79" s="6"/>
       <c r="G79" s="11">
         <f t="shared" si="13"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H79" s="11"/>
       <c r="I79" s="11"/>
       <c r="J79" s="6"/>
-      <c r="K79" s="10">
+      <c r="K79" s="10" t="e">
         <f t="shared" si="14"/>
-        <v>-1</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L79" s="10"/>
       <c r="M79" s="10"/>
@@ -3284,7 +3284,7 @@
         <v>47</v>
       </c>
       <c r="B80" s="1">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="C80" s="11">
         <v>0</v>
@@ -3294,14 +3294,14 @@
       <c r="F80" s="6"/>
       <c r="G80" s="11">
         <f t="shared" si="13"/>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H80" s="11"/>
       <c r="I80" s="11"/>
       <c r="J80" s="6"/>
-      <c r="K80" s="10">
+      <c r="K80" s="10" t="e">
         <f t="shared" si="14"/>
-        <v>-1</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L80" s="10"/>
       <c r="M80" s="10"/>
@@ -3312,7 +3312,7 @@
         <v>48</v>
       </c>
       <c r="B81" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C81" s="11">
         <v>0</v>
@@ -3322,14 +3322,14 @@
       <c r="F81" s="6"/>
       <c r="G81" s="11">
         <f t="shared" si="13"/>
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="H81" s="11"/>
       <c r="I81" s="11"/>
       <c r="J81" s="6"/>
-      <c r="K81" s="10">
+      <c r="K81" s="10" t="e">
         <f t="shared" si="14"/>
-        <v>-1</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L81" s="10"/>
       <c r="M81" s="10"/>
@@ -3340,7 +3340,7 @@
         <v>49</v>
       </c>
       <c r="B82" s="1">
-        <v>6.7904970000000002</v>
+        <v>8</v>
       </c>
       <c r="C82" s="11">
         <v>8</v>
@@ -3350,14 +3350,14 @@
       <c r="F82" s="6"/>
       <c r="G82" s="11">
         <f t="shared" si="13"/>
-        <v>1.2095029999999998</v>
+        <v>0</v>
       </c>
       <c r="H82" s="11"/>
       <c r="I82" s="11"/>
       <c r="J82" s="6"/>
       <c r="K82" s="10">
         <f t="shared" si="14"/>
-        <v>0.17811700675223033</v>
+        <v>0</v>
       </c>
       <c r="L82" s="10"/>
       <c r="M82" s="10"/>
@@ -3368,7 +3368,7 @@
         <v>50</v>
       </c>
       <c r="B83" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C83" s="11">
         <v>8</v>
@@ -3378,14 +3378,14 @@
       <c r="F83" s="6"/>
       <c r="G83" s="11">
         <f t="shared" si="13"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H83" s="11"/>
       <c r="I83" s="11"/>
       <c r="J83" s="6"/>
       <c r="K83" s="10">
         <f t="shared" si="14"/>
-        <v>0.14285714285714285</v>
+        <v>0</v>
       </c>
       <c r="L83" s="10"/>
       <c r="M83" s="10"/>
@@ -3424,7 +3424,7 @@
         <v>52</v>
       </c>
       <c r="B85" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C85" s="11">
         <v>8</v>
@@ -3434,14 +3434,14 @@
       <c r="F85" s="6"/>
       <c r="G85" s="11">
         <f t="shared" si="13"/>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H85" s="11"/>
       <c r="I85" s="11"/>
       <c r="J85" s="6"/>
       <c r="K85" s="10">
         <f t="shared" si="14"/>
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="L85" s="10"/>
       <c r="M85" s="10"/>
@@ -3452,7 +3452,7 @@
         <v>77</v>
       </c>
       <c r="B86" s="1">
-        <v>61</v>
+        <v>3136</v>
       </c>
       <c r="C86" s="11">
         <v>3136</v>
@@ -3462,14 +3462,14 @@
       <c r="F86" s="6"/>
       <c r="G86" s="11">
         <f t="shared" si="13"/>
-        <v>3075</v>
+        <v>0</v>
       </c>
       <c r="H86" s="11"/>
       <c r="I86" s="11"/>
       <c r="J86" s="6"/>
       <c r="K86" s="10">
         <f t="shared" si="14"/>
-        <v>50.409836065573771</v>
+        <v>0</v>
       </c>
       <c r="L86" s="10"/>
       <c r="M86" s="10"/>
@@ -3480,7 +3480,7 @@
         <v>53</v>
       </c>
       <c r="B87" s="5">
-        <v>1.9451530000000002E-2</v>
+        <v>1</v>
       </c>
       <c r="C87" s="10">
         <v>1</v>
@@ -3490,14 +3490,14 @@
       <c r="F87" s="6"/>
       <c r="G87" s="11">
         <f t="shared" si="13"/>
-        <v>0.98054847000000001</v>
+        <v>0</v>
       </c>
       <c r="H87" s="11"/>
       <c r="I87" s="11"/>
       <c r="J87" s="6"/>
       <c r="K87" s="10">
         <f t="shared" si="14"/>
-        <v>50.409837683719481</v>
+        <v>0</v>
       </c>
       <c r="L87" s="10"/>
       <c r="M87" s="10"/>
@@ -3548,7 +3548,7 @@
         <v>32</v>
       </c>
       <c r="B90" s="1">
-        <v>36.935268000000001</v>
+        <v>8.9113520000000008</v>
       </c>
       <c r="C90" s="11">
         <v>8.6871810000000007</v>
@@ -3558,14 +3558,14 @@
       <c r="F90" s="6"/>
       <c r="G90" s="11">
         <f t="shared" ref="G90:G101" si="15">C90-B90</f>
-        <v>-28.248086999999998</v>
+        <v>-0.22417100000000012</v>
       </c>
       <c r="H90" s="11"/>
       <c r="I90" s="11"/>
       <c r="J90" s="6"/>
       <c r="K90" s="10">
         <f>G90/B90</f>
-        <v>-0.76479983846333532</v>
+        <v>-2.5155666614897505E-2</v>
       </c>
       <c r="L90" s="10"/>
       <c r="M90" s="10"/>
@@ -3576,7 +3576,7 @@
         <v>33</v>
       </c>
       <c r="B91" s="1">
-        <v>4.1183040000000002</v>
+        <v>2.2079080000000002</v>
       </c>
       <c r="C91" s="11">
         <v>2.1980230000000001</v>
@@ -3586,14 +3586,14 @@
       <c r="F91" s="6"/>
       <c r="G91" s="11">
         <f t="shared" si="15"/>
-        <v>-1.9202810000000001</v>
+        <v>-9.8850000000001437E-3</v>
       </c>
       <c r="H91" s="11"/>
       <c r="I91" s="11"/>
       <c r="J91" s="6"/>
       <c r="K91" s="10">
         <f>G91/B91</f>
-        <v>-0.46627956556873901</v>
+        <v>-4.4770887192764116E-3</v>
       </c>
       <c r="L91" s="10"/>
       <c r="M91" s="10"/>
@@ -3687,7 +3687,7 @@
         <v>37</v>
       </c>
       <c r="B95" s="1">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C95" s="11">
         <v>12</v>
@@ -3697,14 +3697,14 @@
       <c r="F95" s="6"/>
       <c r="G95" s="11">
         <f t="shared" si="15"/>
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="H95" s="11"/>
       <c r="I95" s="11"/>
       <c r="J95" s="6"/>
       <c r="K95" s="10">
         <f t="shared" ref="K95:K101" si="16">G95/B95</f>
-        <v>-0.47826086956521741</v>
+        <v>0</v>
       </c>
       <c r="L95" s="10"/>
       <c r="M95" s="10"/>
@@ -3715,7 +3715,7 @@
         <v>38</v>
       </c>
       <c r="B96" s="1">
-        <v>6.6195789999999999</v>
+        <v>6.8000639999999999</v>
       </c>
       <c r="C96" s="11">
         <v>6.7997449999999997</v>
@@ -3725,14 +3725,14 @@
       <c r="F96" s="6"/>
       <c r="G96" s="11">
         <f t="shared" si="15"/>
-        <v>0.18016599999999983</v>
+        <v>-3.1900000000018025E-4</v>
       </c>
       <c r="H96" s="11"/>
       <c r="I96" s="11"/>
       <c r="J96" s="6"/>
       <c r="K96" s="10">
         <f t="shared" si="16"/>
-        <v>2.7217138733445109E-2</v>
+        <v>-4.6911323187572975E-5</v>
       </c>
       <c r="L96" s="10"/>
       <c r="M96" s="10"/>
@@ -3799,7 +3799,7 @@
         <v>41</v>
       </c>
       <c r="B99" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C99" s="11">
         <v>4</v>
@@ -3809,14 +3809,14 @@
       <c r="F99" s="6"/>
       <c r="G99" s="11">
         <f t="shared" si="15"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H99" s="11"/>
       <c r="I99" s="11"/>
       <c r="J99" s="6"/>
       <c r="K99" s="10">
         <f t="shared" si="16"/>
-        <v>0.33333333333333331</v>
+        <v>0</v>
       </c>
       <c r="L99" s="10"/>
       <c r="M99" s="10"/>
@@ -3827,7 +3827,7 @@
         <v>76</v>
       </c>
       <c r="B100" s="1">
-        <v>471</v>
+        <v>211</v>
       </c>
       <c r="C100" s="11">
         <v>194</v>
@@ -3837,14 +3837,14 @@
       <c r="F100" s="6"/>
       <c r="G100" s="11">
         <f t="shared" si="15"/>
-        <v>-277</v>
+        <v>-17</v>
       </c>
       <c r="H100" s="11"/>
       <c r="I100" s="11"/>
       <c r="J100" s="6"/>
       <c r="K100" s="10">
         <f t="shared" si="16"/>
-        <v>-0.58811040339702758</v>
+        <v>-8.0568720379146919E-2</v>
       </c>
       <c r="L100" s="10"/>
       <c r="M100" s="10"/>
@@ -3855,7 +3855,7 @@
         <v>42</v>
       </c>
       <c r="B101" s="5">
-        <v>0.15019133000000001</v>
+        <v>6.7283159999999995E-2</v>
       </c>
       <c r="C101" s="12">
         <v>6.1862239999999999E-2</v>
@@ -3865,14 +3865,14 @@
       <c r="F101" s="6"/>
       <c r="G101" s="11">
         <f t="shared" si="15"/>
-        <v>-8.8329090000000013E-2</v>
+        <v>-5.4209199999999957E-3</v>
       </c>
       <c r="H101" s="11"/>
       <c r="I101" s="11"/>
       <c r="J101" s="6"/>
       <c r="K101" s="10">
         <f t="shared" si="16"/>
-        <v>-0.58811044552305392</v>
+        <v>-8.0568748554615988E-2</v>
       </c>
       <c r="L101" s="10"/>
       <c r="M101" s="10"/>
@@ -3923,7 +3923,7 @@
         <v>43</v>
       </c>
       <c r="B104" s="1">
-        <v>3.401786</v>
+        <v>9.8849999999999997E-3</v>
       </c>
       <c r="C104" s="11">
         <v>0.11926</v>
@@ -3933,14 +3933,14 @@
       <c r="F104" s="6"/>
       <c r="G104" s="11">
         <f t="shared" ref="G104:G115" si="17">C104-B104</f>
-        <v>-3.2825259999999998</v>
+        <v>0.109375</v>
       </c>
       <c r="H104" s="11"/>
       <c r="I104" s="11"/>
       <c r="J104" s="6"/>
       <c r="K104" s="10">
         <f t="shared" ref="K104:K115" si="18">G104/B104</f>
-        <v>-0.96494194520172638</v>
+        <v>11.064744562468388</v>
       </c>
       <c r="L104" s="10"/>
       <c r="M104" s="10"/>
@@ -3951,7 +3951,7 @@
         <v>44</v>
       </c>
       <c r="B105" s="1">
-        <v>1.770408</v>
+        <v>9.8849999999999997E-3</v>
       </c>
       <c r="C105" s="11">
         <v>2.6148000000000001E-2</v>
@@ -3961,14 +3961,14 @@
       <c r="F105" s="6"/>
       <c r="G105" s="11">
         <f t="shared" si="17"/>
-        <v>-1.7442599999999999</v>
+        <v>1.6263E-2</v>
       </c>
       <c r="H105" s="11"/>
       <c r="I105" s="11"/>
       <c r="J105" s="6"/>
       <c r="K105" s="10">
         <f t="shared" si="18"/>
-        <v>-0.98523052313365056</v>
+        <v>1.6452200303490137</v>
       </c>
       <c r="L105" s="10"/>
       <c r="M105" s="10"/>
@@ -3979,7 +3979,7 @@
         <v>45</v>
       </c>
       <c r="B106" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C106" s="11">
         <v>0</v>
@@ -3989,14 +3989,14 @@
       <c r="F106" s="6"/>
       <c r="G106" s="11">
         <f t="shared" si="17"/>
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="H106" s="11"/>
       <c r="I106" s="11"/>
       <c r="J106" s="6"/>
-      <c r="K106" s="10">
+      <c r="K106" s="10" t="e">
         <f t="shared" si="18"/>
-        <v>-1</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L106" s="10"/>
       <c r="M106" s="10"/>
@@ -4007,7 +4007,7 @@
         <v>46</v>
       </c>
       <c r="B107" s="1">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="C107" s="11">
         <v>0</v>
@@ -4017,14 +4017,14 @@
       <c r="F107" s="6"/>
       <c r="G107" s="11">
         <f t="shared" si="17"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H107" s="11"/>
       <c r="I107" s="11"/>
       <c r="J107" s="6"/>
-      <c r="K107" s="10">
+      <c r="K107" s="10" t="e">
         <f t="shared" si="18"/>
-        <v>-1</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L107" s="10"/>
       <c r="M107" s="10"/>
@@ -4035,7 +4035,7 @@
         <v>47</v>
       </c>
       <c r="B108" s="1">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="C108" s="11">
         <v>-1</v>
@@ -4045,14 +4045,14 @@
       <c r="F108" s="6"/>
       <c r="G108" s="11">
         <f t="shared" si="17"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H108" s="11"/>
       <c r="I108" s="11"/>
       <c r="J108" s="6"/>
       <c r="K108" s="10">
         <f t="shared" si="18"/>
-        <v>-0.66666666666666663</v>
+        <v>0</v>
       </c>
       <c r="L108" s="10"/>
       <c r="M108" s="10"/>
@@ -4063,7 +4063,7 @@
         <v>48</v>
       </c>
       <c r="B109" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C109" s="11">
         <v>11</v>
@@ -4073,14 +4073,14 @@
       <c r="F109" s="6"/>
       <c r="G109" s="11">
         <f t="shared" si="17"/>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H109" s="11"/>
       <c r="I109" s="11"/>
       <c r="J109" s="6"/>
-      <c r="K109" s="10">
+      <c r="K109" s="10" t="e">
         <f t="shared" si="18"/>
-        <v>4.5</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L109" s="10"/>
       <c r="M109" s="10"/>
@@ -4091,7 +4091,7 @@
         <v>49</v>
       </c>
       <c r="B110" s="1">
-        <v>6.7904970000000002</v>
+        <v>7.9901150000000003</v>
       </c>
       <c r="C110" s="11">
         <v>7.9846940000000002</v>
@@ -4101,14 +4101,14 @@
       <c r="F110" s="6"/>
       <c r="G110" s="11">
         <f t="shared" si="17"/>
-        <v>1.194197</v>
+        <v>-5.4210000000001202E-3</v>
       </c>
       <c r="H110" s="11"/>
       <c r="I110" s="11"/>
       <c r="J110" s="6"/>
       <c r="K110" s="10">
         <f t="shared" si="18"/>
-        <v>0.17586297438906165</v>
+        <v>-6.7846332624750961E-4</v>
       </c>
       <c r="L110" s="10"/>
       <c r="M110" s="10"/>
@@ -4119,7 +4119,7 @@
         <v>50</v>
       </c>
       <c r="B111" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C111" s="11">
         <v>8</v>
@@ -4129,14 +4129,14 @@
       <c r="F111" s="6"/>
       <c r="G111" s="11">
         <f t="shared" si="17"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H111" s="11"/>
       <c r="I111" s="11"/>
       <c r="J111" s="6"/>
       <c r="K111" s="10">
         <f t="shared" si="18"/>
-        <v>0.14285714285714285</v>
+        <v>0</v>
       </c>
       <c r="L111" s="10"/>
       <c r="M111" s="10"/>
@@ -4175,7 +4175,7 @@
         <v>52</v>
       </c>
       <c r="B113" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C113" s="11">
         <v>5</v>
@@ -4185,14 +4185,14 @@
       <c r="F113" s="6"/>
       <c r="G113" s="11">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="H113" s="11"/>
       <c r="I113" s="11"/>
       <c r="J113" s="6"/>
       <c r="K113" s="10">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>-0.2857142857142857</v>
       </c>
       <c r="L113" s="10"/>
       <c r="M113" s="10"/>
@@ -4203,7 +4203,7 @@
         <v>77</v>
       </c>
       <c r="B114" s="1">
-        <v>61</v>
+        <v>3105</v>
       </c>
       <c r="C114" s="11">
         <v>3093</v>
@@ -4213,14 +4213,14 @@
       <c r="F114" s="6"/>
       <c r="G114" s="11">
         <f t="shared" si="17"/>
-        <v>3032</v>
+        <v>-12</v>
       </c>
       <c r="H114" s="11"/>
       <c r="I114" s="11"/>
       <c r="J114" s="6"/>
       <c r="K114" s="10">
         <f t="shared" si="18"/>
-        <v>49.704918032786885</v>
+        <v>-3.8647342995169081E-3</v>
       </c>
       <c r="L114" s="10"/>
       <c r="M114" s="10"/>
@@ -4231,7 +4231,7 @@
         <v>53</v>
       </c>
       <c r="B115" s="5">
-        <v>1.9451530000000002E-2</v>
+        <v>0.99011479999999996</v>
       </c>
       <c r="C115" s="10">
         <v>0.98628826999999997</v>
@@ -4241,14 +4241,14 @@
       <c r="F115" s="6"/>
       <c r="G115" s="11">
         <f t="shared" si="17"/>
-        <v>0.96683673999999997</v>
+        <v>-3.8265299999999947E-3</v>
       </c>
       <c r="H115" s="11"/>
       <c r="I115" s="11"/>
       <c r="J115" s="6"/>
       <c r="K115" s="10">
         <f t="shared" si="18"/>
-        <v>49.704919870056486</v>
+        <v>-3.8647336652275015E-3</v>
       </c>
       <c r="L115" s="10"/>
       <c r="M115" s="10"/>

</xml_diff>

<commit_message>
DONE: Comparison of estimation to truth for central images.
TODO: Test different region (bottom left).
</commit_message>
<xml_diff>
--- a/FPGA_Performance_Comparison_RGB.xlsx
+++ b/FPGA_Performance_Comparison_RGB.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/DanielBiswas/Desktop/Documents/University/Year 5/Semester 1/AMME4112/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B736910-53A8-2840-8C5D-D3FB1DFCD8F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C66D13FC-801E-7943-A9A3-DB3D576B41D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="18060" windowHeight="17760" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="24660" windowHeight="26820" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -365,17 +365,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -722,15 +722,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
+      <c r="B1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
       <c r="F1" s="6"/>
       <c r="G1" s="11" t="s">
         <v>55</v>
@@ -746,7 +746,7 @@
       <c r="N1" s="6"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A2" s="14"/>
+      <c r="A2" s="12"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2355,11 +2355,11 @@
       <c r="B45" s="5">
         <v>0.15019133000000001</v>
       </c>
-      <c r="C45" s="12">
+      <c r="C45" s="15">
         <v>0.14508929000000001</v>
       </c>
-      <c r="D45" s="12"/>
-      <c r="E45" s="12"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15"/>
       <c r="F45" s="6"/>
       <c r="G45" s="11">
         <f t="shared" si="7"/>
@@ -2421,24 +2421,24 @@
         <v>43</v>
       </c>
       <c r="B48" s="1">
-        <v>3.401786</v>
+        <v>3.3816959999999998</v>
       </c>
       <c r="C48" s="11">
-        <v>3.4068879999999999</v>
+        <v>3.3852039999999999</v>
       </c>
       <c r="D48" s="11"/>
       <c r="E48" s="11"/>
       <c r="F48" s="6"/>
       <c r="G48" s="11">
         <f t="shared" ref="G48:G59" si="9">C48-B48</f>
-        <v>5.1019999999999399E-3</v>
+        <v>3.5080000000000666E-3</v>
       </c>
       <c r="H48" s="11"/>
       <c r="I48" s="11"/>
       <c r="J48" s="6"/>
       <c r="K48" s="10">
         <f t="shared" ref="K48:K59" si="10">G48/B48</f>
-        <v>1.4998003989668779E-3</v>
+        <v>1.0373493063835623E-3</v>
       </c>
       <c r="L48" s="10"/>
       <c r="M48" s="10"/>
@@ -2449,24 +2449,24 @@
         <v>44</v>
       </c>
       <c r="B49" s="1">
-        <v>1.770408</v>
+        <v>1.7662629999999999</v>
       </c>
       <c r="C49" s="11">
-        <v>1.772321</v>
+        <v>1.767857</v>
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="11"/>
       <c r="F49" s="6"/>
       <c r="G49" s="11">
         <f t="shared" si="9"/>
-        <v>1.9130000000000535E-3</v>
+        <v>1.5940000000000953E-3</v>
       </c>
       <c r="H49" s="11"/>
       <c r="I49" s="11"/>
       <c r="J49" s="6"/>
       <c r="K49" s="10">
         <f t="shared" si="10"/>
-        <v>1.0805418863900601E-3</v>
+        <v>9.0247035690613198E-4</v>
       </c>
       <c r="L49" s="10"/>
       <c r="M49" s="10"/>
@@ -2589,24 +2589,24 @@
         <v>49</v>
       </c>
       <c r="B54" s="1">
-        <v>6.7904970000000002</v>
+        <v>6.7936860000000001</v>
       </c>
       <c r="C54" s="11">
-        <v>6.78986</v>
+        <v>6.7933669999999999</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="11"/>
       <c r="F54" s="6"/>
       <c r="G54" s="11">
         <f t="shared" si="9"/>
-        <v>-6.3700000000022072E-4</v>
+        <v>-3.1900000000018025E-4</v>
       </c>
       <c r="H54" s="11"/>
       <c r="I54" s="11"/>
       <c r="J54" s="6"/>
       <c r="K54" s="10">
         <f t="shared" si="10"/>
-        <v>-9.3807566662678849E-5</v>
+        <v>-4.6955364142555343E-5</v>
       </c>
       <c r="L54" s="10"/>
       <c r="M54" s="10"/>
@@ -3106,11 +3106,11 @@
       <c r="B73" s="5">
         <v>7.33418E-3</v>
       </c>
-      <c r="C73" s="12">
+      <c r="C73" s="15">
         <v>7.33418E-3</v>
       </c>
-      <c r="D73" s="12"/>
-      <c r="E73" s="12"/>
+      <c r="D73" s="15"/>
+      <c r="E73" s="15"/>
       <c r="F73" s="6"/>
       <c r="G73" s="11">
         <f t="shared" si="11"/>
@@ -3187,9 +3187,8 @@
       <c r="H76" s="11"/>
       <c r="I76" s="11"/>
       <c r="J76" s="6"/>
-      <c r="K76" s="10" t="e">
-        <f t="shared" ref="K76:K87" si="14">G76/B76</f>
-        <v>#DIV/0!</v>
+      <c r="K76" s="10">
+        <v>0</v>
       </c>
       <c r="L76" s="10"/>
       <c r="M76" s="10"/>
@@ -3215,9 +3214,8 @@
       <c r="H77" s="11"/>
       <c r="I77" s="11"/>
       <c r="J77" s="6"/>
-      <c r="K77" s="10" t="e">
-        <f t="shared" si="14"/>
-        <v>#DIV/0!</v>
+      <c r="K77" s="10">
+        <v>0</v>
       </c>
       <c r="L77" s="10"/>
       <c r="M77" s="10"/>
@@ -3243,9 +3241,8 @@
       <c r="H78" s="11"/>
       <c r="I78" s="11"/>
       <c r="J78" s="6"/>
-      <c r="K78" s="10" t="e">
-        <f t="shared" si="14"/>
-        <v>#DIV/0!</v>
+      <c r="K78" s="10">
+        <v>0</v>
       </c>
       <c r="L78" s="10"/>
       <c r="M78" s="10"/>
@@ -3271,9 +3268,8 @@
       <c r="H79" s="11"/>
       <c r="I79" s="11"/>
       <c r="J79" s="6"/>
-      <c r="K79" s="10" t="e">
-        <f t="shared" si="14"/>
-        <v>#DIV/0!</v>
+      <c r="K79" s="10">
+        <v>0</v>
       </c>
       <c r="L79" s="10"/>
       <c r="M79" s="10"/>
@@ -3299,9 +3295,8 @@
       <c r="H80" s="11"/>
       <c r="I80" s="11"/>
       <c r="J80" s="6"/>
-      <c r="K80" s="10" t="e">
-        <f t="shared" si="14"/>
-        <v>#DIV/0!</v>
+      <c r="K80" s="10">
+        <v>0</v>
       </c>
       <c r="L80" s="10"/>
       <c r="M80" s="10"/>
@@ -3327,9 +3322,8 @@
       <c r="H81" s="11"/>
       <c r="I81" s="11"/>
       <c r="J81" s="6"/>
-      <c r="K81" s="10" t="e">
-        <f t="shared" si="14"/>
-        <v>#DIV/0!</v>
+      <c r="K81" s="10">
+        <v>0</v>
       </c>
       <c r="L81" s="10"/>
       <c r="M81" s="10"/>
@@ -3356,7 +3350,7 @@
       <c r="I82" s="11"/>
       <c r="J82" s="6"/>
       <c r="K82" s="10">
-        <f t="shared" si="14"/>
+        <f t="shared" ref="K76:K87" si="14">G82/B82</f>
         <v>0</v>
       </c>
       <c r="L82" s="10"/>
@@ -3857,11 +3851,11 @@
       <c r="B101" s="5">
         <v>6.7283159999999995E-2</v>
       </c>
-      <c r="C101" s="12">
+      <c r="C101" s="15">
         <v>6.1862239999999999E-2</v>
       </c>
-      <c r="D101" s="12"/>
-      <c r="E101" s="12"/>
+      <c r="D101" s="15"/>
+      <c r="E101" s="15"/>
       <c r="F101" s="6"/>
       <c r="G101" s="11">
         <f t="shared" si="15"/>
@@ -3926,21 +3920,21 @@
         <v>9.8849999999999997E-3</v>
       </c>
       <c r="C104" s="11">
-        <v>0.11926</v>
+        <v>9.8849999999999997E-3</v>
       </c>
       <c r="D104" s="11"/>
       <c r="E104" s="11"/>
       <c r="F104" s="6"/>
       <c r="G104" s="11">
         <f t="shared" ref="G104:G115" si="17">C104-B104</f>
-        <v>0.109375</v>
+        <v>0</v>
       </c>
       <c r="H104" s="11"/>
       <c r="I104" s="11"/>
       <c r="J104" s="6"/>
       <c r="K104" s="10">
         <f t="shared" ref="K104:K115" si="18">G104/B104</f>
-        <v>11.064744562468388</v>
+        <v>0</v>
       </c>
       <c r="L104" s="10"/>
       <c r="M104" s="10"/>
@@ -3954,21 +3948,21 @@
         <v>9.8849999999999997E-3</v>
       </c>
       <c r="C105" s="11">
-        <v>2.6148000000000001E-2</v>
+        <v>9.8849999999999997E-3</v>
       </c>
       <c r="D105" s="11"/>
       <c r="E105" s="11"/>
       <c r="F105" s="6"/>
       <c r="G105" s="11">
         <f t="shared" si="17"/>
-        <v>1.6263E-2</v>
+        <v>0</v>
       </c>
       <c r="H105" s="11"/>
       <c r="I105" s="11"/>
       <c r="J105" s="6"/>
       <c r="K105" s="10">
         <f t="shared" si="18"/>
-        <v>1.6452200303490137</v>
+        <v>0</v>
       </c>
       <c r="L105" s="10"/>
       <c r="M105" s="10"/>
@@ -3994,9 +3988,8 @@
       <c r="H106" s="11"/>
       <c r="I106" s="11"/>
       <c r="J106" s="6"/>
-      <c r="K106" s="10" t="e">
-        <f t="shared" si="18"/>
-        <v>#DIV/0!</v>
+      <c r="K106" s="10">
+        <v>0</v>
       </c>
       <c r="L106" s="10"/>
       <c r="M106" s="10"/>
@@ -4022,9 +4015,8 @@
       <c r="H107" s="11"/>
       <c r="I107" s="11"/>
       <c r="J107" s="6"/>
-      <c r="K107" s="10" t="e">
-        <f t="shared" si="18"/>
-        <v>#DIV/0!</v>
+      <c r="K107" s="10">
+        <v>0</v>
       </c>
       <c r="L107" s="10"/>
       <c r="M107" s="10"/>
@@ -4066,21 +4058,20 @@
         <v>0</v>
       </c>
       <c r="C109" s="11">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="D109" s="11"/>
       <c r="E109" s="11"/>
       <c r="F109" s="6"/>
       <c r="G109" s="11">
         <f t="shared" si="17"/>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H109" s="11"/>
       <c r="I109" s="11"/>
       <c r="J109" s="6"/>
-      <c r="K109" s="10" t="e">
-        <f t="shared" si="18"/>
-        <v>#DIV/0!</v>
+      <c r="K109" s="10">
+        <v>0</v>
       </c>
       <c r="L109" s="10"/>
       <c r="M109" s="10"/>
@@ -4094,21 +4085,21 @@
         <v>7.9901150000000003</v>
       </c>
       <c r="C110" s="11">
-        <v>7.9846940000000002</v>
+        <v>7.9901150000000003</v>
       </c>
       <c r="D110" s="11"/>
       <c r="E110" s="11"/>
       <c r="F110" s="6"/>
       <c r="G110" s="11">
         <f t="shared" si="17"/>
-        <v>-5.4210000000001202E-3</v>
+        <v>0</v>
       </c>
       <c r="H110" s="11"/>
       <c r="I110" s="11"/>
       <c r="J110" s="6"/>
       <c r="K110" s="10">
         <f t="shared" si="18"/>
-        <v>-6.7846332624750961E-4</v>
+        <v>0</v>
       </c>
       <c r="L110" s="10"/>
       <c r="M110" s="10"/>
@@ -4178,21 +4169,21 @@
         <v>7</v>
       </c>
       <c r="C113" s="11">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D113" s="11"/>
       <c r="E113" s="11"/>
       <c r="F113" s="6"/>
       <c r="G113" s="11">
         <f t="shared" si="17"/>
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="H113" s="11"/>
       <c r="I113" s="11"/>
       <c r="J113" s="6"/>
       <c r="K113" s="10">
         <f t="shared" si="18"/>
-        <v>-0.2857142857142857</v>
+        <v>0</v>
       </c>
       <c r="L113" s="10"/>
       <c r="M113" s="10"/>
@@ -4206,21 +4197,21 @@
         <v>3105</v>
       </c>
       <c r="C114" s="11">
-        <v>3093</v>
+        <v>3105</v>
       </c>
       <c r="D114" s="11"/>
       <c r="E114" s="11"/>
       <c r="F114" s="6"/>
       <c r="G114" s="11">
         <f t="shared" si="17"/>
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="H114" s="11"/>
       <c r="I114" s="11"/>
       <c r="J114" s="6"/>
       <c r="K114" s="10">
         <f t="shared" si="18"/>
-        <v>-3.8647342995169081E-3</v>
+        <v>0</v>
       </c>
       <c r="L114" s="10"/>
       <c r="M114" s="10"/>
@@ -4234,21 +4225,21 @@
         <v>0.99011479999999996</v>
       </c>
       <c r="C115" s="10">
-        <v>0.98628826999999997</v>
+        <v>0.99011479999999996</v>
       </c>
       <c r="D115" s="10"/>
       <c r="E115" s="10"/>
       <c r="F115" s="6"/>
       <c r="G115" s="11">
         <f t="shared" si="17"/>
-        <v>-3.8265299999999947E-3</v>
+        <v>0</v>
       </c>
       <c r="H115" s="11"/>
       <c r="I115" s="11"/>
       <c r="J115" s="6"/>
       <c r="K115" s="10">
         <f t="shared" si="18"/>
-        <v>-3.8647336652275015E-3</v>
+        <v>0</v>
       </c>
       <c r="L115" s="10"/>
       <c r="M115" s="10"/>
@@ -4299,7 +4290,8 @@
         <v>32</v>
       </c>
       <c r="B118" s="1">
-        <v>36.935268000000001</v>
+        <f>AVERAGE(B62,B34,B90)</f>
+        <v>57.957057999999996</v>
       </c>
       <c r="C118" s="11">
         <f>AVERAGE(C62,C34,C90)</f>
@@ -4310,14 +4302,14 @@
       <c r="F118" s="6"/>
       <c r="G118" s="11">
         <f t="shared" ref="G118:G129" si="19">C118-B118</f>
-        <v>19.180059333333332</v>
+        <v>-1.8417306666666633</v>
       </c>
       <c r="H118" s="11"/>
       <c r="I118" s="11"/>
       <c r="J118" s="6"/>
       <c r="K118" s="10">
         <f>G118/B118</f>
-        <v>0.51928848420250617</v>
+        <v>-3.17775044182999E-2</v>
       </c>
       <c r="L118" s="10"/>
       <c r="M118" s="10"/>
@@ -4328,10 +4320,11 @@
         <v>33</v>
       </c>
       <c r="B119" s="1">
-        <v>4.1183040000000002</v>
+        <f t="shared" ref="B119:B128" si="20">AVERAGE(B63,B35,B91)</f>
+        <v>5.2387329999999999</v>
       </c>
       <c r="C119" s="11">
-        <f t="shared" ref="C119:C129" si="20">AVERAGE(C63,C35,C91)</f>
+        <f t="shared" ref="C119:C129" si="21">AVERAGE(C63,C35,C91)</f>
         <v>5.1716623333333329</v>
       </c>
       <c r="D119" s="11"/>
@@ -4339,14 +4332,14 @@
       <c r="F119" s="6"/>
       <c r="G119" s="11">
         <f t="shared" si="19"/>
-        <v>1.0533583333333327</v>
+        <v>-6.7070666666666945E-2</v>
       </c>
       <c r="H119" s="11"/>
       <c r="I119" s="11"/>
       <c r="J119" s="6"/>
       <c r="K119" s="10">
         <f>G119/B119</f>
-        <v>0.25577478819760091</v>
+        <v>-1.2802841195889722E-2</v>
       </c>
       <c r="L119" s="10"/>
       <c r="M119" s="10"/>
@@ -4357,10 +4350,11 @@
         <v>34</v>
       </c>
       <c r="B120" s="1">
-        <v>2</v>
+        <f t="shared" si="20"/>
+        <v>4</v>
       </c>
       <c r="C120" s="11">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>4</v>
       </c>
       <c r="D120" s="11"/>
@@ -4368,14 +4362,14 @@
       <c r="F120" s="6"/>
       <c r="G120" s="11">
         <f t="shared" si="19"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H120" s="11"/>
       <c r="I120" s="11"/>
       <c r="J120" s="6"/>
       <c r="K120" s="10">
         <f>G120/B120</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L120" s="10"/>
       <c r="M120" s="10"/>
@@ -4386,10 +4380,11 @@
         <v>35</v>
       </c>
       <c r="B121" s="1">
-        <v>2</v>
+        <f t="shared" si="20"/>
+        <v>4</v>
       </c>
       <c r="C121" s="11">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>4</v>
       </c>
       <c r="D121" s="11"/>
@@ -4397,14 +4392,14 @@
       <c r="F121" s="6"/>
       <c r="G121" s="11">
         <f t="shared" si="19"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H121" s="11"/>
       <c r="I121" s="11"/>
       <c r="J121" s="6"/>
       <c r="K121" s="10">
         <f>G121/B121</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L121" s="10"/>
       <c r="M121" s="10"/>
@@ -4415,10 +4410,11 @@
         <v>36</v>
       </c>
       <c r="B122" s="1">
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="C122" s="11">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="D122" s="11"/>
@@ -4443,10 +4439,11 @@
         <v>37</v>
       </c>
       <c r="B123" s="1">
-        <v>23</v>
+        <f t="shared" si="20"/>
+        <v>25</v>
       </c>
       <c r="C123" s="11">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>24.666666666666668</v>
       </c>
       <c r="D123" s="11"/>
@@ -4454,14 +4451,14 @@
       <c r="F123" s="6"/>
       <c r="G123" s="11">
         <f t="shared" si="19"/>
-        <v>1.6666666666666679</v>
+        <v>-0.33333333333333215</v>
       </c>
       <c r="H123" s="11"/>
       <c r="I123" s="11"/>
       <c r="J123" s="6"/>
       <c r="K123" s="10">
-        <f t="shared" ref="K123:K129" si="21">G123/B123</f>
-        <v>7.2463768115942087E-2</v>
+        <f t="shared" ref="K123:K129" si="22">G123/B123</f>
+        <v>-1.3333333333333286E-2</v>
       </c>
       <c r="L123" s="10"/>
       <c r="M123" s="10"/>
@@ -4472,10 +4469,11 @@
         <v>38</v>
       </c>
       <c r="B124" s="1">
-        <v>6.6195789999999999</v>
+        <f t="shared" si="20"/>
+        <v>6.4259139999999997</v>
       </c>
       <c r="C124" s="11">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>6.4202806666666667</v>
       </c>
       <c r="D124" s="11"/>
@@ -4483,14 +4481,14 @@
       <c r="F124" s="6"/>
       <c r="G124" s="11">
         <f t="shared" si="19"/>
-        <v>-0.19929833333333313</v>
+        <v>-5.633333333332935E-3</v>
       </c>
       <c r="H124" s="11"/>
       <c r="I124" s="11"/>
       <c r="J124" s="6"/>
       <c r="K124" s="10">
-        <f t="shared" si="21"/>
-        <v>-3.0107403104235653E-2</v>
+        <f t="shared" si="22"/>
+        <v>-8.7665868751634951E-4</v>
       </c>
       <c r="L124" s="10"/>
       <c r="M124" s="10"/>
@@ -4501,10 +4499,11 @@
         <v>39</v>
       </c>
       <c r="B125" s="1">
-        <v>7</v>
+        <f t="shared" si="20"/>
+        <v>6.666666666666667</v>
       </c>
       <c r="C125" s="11">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>6.666666666666667</v>
       </c>
       <c r="D125" s="11"/>
@@ -4512,14 +4511,14 @@
       <c r="F125" s="6"/>
       <c r="G125" s="11">
         <f t="shared" si="19"/>
-        <v>-0.33333333333333304</v>
+        <v>0</v>
       </c>
       <c r="H125" s="11"/>
       <c r="I125" s="11"/>
       <c r="J125" s="6"/>
       <c r="K125" s="10">
-        <f t="shared" si="21"/>
-        <v>-4.7619047619047575E-2</v>
+        <f t="shared" si="22"/>
+        <v>0</v>
       </c>
       <c r="L125" s="10"/>
       <c r="M125" s="10"/>
@@ -4530,10 +4529,11 @@
         <v>40</v>
       </c>
       <c r="B126" s="1">
+        <f t="shared" si="20"/>
         <v>8</v>
       </c>
       <c r="C126" s="11">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>8</v>
       </c>
       <c r="D126" s="11"/>
@@ -4547,7 +4547,7 @@
       <c r="I126" s="11"/>
       <c r="J126" s="6"/>
       <c r="K126" s="10">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="L126" s="10"/>
@@ -4559,10 +4559,11 @@
         <v>41</v>
       </c>
       <c r="B127" s="1">
-        <v>3</v>
+        <f t="shared" si="20"/>
+        <v>3.3333333333333335</v>
       </c>
       <c r="C127" s="11">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>3.3333333333333335</v>
       </c>
       <c r="D127" s="11"/>
@@ -4570,14 +4571,14 @@
       <c r="F127" s="6"/>
       <c r="G127" s="11">
         <f t="shared" si="19"/>
-        <v>0.33333333333333348</v>
+        <v>0</v>
       </c>
       <c r="H127" s="11"/>
       <c r="I127" s="11"/>
       <c r="J127" s="6"/>
       <c r="K127" s="10">
-        <f t="shared" si="21"/>
-        <v>0.11111111111111116</v>
+        <f t="shared" si="22"/>
+        <v>0</v>
       </c>
       <c r="L127" s="10"/>
       <c r="M127" s="10"/>
@@ -4588,10 +4589,11 @@
         <v>76</v>
       </c>
       <c r="B128" s="1">
-        <v>471</v>
+        <f t="shared" si="20"/>
+        <v>235</v>
       </c>
       <c r="C128" s="11">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>224</v>
       </c>
       <c r="D128" s="11"/>
@@ -4599,14 +4601,14 @@
       <c r="F128" s="6"/>
       <c r="G128" s="11">
         <f t="shared" si="19"/>
-        <v>-247</v>
+        <v>-11</v>
       </c>
       <c r="H128" s="11"/>
       <c r="I128" s="11"/>
       <c r="J128" s="6"/>
       <c r="K128" s="10">
-        <f t="shared" si="21"/>
-        <v>-0.52441613588110403</v>
+        <f t="shared" si="22"/>
+        <v>-4.6808510638297871E-2</v>
       </c>
       <c r="L128" s="10"/>
       <c r="M128" s="10"/>
@@ -4617,10 +4619,11 @@
         <v>42</v>
       </c>
       <c r="B129" s="5">
-        <v>0.15019133000000001</v>
-      </c>
-      <c r="C129" s="13">
-        <f t="shared" si="20"/>
+        <f>AVERAGE(B73,B45,B101)</f>
+        <v>7.4936223333333329E-2</v>
+      </c>
+      <c r="C129" s="14">
+        <f t="shared" si="21"/>
         <v>7.1428570000000011E-2</v>
       </c>
       <c r="D129" s="11"/>
@@ -4628,14 +4631,14 @@
       <c r="F129" s="6"/>
       <c r="G129" s="11">
         <f t="shared" si="19"/>
-        <v>-7.8762760000000001E-2</v>
+        <v>-3.5076533333333187E-3</v>
       </c>
       <c r="H129" s="11"/>
       <c r="I129" s="11"/>
       <c r="J129" s="6"/>
       <c r="K129" s="10">
-        <f t="shared" si="21"/>
-        <v>-0.52441615637866712</v>
+        <f t="shared" si="22"/>
+        <v>-4.6808514991881572E-2</v>
       </c>
       <c r="L129" s="10"/>
       <c r="M129" s="10"/>
@@ -4686,25 +4689,26 @@
         <v>43</v>
       </c>
       <c r="B132" s="1">
-        <v>3.401786</v>
+        <f>AVERAGE(B76,B48,B104)</f>
+        <v>1.1305270000000001</v>
       </c>
       <c r="C132" s="11">
         <f>AVERAGE(C76,C48,C104)</f>
-        <v>1.1753826666666667</v>
+        <v>1.1316963333333334</v>
       </c>
       <c r="D132" s="11"/>
       <c r="E132" s="11"/>
       <c r="F132" s="6"/>
       <c r="G132" s="11">
-        <f t="shared" ref="G132:G143" si="22">C132-B132</f>
-        <v>-2.2264033333333333</v>
+        <f t="shared" ref="G132:G143" si="23">C132-B132</f>
+        <v>1.1693333333333555E-3</v>
       </c>
       <c r="H132" s="11"/>
       <c r="I132" s="11"/>
       <c r="J132" s="6"/>
       <c r="K132" s="10">
-        <f t="shared" ref="K132:K143" si="23">G132/B132</f>
-        <v>-0.65448071493425319</v>
+        <f t="shared" ref="K132:K143" si="24">G132/B132</f>
+        <v>1.0343258792875848E-3</v>
       </c>
       <c r="L132" s="10"/>
       <c r="M132" s="10"/>
@@ -4715,25 +4719,26 @@
         <v>44</v>
       </c>
       <c r="B133" s="1">
-        <v>1.770408</v>
+        <f t="shared" ref="B133:B142" si="25">AVERAGE(B77,B49,B105)</f>
+        <v>0.59204933333333332</v>
       </c>
       <c r="C133" s="11">
-        <f t="shared" ref="C133:C143" si="24">AVERAGE(C77,C49,C105)</f>
-        <v>0.5994896666666667</v>
+        <f t="shared" ref="C133:C143" si="26">AVERAGE(C77,C49,C105)</f>
+        <v>0.59258066666666664</v>
       </c>
       <c r="D133" s="11"/>
       <c r="E133" s="11"/>
       <c r="F133" s="6"/>
       <c r="G133" s="11">
-        <f t="shared" si="22"/>
-        <v>-1.1709183333333333</v>
+        <f t="shared" si="23"/>
+        <v>5.3133333333332811E-4</v>
       </c>
       <c r="H133" s="11"/>
       <c r="I133" s="11"/>
       <c r="J133" s="6"/>
       <c r="K133" s="10">
-        <f t="shared" si="23"/>
-        <v>-0.6613833270824202</v>
+        <f t="shared" si="24"/>
+        <v>8.9744773521124616E-4</v>
       </c>
       <c r="L133" s="10"/>
       <c r="M133" s="10"/>
@@ -4744,25 +4749,26 @@
         <v>45</v>
       </c>
       <c r="B134" s="1">
-        <v>2</v>
+        <f t="shared" si="25"/>
+        <v>0.66666666666666663</v>
       </c>
       <c r="C134" s="11">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>0.66666666666666663</v>
       </c>
       <c r="D134" s="11"/>
       <c r="E134" s="11"/>
       <c r="F134" s="6"/>
       <c r="G134" s="11">
-        <f t="shared" si="22"/>
-        <v>-1.3333333333333335</v>
+        <f t="shared" si="23"/>
+        <v>0</v>
       </c>
       <c r="H134" s="11"/>
       <c r="I134" s="11"/>
       <c r="J134" s="6"/>
       <c r="K134" s="10">
-        <f t="shared" si="23"/>
-        <v>-0.66666666666666674</v>
+        <f t="shared" si="24"/>
+        <v>0</v>
       </c>
       <c r="L134" s="10"/>
       <c r="M134" s="10"/>
@@ -4773,25 +4779,26 @@
         <v>46</v>
       </c>
       <c r="B135" s="1">
-        <v>-2</v>
+        <f t="shared" si="25"/>
+        <v>-0.66666666666666663</v>
       </c>
       <c r="C135" s="11">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>-0.66666666666666663</v>
       </c>
       <c r="D135" s="11"/>
       <c r="E135" s="11"/>
       <c r="F135" s="6"/>
       <c r="G135" s="11">
-        <f t="shared" si="22"/>
-        <v>1.3333333333333335</v>
+        <f t="shared" si="23"/>
+        <v>0</v>
       </c>
       <c r="H135" s="11"/>
       <c r="I135" s="11"/>
       <c r="J135" s="6"/>
       <c r="K135" s="10">
-        <f t="shared" si="23"/>
-        <v>-0.66666666666666674</v>
+        <f t="shared" si="24"/>
+        <v>0</v>
       </c>
       <c r="L135" s="10"/>
       <c r="M135" s="10"/>
@@ -4802,25 +4809,26 @@
         <v>47</v>
       </c>
       <c r="B136" s="1">
-        <v>-3</v>
+        <f t="shared" si="25"/>
+        <v>-1.3333333333333333</v>
       </c>
       <c r="C136" s="11">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>-1.3333333333333333</v>
       </c>
       <c r="D136" s="11"/>
       <c r="E136" s="11"/>
       <c r="F136" s="6"/>
       <c r="G136" s="11">
-        <f t="shared" si="22"/>
-        <v>1.6666666666666667</v>
+        <f t="shared" si="23"/>
+        <v>0</v>
       </c>
       <c r="H136" s="11"/>
       <c r="I136" s="11"/>
       <c r="J136" s="6"/>
       <c r="K136" s="10">
-        <f t="shared" si="23"/>
-        <v>-0.55555555555555558</v>
+        <f t="shared" si="24"/>
+        <v>0</v>
       </c>
       <c r="L136" s="10"/>
       <c r="M136" s="10"/>
@@ -4831,25 +4839,26 @@
         <v>48</v>
       </c>
       <c r="B137" s="1">
-        <v>2</v>
+        <f t="shared" si="25"/>
+        <v>0.66666666666666663</v>
       </c>
       <c r="C137" s="11">
-        <f t="shared" si="24"/>
-        <v>4.333333333333333</v>
+        <f t="shared" si="26"/>
+        <v>0.66666666666666663</v>
       </c>
       <c r="D137" s="11"/>
       <c r="E137" s="11"/>
       <c r="F137" s="6"/>
       <c r="G137" s="11">
-        <f t="shared" si="22"/>
-        <v>2.333333333333333</v>
+        <f t="shared" si="23"/>
+        <v>0</v>
       </c>
       <c r="H137" s="11"/>
       <c r="I137" s="11"/>
       <c r="J137" s="6"/>
       <c r="K137" s="10">
-        <f t="shared" si="23"/>
-        <v>1.1666666666666665</v>
+        <f t="shared" si="24"/>
+        <v>0</v>
       </c>
       <c r="L137" s="10"/>
       <c r="M137" s="10"/>
@@ -4860,25 +4869,26 @@
         <v>49</v>
       </c>
       <c r="B138" s="1">
-        <v>6.7904970000000002</v>
+        <f t="shared" si="25"/>
+        <v>7.5946003333333332</v>
       </c>
       <c r="C138" s="11">
-        <f t="shared" si="24"/>
-        <v>7.5915180000000007</v>
+        <f t="shared" si="26"/>
+        <v>7.5944940000000001</v>
       </c>
       <c r="D138" s="11"/>
       <c r="E138" s="11"/>
       <c r="F138" s="6"/>
       <c r="G138" s="11">
-        <f t="shared" si="22"/>
-        <v>0.80102100000000043</v>
+        <f t="shared" si="23"/>
+        <v>-1.0633333333309736E-4</v>
       </c>
       <c r="H138" s="11"/>
       <c r="I138" s="11"/>
       <c r="J138" s="6"/>
       <c r="K138" s="10">
-        <f t="shared" si="23"/>
-        <v>0.11796205785820985</v>
+        <f t="shared" si="24"/>
+        <v>-1.4001175659816029E-5</v>
       </c>
       <c r="L138" s="10"/>
       <c r="M138" s="10"/>
@@ -4889,25 +4899,26 @@
         <v>50</v>
       </c>
       <c r="B139" s="1">
-        <v>7</v>
+        <f t="shared" si="25"/>
+        <v>7.666666666666667</v>
       </c>
       <c r="C139" s="11">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>7.666666666666667</v>
       </c>
       <c r="D139" s="11"/>
       <c r="E139" s="11"/>
       <c r="F139" s="6"/>
       <c r="G139" s="11">
-        <f t="shared" si="22"/>
-        <v>0.66666666666666696</v>
+        <f t="shared" si="23"/>
+        <v>0</v>
       </c>
       <c r="H139" s="11"/>
       <c r="I139" s="11"/>
       <c r="J139" s="6"/>
       <c r="K139" s="10">
-        <f t="shared" si="23"/>
-        <v>9.5238095238095274E-2</v>
+        <f t="shared" si="24"/>
+        <v>0</v>
       </c>
       <c r="L139" s="10"/>
       <c r="M139" s="10"/>
@@ -4918,24 +4929,25 @@
         <v>51</v>
       </c>
       <c r="B140" s="1">
+        <f t="shared" si="25"/>
         <v>8</v>
       </c>
       <c r="C140" s="11">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>8</v>
       </c>
       <c r="D140" s="11"/>
       <c r="E140" s="11"/>
       <c r="F140" s="6"/>
       <c r="G140" s="11">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="H140" s="11"/>
       <c r="I140" s="11"/>
       <c r="J140" s="6"/>
       <c r="K140" s="10">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="L140" s="10"/>
@@ -4947,25 +4959,26 @@
         <v>52</v>
       </c>
       <c r="B141" s="1">
-        <v>5</v>
+        <f t="shared" si="25"/>
+        <v>6.666666666666667</v>
       </c>
       <c r="C141" s="11">
-        <f t="shared" si="24"/>
-        <v>6</v>
+        <f t="shared" si="26"/>
+        <v>6.666666666666667</v>
       </c>
       <c r="D141" s="11"/>
       <c r="E141" s="11"/>
       <c r="F141" s="6"/>
       <c r="G141" s="11">
-        <f t="shared" si="22"/>
-        <v>1</v>
+        <f t="shared" si="23"/>
+        <v>0</v>
       </c>
       <c r="H141" s="11"/>
       <c r="I141" s="11"/>
       <c r="J141" s="6"/>
       <c r="K141" s="10">
-        <f t="shared" si="23"/>
-        <v>0.2</v>
+        <f t="shared" si="24"/>
+        <v>0</v>
       </c>
       <c r="L141" s="10"/>
       <c r="M141" s="10"/>
@@ -4976,25 +4989,26 @@
         <v>77</v>
       </c>
       <c r="B142" s="1">
-        <v>61</v>
+        <f t="shared" si="25"/>
+        <v>2100.6666666666665</v>
       </c>
       <c r="C142" s="11">
         <f>AVERAGE(C86,C58,C114)</f>
-        <v>2096.3333333333335</v>
+        <v>2100.3333333333335</v>
       </c>
       <c r="D142" s="11"/>
       <c r="E142" s="11"/>
       <c r="F142" s="6"/>
       <c r="G142" s="11">
-        <f t="shared" si="22"/>
-        <v>2035.3333333333335</v>
+        <f t="shared" si="23"/>
+        <v>-0.33333333333303017</v>
       </c>
       <c r="H142" s="11"/>
       <c r="I142" s="11"/>
       <c r="J142" s="6"/>
       <c r="K142" s="10">
-        <f t="shared" si="23"/>
-        <v>33.36612021857924</v>
+        <f t="shared" si="24"/>
+        <v>-1.5867978419534918E-4</v>
       </c>
       <c r="L142" s="10"/>
       <c r="M142" s="10"/>
@@ -5005,25 +5019,26 @@
         <v>53</v>
       </c>
       <c r="B143" s="5">
-        <v>1.9451530000000002E-2</v>
-      </c>
-      <c r="C143" s="13">
-        <f t="shared" si="24"/>
-        <v>0.66847363999999987</v>
+        <f>AVERAGE(B87,B59,B115)</f>
+        <v>0.66985544333333336</v>
+      </c>
+      <c r="C143" s="14">
+        <f t="shared" si="26"/>
+        <v>0.66974915000000002</v>
       </c>
       <c r="D143" s="11"/>
       <c r="E143" s="11"/>
       <c r="F143" s="6"/>
       <c r="G143" s="11">
-        <f t="shared" si="22"/>
-        <v>0.64902210999999987</v>
+        <f t="shared" si="23"/>
+        <v>-1.0629333333334046E-4</v>
       </c>
       <c r="H143" s="11"/>
       <c r="I143" s="11"/>
       <c r="J143" s="6"/>
       <c r="K143" s="10">
-        <f t="shared" si="23"/>
-        <v>33.366121328245121</v>
+        <f t="shared" si="24"/>
+        <v>-1.5868100258229414E-4</v>
       </c>
       <c r="L143" s="10"/>
       <c r="M143" s="10"/>
@@ -5062,11 +5077,11 @@
       <c r="H145" s="11"/>
       <c r="I145" s="11"/>
       <c r="J145" s="6"/>
-      <c r="K145" s="15">
-        <v>0</v>
-      </c>
-      <c r="L145" s="15"/>
-      <c r="M145" s="15"/>
+      <c r="K145" s="13">
+        <v>0</v>
+      </c>
+      <c r="L145" s="13"/>
+      <c r="M145" s="13"/>
       <c r="N145" s="6"/>
     </row>
     <row r="146" spans="1:14" x14ac:dyDescent="0.2">
@@ -5315,7 +5330,7 @@
         <v>-8.0530056000001196</v>
       </c>
       <c r="H154" s="1">
-        <f t="shared" ref="H154" si="25">D154-B154</f>
+        <f t="shared" ref="H154" si="27">D154-B154</f>
         <v>33.1681319999999</v>
       </c>
       <c r="I154" s="1">
@@ -5328,7 +5343,7 @@
         <v>-8.4326779171183582E-3</v>
       </c>
       <c r="L154" s="5">
-        <f t="shared" ref="L154" si="26">H154/B154</f>
+        <f t="shared" ref="L154" si="28">H154/B154</f>
         <v>3.4731898642720645E-2</v>
       </c>
       <c r="M154" s="5">
@@ -5389,6 +5404,342 @@
     </row>
   </sheetData>
   <mergeCells count="360">
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="G59:I59"/>
+    <mergeCell ref="K59:M59"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="G56:I56"/>
+    <mergeCell ref="K56:M56"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="G57:I57"/>
+    <mergeCell ref="K57:M57"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="G58:I58"/>
+    <mergeCell ref="K58:M58"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="G53:I53"/>
+    <mergeCell ref="K53:M53"/>
+    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="G54:I54"/>
+    <mergeCell ref="K54:M54"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="G55:I55"/>
+    <mergeCell ref="K55:M55"/>
+    <mergeCell ref="C50:E50"/>
+    <mergeCell ref="G50:I50"/>
+    <mergeCell ref="K50:M50"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="G51:I51"/>
+    <mergeCell ref="K51:M51"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="G52:I52"/>
+    <mergeCell ref="K52:M52"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="G47:I47"/>
+    <mergeCell ref="K47:M47"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="G48:I48"/>
+    <mergeCell ref="K48:M48"/>
+    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="G49:I49"/>
+    <mergeCell ref="K49:M49"/>
+    <mergeCell ref="C43:E43"/>
+    <mergeCell ref="G43:I43"/>
+    <mergeCell ref="K43:M43"/>
+    <mergeCell ref="C44:E44"/>
+    <mergeCell ref="G44:I44"/>
+    <mergeCell ref="K44:M44"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="G45:I45"/>
+    <mergeCell ref="K45:M45"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="G40:I40"/>
+    <mergeCell ref="K40:M40"/>
+    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="G41:I41"/>
+    <mergeCell ref="K41:M41"/>
+    <mergeCell ref="C42:E42"/>
+    <mergeCell ref="G42:I42"/>
+    <mergeCell ref="K42:M42"/>
+    <mergeCell ref="C87:E87"/>
+    <mergeCell ref="G87:I87"/>
+    <mergeCell ref="K87:M87"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="K33:M33"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="K34:M34"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="K35:M35"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="G36:I36"/>
+    <mergeCell ref="K36:M36"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="G37:I37"/>
+    <mergeCell ref="K37:M37"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="G38:I38"/>
+    <mergeCell ref="K38:M38"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="G39:I39"/>
+    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="C84:E84"/>
+    <mergeCell ref="G84:I84"/>
+    <mergeCell ref="K84:M84"/>
+    <mergeCell ref="C85:E85"/>
+    <mergeCell ref="G85:I85"/>
+    <mergeCell ref="K85:M85"/>
+    <mergeCell ref="C86:E86"/>
+    <mergeCell ref="G86:I86"/>
+    <mergeCell ref="K86:M86"/>
+    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="G81:I81"/>
+    <mergeCell ref="K81:M81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="G82:I82"/>
+    <mergeCell ref="K82:M82"/>
+    <mergeCell ref="C83:E83"/>
+    <mergeCell ref="G83:I83"/>
+    <mergeCell ref="K83:M83"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="G78:I78"/>
+    <mergeCell ref="K78:M78"/>
+    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="G79:I79"/>
+    <mergeCell ref="K79:M79"/>
+    <mergeCell ref="C80:E80"/>
+    <mergeCell ref="G80:I80"/>
+    <mergeCell ref="K80:M80"/>
+    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="G75:I75"/>
+    <mergeCell ref="K75:M75"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="G76:I76"/>
+    <mergeCell ref="K76:M76"/>
+    <mergeCell ref="C77:E77"/>
+    <mergeCell ref="G77:I77"/>
+    <mergeCell ref="K77:M77"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="G71:I71"/>
+    <mergeCell ref="K71:M71"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="G72:I72"/>
+    <mergeCell ref="K72:M72"/>
+    <mergeCell ref="C73:E73"/>
+    <mergeCell ref="G73:I73"/>
+    <mergeCell ref="K73:M73"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="G68:I68"/>
+    <mergeCell ref="K68:M68"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="G69:I69"/>
+    <mergeCell ref="K69:M69"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="G70:I70"/>
+    <mergeCell ref="K70:M70"/>
+    <mergeCell ref="C115:E115"/>
+    <mergeCell ref="G115:I115"/>
+    <mergeCell ref="K115:M115"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="G61:I61"/>
+    <mergeCell ref="K61:M61"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="G62:I62"/>
+    <mergeCell ref="K62:M62"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="G63:I63"/>
+    <mergeCell ref="K63:M63"/>
+    <mergeCell ref="C64:E64"/>
+    <mergeCell ref="G64:I64"/>
+    <mergeCell ref="K64:M64"/>
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="G65:I65"/>
+    <mergeCell ref="K65:M65"/>
+    <mergeCell ref="C66:E66"/>
+    <mergeCell ref="G66:I66"/>
+    <mergeCell ref="K66:M66"/>
+    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="G67:I67"/>
+    <mergeCell ref="K67:M67"/>
+    <mergeCell ref="C112:E112"/>
+    <mergeCell ref="G112:I112"/>
+    <mergeCell ref="K112:M112"/>
+    <mergeCell ref="C113:E113"/>
+    <mergeCell ref="G113:I113"/>
+    <mergeCell ref="K113:M113"/>
+    <mergeCell ref="C114:E114"/>
+    <mergeCell ref="G114:I114"/>
+    <mergeCell ref="K114:M114"/>
+    <mergeCell ref="C109:E109"/>
+    <mergeCell ref="G109:I109"/>
+    <mergeCell ref="K109:M109"/>
+    <mergeCell ref="C110:E110"/>
+    <mergeCell ref="G110:I110"/>
+    <mergeCell ref="K110:M110"/>
+    <mergeCell ref="C111:E111"/>
+    <mergeCell ref="G111:I111"/>
+    <mergeCell ref="K111:M111"/>
+    <mergeCell ref="C106:E106"/>
+    <mergeCell ref="G106:I106"/>
+    <mergeCell ref="K106:M106"/>
+    <mergeCell ref="C107:E107"/>
+    <mergeCell ref="G107:I107"/>
+    <mergeCell ref="K107:M107"/>
+    <mergeCell ref="C108:E108"/>
+    <mergeCell ref="G108:I108"/>
+    <mergeCell ref="K108:M108"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="G103:I103"/>
+    <mergeCell ref="K103:M103"/>
+    <mergeCell ref="C104:E104"/>
+    <mergeCell ref="G104:I104"/>
+    <mergeCell ref="K104:M104"/>
+    <mergeCell ref="C105:E105"/>
+    <mergeCell ref="G105:I105"/>
+    <mergeCell ref="K105:M105"/>
+    <mergeCell ref="C99:E99"/>
+    <mergeCell ref="G99:I99"/>
+    <mergeCell ref="K99:M99"/>
+    <mergeCell ref="C100:E100"/>
+    <mergeCell ref="G100:I100"/>
+    <mergeCell ref="K100:M100"/>
+    <mergeCell ref="C101:E101"/>
+    <mergeCell ref="G101:I101"/>
+    <mergeCell ref="K101:M101"/>
+    <mergeCell ref="G95:I95"/>
+    <mergeCell ref="K95:M95"/>
+    <mergeCell ref="C96:E96"/>
+    <mergeCell ref="G96:I96"/>
+    <mergeCell ref="K96:M96"/>
+    <mergeCell ref="C97:E97"/>
+    <mergeCell ref="G97:I97"/>
+    <mergeCell ref="K97:M97"/>
+    <mergeCell ref="C98:E98"/>
+    <mergeCell ref="G98:I98"/>
+    <mergeCell ref="K98:M98"/>
+    <mergeCell ref="B117:E117"/>
+    <mergeCell ref="B131:E131"/>
+    <mergeCell ref="G131:I131"/>
+    <mergeCell ref="K131:M131"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="G89:I89"/>
+    <mergeCell ref="K89:M89"/>
+    <mergeCell ref="C90:E90"/>
+    <mergeCell ref="G90:I90"/>
+    <mergeCell ref="K90:M90"/>
+    <mergeCell ref="C91:E91"/>
+    <mergeCell ref="G91:I91"/>
+    <mergeCell ref="K91:M91"/>
+    <mergeCell ref="C92:E92"/>
+    <mergeCell ref="G92:I92"/>
+    <mergeCell ref="K92:M92"/>
+    <mergeCell ref="C93:E93"/>
+    <mergeCell ref="G93:I93"/>
+    <mergeCell ref="K93:M93"/>
+    <mergeCell ref="C94:E94"/>
+    <mergeCell ref="G94:I94"/>
+    <mergeCell ref="K94:M94"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="C127:E127"/>
+    <mergeCell ref="K133:M133"/>
+    <mergeCell ref="K143:M143"/>
+    <mergeCell ref="K135:M135"/>
+    <mergeCell ref="K136:M136"/>
+    <mergeCell ref="K137:M137"/>
+    <mergeCell ref="K138:M138"/>
+    <mergeCell ref="K139:M139"/>
+    <mergeCell ref="K117:M117"/>
+    <mergeCell ref="G117:I117"/>
+    <mergeCell ref="K122:M122"/>
+    <mergeCell ref="K123:M123"/>
+    <mergeCell ref="K124:M124"/>
+    <mergeCell ref="K125:M125"/>
+    <mergeCell ref="K126:M126"/>
+    <mergeCell ref="K127:M127"/>
+    <mergeCell ref="K128:M128"/>
+    <mergeCell ref="K129:M129"/>
+    <mergeCell ref="K132:M132"/>
+    <mergeCell ref="C128:E128"/>
+    <mergeCell ref="C129:E129"/>
+    <mergeCell ref="C137:E137"/>
+    <mergeCell ref="C141:E141"/>
+    <mergeCell ref="C142:E142"/>
+    <mergeCell ref="C143:E143"/>
+    <mergeCell ref="G132:I132"/>
+    <mergeCell ref="G133:I133"/>
+    <mergeCell ref="G134:I134"/>
+    <mergeCell ref="G135:I135"/>
+    <mergeCell ref="G136:I136"/>
+    <mergeCell ref="G137:I137"/>
+    <mergeCell ref="G138:I138"/>
+    <mergeCell ref="G139:I139"/>
+    <mergeCell ref="G140:I140"/>
+    <mergeCell ref="G141:I141"/>
+    <mergeCell ref="G142:I142"/>
+    <mergeCell ref="G143:I143"/>
+    <mergeCell ref="C136:E136"/>
+    <mergeCell ref="B147:E147"/>
+    <mergeCell ref="B148:E148"/>
+    <mergeCell ref="B149:E149"/>
+    <mergeCell ref="B150:E150"/>
+    <mergeCell ref="C138:E138"/>
+    <mergeCell ref="C139:E139"/>
+    <mergeCell ref="C140:E140"/>
+    <mergeCell ref="G129:I129"/>
+    <mergeCell ref="C132:E132"/>
+    <mergeCell ref="C133:E133"/>
+    <mergeCell ref="C134:E134"/>
+    <mergeCell ref="C135:E135"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="B145:E145"/>
+    <mergeCell ref="G118:I118"/>
+    <mergeCell ref="G119:I119"/>
+    <mergeCell ref="G120:I120"/>
+    <mergeCell ref="G121:I121"/>
+    <mergeCell ref="G122:I122"/>
+    <mergeCell ref="G123:I123"/>
+    <mergeCell ref="G124:I124"/>
+    <mergeCell ref="G125:I125"/>
+    <mergeCell ref="G126:I126"/>
+    <mergeCell ref="K145:M145"/>
+    <mergeCell ref="C118:E118"/>
+    <mergeCell ref="C119:E119"/>
+    <mergeCell ref="C120:E120"/>
+    <mergeCell ref="C121:E121"/>
+    <mergeCell ref="C122:E122"/>
+    <mergeCell ref="C123:E123"/>
+    <mergeCell ref="C124:E124"/>
+    <mergeCell ref="C125:E125"/>
+    <mergeCell ref="C126:E126"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="B153:D153"/>
+    <mergeCell ref="B155:D155"/>
+    <mergeCell ref="B151:D151"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="G127:I127"/>
+    <mergeCell ref="G128:I128"/>
+    <mergeCell ref="B152:E152"/>
+    <mergeCell ref="G145:I145"/>
+    <mergeCell ref="G146:I146"/>
+    <mergeCell ref="G147:I147"/>
+    <mergeCell ref="G148:I148"/>
+    <mergeCell ref="G149:I149"/>
+    <mergeCell ref="G150:I150"/>
+    <mergeCell ref="G152:I152"/>
+    <mergeCell ref="B146:E146"/>
     <mergeCell ref="L7:M7"/>
     <mergeCell ref="L8:M8"/>
     <mergeCell ref="L9:M9"/>
@@ -5413,342 +5764,6 @@
     <mergeCell ref="K119:M119"/>
     <mergeCell ref="K120:M120"/>
     <mergeCell ref="K121:M121"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="B153:D153"/>
-    <mergeCell ref="B155:D155"/>
-    <mergeCell ref="B151:D151"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="G127:I127"/>
-    <mergeCell ref="G128:I128"/>
-    <mergeCell ref="B152:E152"/>
-    <mergeCell ref="G145:I145"/>
-    <mergeCell ref="G146:I146"/>
-    <mergeCell ref="G147:I147"/>
-    <mergeCell ref="G148:I148"/>
-    <mergeCell ref="G149:I149"/>
-    <mergeCell ref="G150:I150"/>
-    <mergeCell ref="G152:I152"/>
-    <mergeCell ref="B146:E146"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="B145:E145"/>
-    <mergeCell ref="G118:I118"/>
-    <mergeCell ref="G119:I119"/>
-    <mergeCell ref="G120:I120"/>
-    <mergeCell ref="G121:I121"/>
-    <mergeCell ref="G122:I122"/>
-    <mergeCell ref="G123:I123"/>
-    <mergeCell ref="G124:I124"/>
-    <mergeCell ref="G125:I125"/>
-    <mergeCell ref="G126:I126"/>
-    <mergeCell ref="K145:M145"/>
-    <mergeCell ref="C118:E118"/>
-    <mergeCell ref="C119:E119"/>
-    <mergeCell ref="C120:E120"/>
-    <mergeCell ref="C121:E121"/>
-    <mergeCell ref="C122:E122"/>
-    <mergeCell ref="C123:E123"/>
-    <mergeCell ref="C124:E124"/>
-    <mergeCell ref="C125:E125"/>
-    <mergeCell ref="C126:E126"/>
-    <mergeCell ref="B147:E147"/>
-    <mergeCell ref="B148:E148"/>
-    <mergeCell ref="B149:E149"/>
-    <mergeCell ref="B150:E150"/>
-    <mergeCell ref="C138:E138"/>
-    <mergeCell ref="C139:E139"/>
-    <mergeCell ref="C140:E140"/>
-    <mergeCell ref="G129:I129"/>
-    <mergeCell ref="C132:E132"/>
-    <mergeCell ref="C133:E133"/>
-    <mergeCell ref="C134:E134"/>
-    <mergeCell ref="C135:E135"/>
-    <mergeCell ref="C128:E128"/>
-    <mergeCell ref="C129:E129"/>
-    <mergeCell ref="C137:E137"/>
-    <mergeCell ref="C141:E141"/>
-    <mergeCell ref="C142:E142"/>
-    <mergeCell ref="C143:E143"/>
-    <mergeCell ref="G132:I132"/>
-    <mergeCell ref="G133:I133"/>
-    <mergeCell ref="G134:I134"/>
-    <mergeCell ref="G135:I135"/>
-    <mergeCell ref="G136:I136"/>
-    <mergeCell ref="G137:I137"/>
-    <mergeCell ref="G138:I138"/>
-    <mergeCell ref="G139:I139"/>
-    <mergeCell ref="G140:I140"/>
-    <mergeCell ref="G141:I141"/>
-    <mergeCell ref="G142:I142"/>
-    <mergeCell ref="G143:I143"/>
-    <mergeCell ref="C136:E136"/>
-    <mergeCell ref="K133:M133"/>
-    <mergeCell ref="K143:M143"/>
-    <mergeCell ref="K135:M135"/>
-    <mergeCell ref="K136:M136"/>
-    <mergeCell ref="K137:M137"/>
-    <mergeCell ref="K138:M138"/>
-    <mergeCell ref="K139:M139"/>
-    <mergeCell ref="K117:M117"/>
-    <mergeCell ref="G117:I117"/>
-    <mergeCell ref="K122:M122"/>
-    <mergeCell ref="K123:M123"/>
-    <mergeCell ref="K124:M124"/>
-    <mergeCell ref="K125:M125"/>
-    <mergeCell ref="K126:M126"/>
-    <mergeCell ref="K127:M127"/>
-    <mergeCell ref="K128:M128"/>
-    <mergeCell ref="K129:M129"/>
-    <mergeCell ref="K132:M132"/>
-    <mergeCell ref="B117:E117"/>
-    <mergeCell ref="B131:E131"/>
-    <mergeCell ref="G131:I131"/>
-    <mergeCell ref="K131:M131"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="G89:I89"/>
-    <mergeCell ref="K89:M89"/>
-    <mergeCell ref="C90:E90"/>
-    <mergeCell ref="G90:I90"/>
-    <mergeCell ref="K90:M90"/>
-    <mergeCell ref="C91:E91"/>
-    <mergeCell ref="G91:I91"/>
-    <mergeCell ref="K91:M91"/>
-    <mergeCell ref="C92:E92"/>
-    <mergeCell ref="G92:I92"/>
-    <mergeCell ref="K92:M92"/>
-    <mergeCell ref="C93:E93"/>
-    <mergeCell ref="G93:I93"/>
-    <mergeCell ref="K93:M93"/>
-    <mergeCell ref="C94:E94"/>
-    <mergeCell ref="G94:I94"/>
-    <mergeCell ref="K94:M94"/>
-    <mergeCell ref="C95:E95"/>
-    <mergeCell ref="C127:E127"/>
-    <mergeCell ref="G95:I95"/>
-    <mergeCell ref="K95:M95"/>
-    <mergeCell ref="C96:E96"/>
-    <mergeCell ref="G96:I96"/>
-    <mergeCell ref="K96:M96"/>
-    <mergeCell ref="C97:E97"/>
-    <mergeCell ref="G97:I97"/>
-    <mergeCell ref="K97:M97"/>
-    <mergeCell ref="C98:E98"/>
-    <mergeCell ref="G98:I98"/>
-    <mergeCell ref="K98:M98"/>
-    <mergeCell ref="C99:E99"/>
-    <mergeCell ref="G99:I99"/>
-    <mergeCell ref="K99:M99"/>
-    <mergeCell ref="C100:E100"/>
-    <mergeCell ref="G100:I100"/>
-    <mergeCell ref="K100:M100"/>
-    <mergeCell ref="C101:E101"/>
-    <mergeCell ref="G101:I101"/>
-    <mergeCell ref="K101:M101"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="G103:I103"/>
-    <mergeCell ref="K103:M103"/>
-    <mergeCell ref="C104:E104"/>
-    <mergeCell ref="G104:I104"/>
-    <mergeCell ref="K104:M104"/>
-    <mergeCell ref="C105:E105"/>
-    <mergeCell ref="G105:I105"/>
-    <mergeCell ref="K105:M105"/>
-    <mergeCell ref="C106:E106"/>
-    <mergeCell ref="G106:I106"/>
-    <mergeCell ref="K106:M106"/>
-    <mergeCell ref="C107:E107"/>
-    <mergeCell ref="G107:I107"/>
-    <mergeCell ref="K107:M107"/>
-    <mergeCell ref="C108:E108"/>
-    <mergeCell ref="G108:I108"/>
-    <mergeCell ref="K108:M108"/>
-    <mergeCell ref="C109:E109"/>
-    <mergeCell ref="G109:I109"/>
-    <mergeCell ref="K109:M109"/>
-    <mergeCell ref="C110:E110"/>
-    <mergeCell ref="G110:I110"/>
-    <mergeCell ref="K110:M110"/>
-    <mergeCell ref="C111:E111"/>
-    <mergeCell ref="G111:I111"/>
-    <mergeCell ref="K111:M111"/>
-    <mergeCell ref="C112:E112"/>
-    <mergeCell ref="G112:I112"/>
-    <mergeCell ref="K112:M112"/>
-    <mergeCell ref="C113:E113"/>
-    <mergeCell ref="G113:I113"/>
-    <mergeCell ref="K113:M113"/>
-    <mergeCell ref="C114:E114"/>
-    <mergeCell ref="G114:I114"/>
-    <mergeCell ref="K114:M114"/>
-    <mergeCell ref="C115:E115"/>
-    <mergeCell ref="G115:I115"/>
-    <mergeCell ref="K115:M115"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="G61:I61"/>
-    <mergeCell ref="K61:M61"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="G62:I62"/>
-    <mergeCell ref="K62:M62"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="G63:I63"/>
-    <mergeCell ref="K63:M63"/>
-    <mergeCell ref="C64:E64"/>
-    <mergeCell ref="G64:I64"/>
-    <mergeCell ref="K64:M64"/>
-    <mergeCell ref="C65:E65"/>
-    <mergeCell ref="G65:I65"/>
-    <mergeCell ref="K65:M65"/>
-    <mergeCell ref="C66:E66"/>
-    <mergeCell ref="G66:I66"/>
-    <mergeCell ref="K66:M66"/>
-    <mergeCell ref="C67:E67"/>
-    <mergeCell ref="G67:I67"/>
-    <mergeCell ref="K67:M67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="G68:I68"/>
-    <mergeCell ref="K68:M68"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="G69:I69"/>
-    <mergeCell ref="K69:M69"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="G70:I70"/>
-    <mergeCell ref="K70:M70"/>
-    <mergeCell ref="C71:E71"/>
-    <mergeCell ref="G71:I71"/>
-    <mergeCell ref="K71:M71"/>
-    <mergeCell ref="C72:E72"/>
-    <mergeCell ref="G72:I72"/>
-    <mergeCell ref="K72:M72"/>
-    <mergeCell ref="C73:E73"/>
-    <mergeCell ref="G73:I73"/>
-    <mergeCell ref="K73:M73"/>
-    <mergeCell ref="B75:E75"/>
-    <mergeCell ref="G75:I75"/>
-    <mergeCell ref="K75:M75"/>
-    <mergeCell ref="C76:E76"/>
-    <mergeCell ref="G76:I76"/>
-    <mergeCell ref="K76:M76"/>
-    <mergeCell ref="C77:E77"/>
-    <mergeCell ref="G77:I77"/>
-    <mergeCell ref="K77:M77"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="G78:I78"/>
-    <mergeCell ref="K78:M78"/>
-    <mergeCell ref="C79:E79"/>
-    <mergeCell ref="G79:I79"/>
-    <mergeCell ref="K79:M79"/>
-    <mergeCell ref="C80:E80"/>
-    <mergeCell ref="G80:I80"/>
-    <mergeCell ref="K80:M80"/>
-    <mergeCell ref="C81:E81"/>
-    <mergeCell ref="G81:I81"/>
-    <mergeCell ref="K81:M81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="G82:I82"/>
-    <mergeCell ref="K82:M82"/>
-    <mergeCell ref="C83:E83"/>
-    <mergeCell ref="G83:I83"/>
-    <mergeCell ref="K83:M83"/>
-    <mergeCell ref="C84:E84"/>
-    <mergeCell ref="G84:I84"/>
-    <mergeCell ref="K84:M84"/>
-    <mergeCell ref="C85:E85"/>
-    <mergeCell ref="G85:I85"/>
-    <mergeCell ref="K85:M85"/>
-    <mergeCell ref="C86:E86"/>
-    <mergeCell ref="G86:I86"/>
-    <mergeCell ref="K86:M86"/>
-    <mergeCell ref="C87:E87"/>
-    <mergeCell ref="G87:I87"/>
-    <mergeCell ref="K87:M87"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="K33:M33"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="K34:M34"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="K35:M35"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="G36:I36"/>
-    <mergeCell ref="K36:M36"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="G37:I37"/>
-    <mergeCell ref="K37:M37"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="G38:I38"/>
-    <mergeCell ref="K38:M38"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="G39:I39"/>
-    <mergeCell ref="K39:M39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="G40:I40"/>
-    <mergeCell ref="K40:M40"/>
-    <mergeCell ref="C41:E41"/>
-    <mergeCell ref="G41:I41"/>
-    <mergeCell ref="K41:M41"/>
-    <mergeCell ref="C42:E42"/>
-    <mergeCell ref="G42:I42"/>
-    <mergeCell ref="K42:M42"/>
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="G43:I43"/>
-    <mergeCell ref="K43:M43"/>
-    <mergeCell ref="C44:E44"/>
-    <mergeCell ref="G44:I44"/>
-    <mergeCell ref="K44:M44"/>
-    <mergeCell ref="C45:E45"/>
-    <mergeCell ref="G45:I45"/>
-    <mergeCell ref="K45:M45"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="G47:I47"/>
-    <mergeCell ref="K47:M47"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="G48:I48"/>
-    <mergeCell ref="K48:M48"/>
-    <mergeCell ref="C49:E49"/>
-    <mergeCell ref="G49:I49"/>
-    <mergeCell ref="K49:M49"/>
-    <mergeCell ref="C50:E50"/>
-    <mergeCell ref="G50:I50"/>
-    <mergeCell ref="K50:M50"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="G51:I51"/>
-    <mergeCell ref="K51:M51"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="G52:I52"/>
-    <mergeCell ref="K52:M52"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="G53:I53"/>
-    <mergeCell ref="K53:M53"/>
-    <mergeCell ref="C54:E54"/>
-    <mergeCell ref="G54:I54"/>
-    <mergeCell ref="K54:M54"/>
-    <mergeCell ref="C55:E55"/>
-    <mergeCell ref="G55:I55"/>
-    <mergeCell ref="K55:M55"/>
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="G59:I59"/>
-    <mergeCell ref="K59:M59"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="G56:I56"/>
-    <mergeCell ref="K56:M56"/>
-    <mergeCell ref="C57:E57"/>
-    <mergeCell ref="G57:I57"/>
-    <mergeCell ref="K57:M57"/>
-    <mergeCell ref="C58:E58"/>
-    <mergeCell ref="G58:I58"/>
-    <mergeCell ref="K58:M58"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
FIX: Converted truth cooparisons to robust normalisation and removed disparity/confidence guess. Decreased sizes to crop original by 5 pixels all around.
</commit_message>
<xml_diff>
--- a/FPGA_Performance_Comparison_RGB.xlsx
+++ b/FPGA_Performance_Comparison_RGB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/DanielBiswas/Desktop/Documents/University/Year 5/Semester 1/AMME4112/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C66D13FC-801E-7943-A9A3-DB3D576B41D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4C74CC7-1F88-564D-B9C2-80C8011B9B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="24660" windowHeight="26820" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="77">
   <si>
     <t>FPGA Implementation</t>
   </si>
@@ -200,9 +200,6 @@
     <t>Disparity Exact Match Fraction</t>
   </si>
   <si>
-    <t>inf</t>
-  </si>
-  <si>
     <t>Change From Standard</t>
   </si>
   <si>
@@ -266,10 +263,10 @@
     <t>Average</t>
   </si>
   <si>
-    <t>Confidence Exact Match Pixels (Out Of 3136)</t>
-  </si>
-  <si>
-    <t>Disparity Exact Match Pixels (Out Of 3136)</t>
+    <t>Confidence Exact Match Pixels (Out Of 2916)</t>
+  </si>
+  <si>
+    <t>Disparity Exact Match Pixels (Out Of 2916)</t>
   </si>
 </sst>
 </file>
@@ -365,17 +362,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -722,31 +719,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
+      <c r="B1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
       <c r="F1" s="6"/>
       <c r="G1" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H1" s="11"/>
       <c r="I1" s="11"/>
       <c r="J1" s="6"/>
       <c r="K1" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L1" s="11"/>
       <c r="M1" s="11"/>
       <c r="N1" s="6"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A2" s="12"/>
+      <c r="A2" s="14"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -754,7 +751,7 @@
         <v>2</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>3</v>
@@ -764,7 +761,7 @@
         <v>2</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>3</v>
@@ -774,7 +771,7 @@
         <v>2</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>3</v>
@@ -2019,23 +2016,23 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C33" s="11"/>
       <c r="D33" s="11"/>
       <c r="E33" s="11"/>
       <c r="F33" s="6"/>
       <c r="G33" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H33" s="11"/>
       <c r="I33" s="11"/>
       <c r="J33" s="6"/>
       <c r="K33" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L33" s="11"/>
       <c r="M33" s="11"/>
@@ -2046,24 +2043,24 @@
         <v>32</v>
       </c>
       <c r="B34" s="1">
-        <v>36.935268000000001</v>
+        <v>36.202331999999998</v>
       </c>
       <c r="C34" s="11">
-        <v>35.655293</v>
+        <v>34.931412999999999</v>
       </c>
       <c r="D34" s="11"/>
       <c r="E34" s="11"/>
       <c r="F34" s="6"/>
       <c r="G34" s="11">
         <f t="shared" ref="G34:G45" si="7">C34-B34</f>
-        <v>-1.2799750000000003</v>
+        <v>-1.2709189999999992</v>
       </c>
       <c r="H34" s="11"/>
       <c r="I34" s="11"/>
       <c r="J34" s="6"/>
       <c r="K34" s="10">
         <f>G34/B34</f>
-        <v>-3.4654547518106552E-2</v>
+        <v>-3.5105998143986947E-2</v>
       </c>
       <c r="L34" s="10"/>
       <c r="M34" s="10"/>
@@ -2074,24 +2071,24 @@
         <v>33</v>
       </c>
       <c r="B35" s="1">
-        <v>4.1183040000000002</v>
+        <v>4.056241</v>
       </c>
       <c r="C35" s="11">
-        <v>4.0647320000000002</v>
+        <v>4.0034289999999997</v>
       </c>
       <c r="D35" s="11"/>
       <c r="E35" s="11"/>
       <c r="F35" s="6"/>
       <c r="G35" s="11">
         <f t="shared" si="7"/>
-        <v>-5.3571999999999953E-2</v>
+        <v>-5.2812000000000303E-2</v>
       </c>
       <c r="H35" s="11"/>
       <c r="I35" s="11"/>
       <c r="J35" s="6"/>
       <c r="K35" s="10">
         <f>G35/B35</f>
-        <v>-1.300826748098245E-2</v>
+        <v>-1.3019936438688012E-2</v>
       </c>
       <c r="L35" s="10"/>
       <c r="M35" s="10"/>
@@ -2173,8 +2170,8 @@
       <c r="H38" s="11"/>
       <c r="I38" s="11"/>
       <c r="J38" s="6"/>
-      <c r="K38" s="10" t="s">
-        <v>54</v>
+      <c r="K38" s="10">
+        <v>0</v>
       </c>
       <c r="L38" s="10"/>
       <c r="M38" s="10"/>
@@ -2213,24 +2210,24 @@
         <v>38</v>
       </c>
       <c r="B40" s="1">
-        <v>6.6195789999999999</v>
+        <v>6.6286009999999997</v>
       </c>
       <c r="C40" s="11">
-        <v>6.6183040000000002</v>
+        <v>6.6279149999999998</v>
       </c>
       <c r="D40" s="11"/>
       <c r="E40" s="11"/>
       <c r="F40" s="6"/>
       <c r="G40" s="11">
         <f t="shared" si="7"/>
-        <v>-1.274999999999693E-3</v>
+        <v>-6.8599999999996442E-4</v>
       </c>
       <c r="H40" s="11"/>
       <c r="I40" s="11"/>
       <c r="J40" s="6"/>
       <c r="K40" s="10">
         <f t="shared" si="8"/>
-        <v>-1.9261043640383973E-4</v>
+        <v>-1.0349091761594406E-4</v>
       </c>
       <c r="L40" s="10"/>
       <c r="M40" s="10"/>
@@ -2322,13 +2319,13 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B44" s="1">
-        <v>471</v>
+        <v>453</v>
       </c>
       <c r="C44" s="11">
-        <v>455</v>
+        <v>437</v>
       </c>
       <c r="D44" s="11"/>
       <c r="E44" s="11"/>
@@ -2342,7 +2339,7 @@
       <c r="J44" s="6"/>
       <c r="K44" s="10">
         <f t="shared" si="8"/>
-        <v>-3.3970276008492568E-2</v>
+        <v>-3.5320088300220751E-2</v>
       </c>
       <c r="L44" s="10"/>
       <c r="M44" s="10"/>
@@ -2353,24 +2350,24 @@
         <v>42</v>
       </c>
       <c r="B45" s="5">
-        <v>0.15019133000000001</v>
-      </c>
-      <c r="C45" s="15">
-        <v>0.14508929000000001</v>
-      </c>
-      <c r="D45" s="15"/>
-      <c r="E45" s="15"/>
+        <v>0.15534978999999999</v>
+      </c>
+      <c r="C45" s="12">
+        <v>0.14986283</v>
+      </c>
+      <c r="D45" s="12"/>
+      <c r="E45" s="12"/>
       <c r="F45" s="6"/>
       <c r="G45" s="11">
         <f t="shared" si="7"/>
-        <v>-5.1020400000000021E-3</v>
+        <v>-5.4869599999999852E-3</v>
       </c>
       <c r="H45" s="11"/>
       <c r="I45" s="11"/>
       <c r="J45" s="6"/>
       <c r="K45" s="10">
         <f t="shared" si="8"/>
-        <v>-3.3970269788542402E-2</v>
+        <v>-3.532003487098364E-2</v>
       </c>
       <c r="L45" s="10"/>
       <c r="M45" s="10"/>
@@ -2394,23 +2391,23 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C47" s="11"/>
       <c r="D47" s="11"/>
       <c r="E47" s="11"/>
       <c r="F47" s="6"/>
       <c r="G47" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H47" s="11"/>
       <c r="I47" s="11"/>
       <c r="J47" s="6"/>
       <c r="K47" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L47" s="11"/>
       <c r="M47" s="11"/>
@@ -2421,24 +2418,24 @@
         <v>43</v>
       </c>
       <c r="B48" s="1">
-        <v>3.3816959999999998</v>
+        <v>3.3545950000000002</v>
       </c>
       <c r="C48" s="11">
-        <v>3.3852039999999999</v>
+        <v>3.358368</v>
       </c>
       <c r="D48" s="11"/>
       <c r="E48" s="11"/>
       <c r="F48" s="6"/>
       <c r="G48" s="11">
         <f t="shared" ref="G48:G59" si="9">C48-B48</f>
-        <v>3.5080000000000666E-3</v>
+        <v>3.7729999999998043E-3</v>
       </c>
       <c r="H48" s="11"/>
       <c r="I48" s="11"/>
       <c r="J48" s="6"/>
       <c r="K48" s="10">
         <f t="shared" ref="K48:K59" si="10">G48/B48</f>
-        <v>1.0373493063835623E-3</v>
+        <v>1.1247259356195916E-3</v>
       </c>
       <c r="L48" s="10"/>
       <c r="M48" s="10"/>
@@ -2449,24 +2446,24 @@
         <v>44</v>
       </c>
       <c r="B49" s="1">
-        <v>1.7662629999999999</v>
+        <v>1.7592589999999999</v>
       </c>
       <c r="C49" s="11">
-        <v>1.767857</v>
+        <v>1.760974</v>
       </c>
       <c r="D49" s="11"/>
       <c r="E49" s="11"/>
       <c r="F49" s="6"/>
       <c r="G49" s="11">
         <f t="shared" si="9"/>
-        <v>1.5940000000000953E-3</v>
+        <v>1.7150000000001331E-3</v>
       </c>
       <c r="H49" s="11"/>
       <c r="I49" s="11"/>
       <c r="J49" s="6"/>
       <c r="K49" s="10">
         <f t="shared" si="10"/>
-        <v>9.0247035690613198E-4</v>
+        <v>9.7484224892419665E-4</v>
       </c>
       <c r="L49" s="10"/>
       <c r="M49" s="10"/>
@@ -2589,24 +2586,24 @@
         <v>49</v>
       </c>
       <c r="B54" s="1">
-        <v>6.7936860000000001</v>
+        <v>6.7962959999999999</v>
       </c>
       <c r="C54" s="11">
-        <v>6.7933669999999999</v>
+        <v>6.7959529999999999</v>
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="11"/>
       <c r="F54" s="6"/>
       <c r="G54" s="11">
         <f t="shared" si="9"/>
-        <v>-3.1900000000018025E-4</v>
+        <v>-3.4299999999998221E-4</v>
       </c>
       <c r="H54" s="11"/>
       <c r="I54" s="11"/>
       <c r="J54" s="6"/>
       <c r="K54" s="10">
         <f t="shared" si="10"/>
-        <v>-4.6955364142555343E-5</v>
+        <v>-5.0468667050402489E-5</v>
       </c>
       <c r="L54" s="10"/>
       <c r="M54" s="10"/>
@@ -2698,13 +2695,13 @@
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B58" s="1">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C58" s="11">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D58" s="11"/>
       <c r="E58" s="11"/>
@@ -2718,7 +2715,7 @@
       <c r="J58" s="6"/>
       <c r="K58" s="10">
         <f t="shared" si="10"/>
-        <v>-1.6393442622950821E-2</v>
+        <v>-1.7857142857142856E-2</v>
       </c>
       <c r="L58" s="10"/>
       <c r="M58" s="10"/>
@@ -2729,24 +2726,24 @@
         <v>53</v>
       </c>
       <c r="B59" s="5">
-        <v>1.9451530000000002E-2</v>
+        <v>1.9204389999999998E-2</v>
       </c>
       <c r="C59" s="10">
-        <v>1.9132650000000001E-2</v>
+        <v>1.8861449999999998E-2</v>
       </c>
       <c r="D59" s="10"/>
       <c r="E59" s="10"/>
       <c r="F59" s="6"/>
       <c r="G59" s="11">
         <f t="shared" si="9"/>
-        <v>-3.1888000000000055E-4</v>
+        <v>-3.4293999999999991E-4</v>
       </c>
       <c r="H59" s="11"/>
       <c r="I59" s="11"/>
       <c r="J59" s="6"/>
       <c r="K59" s="10">
         <f t="shared" si="10"/>
-        <v>-1.6393569040584494E-2</v>
+        <v>-1.7857375318872399E-2</v>
       </c>
       <c r="L59" s="10"/>
       <c r="M59" s="10"/>
@@ -2770,23 +2767,23 @@
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B61" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C61" s="11"/>
       <c r="D61" s="11"/>
       <c r="E61" s="11"/>
       <c r="F61" s="6"/>
       <c r="G61" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H61" s="11"/>
       <c r="I61" s="11"/>
       <c r="J61" s="6"/>
       <c r="K61" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L61" s="11"/>
       <c r="M61" s="11"/>
@@ -2797,24 +2794,24 @@
         <v>32</v>
       </c>
       <c r="B62" s="1">
-        <v>128.02455399999999</v>
+        <v>128.81378599999999</v>
       </c>
       <c r="C62" s="11">
-        <v>124.003508</v>
+        <v>124.748285</v>
       </c>
       <c r="D62" s="11"/>
       <c r="E62" s="11"/>
       <c r="F62" s="6"/>
       <c r="G62" s="11">
         <f t="shared" ref="G62:G73" si="11">C62-B62</f>
-        <v>-4.0210459999999983</v>
+        <v>-4.0655009999999976</v>
       </c>
       <c r="H62" s="11"/>
       <c r="I62" s="11"/>
       <c r="J62" s="6"/>
       <c r="K62" s="10">
         <f>G62/B62</f>
-        <v>-3.140839686112086E-2</v>
+        <v>-3.1561070645031719E-2</v>
       </c>
       <c r="L62" s="10"/>
       <c r="M62" s="10"/>
@@ -2825,24 +2822,24 @@
         <v>33</v>
       </c>
       <c r="B63" s="1">
-        <v>9.3899869999999996</v>
+        <v>9.4557610000000007</v>
       </c>
       <c r="C63" s="11">
-        <v>9.2522319999999993</v>
+        <v>9.316872</v>
       </c>
       <c r="D63" s="11"/>
       <c r="E63" s="11"/>
       <c r="F63" s="6"/>
       <c r="G63" s="11">
         <f t="shared" si="11"/>
-        <v>-0.13775500000000029</v>
+        <v>-0.13888900000000071</v>
       </c>
       <c r="H63" s="11"/>
       <c r="I63" s="11"/>
       <c r="J63" s="6"/>
       <c r="K63" s="10">
         <f>G63/B63</f>
-        <v>-1.4670414346686561E-2</v>
+        <v>-1.4688294257860441E-2</v>
       </c>
       <c r="L63" s="10"/>
       <c r="M63" s="10"/>
@@ -2924,8 +2921,8 @@
       <c r="H66" s="11"/>
       <c r="I66" s="11"/>
       <c r="J66" s="6"/>
-      <c r="K66" s="10" t="s">
-        <v>54</v>
+      <c r="K66" s="10">
+        <v>0</v>
       </c>
       <c r="L66" s="10"/>
       <c r="M66" s="10"/>
@@ -2964,24 +2961,24 @@
         <v>38</v>
       </c>
       <c r="B68" s="1">
-        <v>5.8580990000000002</v>
+        <v>5.8508230000000001</v>
       </c>
       <c r="C68" s="11">
-        <v>5.8427930000000003</v>
+        <v>5.8347049999999996</v>
       </c>
       <c r="D68" s="11"/>
       <c r="E68" s="11"/>
       <c r="F68" s="6"/>
       <c r="G68" s="11">
         <f t="shared" si="11"/>
-        <v>-1.530599999999982E-2</v>
+        <v>-1.6118000000000521E-2</v>
       </c>
       <c r="H68" s="11"/>
       <c r="I68" s="11"/>
       <c r="J68" s="6"/>
       <c r="K68" s="10">
         <f t="shared" si="12"/>
-        <v>-2.6127929896711919E-3</v>
+        <v>-2.7548261159157472E-3</v>
       </c>
       <c r="L68" s="10"/>
       <c r="M68" s="10"/>
@@ -3073,13 +3070,13 @@
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A72" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B72" s="1">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="C72" s="11">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D72" s="11"/>
       <c r="E72" s="11"/>
@@ -3104,13 +3101,13 @@
         <v>42</v>
       </c>
       <c r="B73" s="5">
-        <v>7.33418E-3</v>
-      </c>
-      <c r="C73" s="15">
-        <v>7.33418E-3</v>
-      </c>
-      <c r="D73" s="15"/>
-      <c r="E73" s="15"/>
+        <v>5.14403E-3</v>
+      </c>
+      <c r="C73" s="12">
+        <v>5.14403E-3</v>
+      </c>
+      <c r="D73" s="12"/>
+      <c r="E73" s="12"/>
       <c r="F73" s="6"/>
       <c r="G73" s="11">
         <f t="shared" si="11"/>
@@ -3145,23 +3142,23 @@
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A75" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B75" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C75" s="11"/>
       <c r="D75" s="11"/>
       <c r="E75" s="11"/>
       <c r="F75" s="6"/>
       <c r="G75" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H75" s="11"/>
       <c r="I75" s="11"/>
       <c r="J75" s="6"/>
       <c r="K75" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L75" s="11"/>
       <c r="M75" s="11"/>
@@ -3350,7 +3347,7 @@
       <c r="I82" s="11"/>
       <c r="J82" s="6"/>
       <c r="K82" s="10">
-        <f t="shared" ref="K76:K87" si="14">G82/B82</f>
+        <f t="shared" ref="K82:K87" si="14">G82/B82</f>
         <v>0</v>
       </c>
       <c r="L82" s="10"/>
@@ -3443,13 +3440,13 @@
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B86" s="1">
-        <v>3136</v>
+        <v>2916</v>
       </c>
       <c r="C86" s="11">
-        <v>3136</v>
+        <v>2916</v>
       </c>
       <c r="D86" s="11"/>
       <c r="E86" s="11"/>
@@ -3515,23 +3512,23 @@
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B89" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C89" s="11"/>
       <c r="D89" s="11"/>
       <c r="E89" s="11"/>
       <c r="F89" s="6"/>
       <c r="G89" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H89" s="11"/>
       <c r="I89" s="11"/>
       <c r="J89" s="6"/>
       <c r="K89" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L89" s="11"/>
       <c r="M89" s="11"/>
@@ -3542,24 +3539,24 @@
         <v>32</v>
       </c>
       <c r="B90" s="1">
-        <v>8.9113520000000008</v>
+        <v>8.8847740000000002</v>
       </c>
       <c r="C90" s="11">
-        <v>8.6871810000000007</v>
+        <v>8.6663239999999995</v>
       </c>
       <c r="D90" s="11"/>
       <c r="E90" s="11"/>
       <c r="F90" s="6"/>
       <c r="G90" s="11">
         <f t="shared" ref="G90:G101" si="15">C90-B90</f>
-        <v>-0.22417100000000012</v>
+        <v>-0.2184500000000007</v>
       </c>
       <c r="H90" s="11"/>
       <c r="I90" s="11"/>
       <c r="J90" s="6"/>
       <c r="K90" s="10">
         <f>G90/B90</f>
-        <v>-2.5155666614897505E-2</v>
+        <v>-2.4587006940187863E-2</v>
       </c>
       <c r="L90" s="10"/>
       <c r="M90" s="10"/>
@@ -3570,24 +3567,24 @@
         <v>33</v>
       </c>
       <c r="B91" s="1">
-        <v>2.2079080000000002</v>
+        <v>2.2085050000000002</v>
       </c>
       <c r="C91" s="11">
-        <v>2.1980230000000001</v>
+        <v>2.199246</v>
       </c>
       <c r="D91" s="11"/>
       <c r="E91" s="11"/>
       <c r="F91" s="6"/>
       <c r="G91" s="11">
         <f t="shared" si="15"/>
-        <v>-9.8850000000001437E-3</v>
+        <v>-9.2590000000001282E-3</v>
       </c>
       <c r="H91" s="11"/>
       <c r="I91" s="11"/>
       <c r="J91" s="6"/>
       <c r="K91" s="10">
         <f>G91/B91</f>
-        <v>-4.4770887192764116E-3</v>
+        <v>-4.1924288149676487E-3</v>
       </c>
       <c r="L91" s="10"/>
       <c r="M91" s="10"/>
@@ -3669,8 +3666,8 @@
       <c r="H94" s="11"/>
       <c r="I94" s="11"/>
       <c r="J94" s="6"/>
-      <c r="K94" s="10" t="s">
-        <v>54</v>
+      <c r="K94" s="10">
+        <v>0</v>
       </c>
       <c r="L94" s="10"/>
       <c r="M94" s="10"/>
@@ -3709,24 +3706,24 @@
         <v>38</v>
       </c>
       <c r="B96" s="1">
-        <v>6.8000639999999999</v>
+        <v>6.7962959999999999</v>
       </c>
       <c r="C96" s="11">
-        <v>6.7997449999999997</v>
+        <v>6.7956099999999999</v>
       </c>
       <c r="D96" s="11"/>
       <c r="E96" s="11"/>
       <c r="F96" s="6"/>
       <c r="G96" s="11">
         <f t="shared" si="15"/>
-        <v>-3.1900000000018025E-4</v>
+        <v>-6.8599999999996442E-4</v>
       </c>
       <c r="H96" s="11"/>
       <c r="I96" s="11"/>
       <c r="J96" s="6"/>
       <c r="K96" s="10">
         <f t="shared" si="16"/>
-        <v>-4.6911323187572975E-5</v>
+        <v>-1.0093733410080498E-4</v>
       </c>
       <c r="L96" s="10"/>
       <c r="M96" s="10"/>
@@ -3818,27 +3815,27 @@
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A100" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B100" s="1">
-        <v>211</v>
+        <v>177</v>
       </c>
       <c r="C100" s="11">
-        <v>194</v>
+        <v>161</v>
       </c>
       <c r="D100" s="11"/>
       <c r="E100" s="11"/>
       <c r="F100" s="6"/>
       <c r="G100" s="11">
         <f t="shared" si="15"/>
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="H100" s="11"/>
       <c r="I100" s="11"/>
       <c r="J100" s="6"/>
       <c r="K100" s="10">
         <f t="shared" si="16"/>
-        <v>-8.0568720379146919E-2</v>
+        <v>-9.03954802259887E-2</v>
       </c>
       <c r="L100" s="10"/>
       <c r="M100" s="10"/>
@@ -3849,24 +3846,24 @@
         <v>42</v>
       </c>
       <c r="B101" s="5">
-        <v>6.7283159999999995E-2</v>
-      </c>
-      <c r="C101" s="15">
-        <v>6.1862239999999999E-2</v>
-      </c>
-      <c r="D101" s="15"/>
-      <c r="E101" s="15"/>
+        <v>6.0699589999999998E-2</v>
+      </c>
+      <c r="C101" s="12">
+        <v>5.5212619999999997E-2</v>
+      </c>
+      <c r="D101" s="12"/>
+      <c r="E101" s="12"/>
       <c r="F101" s="6"/>
       <c r="G101" s="11">
         <f t="shared" si="15"/>
-        <v>-5.4209199999999957E-3</v>
+        <v>-5.4869700000000007E-3</v>
       </c>
       <c r="H101" s="11"/>
       <c r="I101" s="11"/>
       <c r="J101" s="6"/>
       <c r="K101" s="10">
         <f t="shared" si="16"/>
-        <v>-8.0568748554615988E-2</v>
+        <v>-9.0395503495163662E-2</v>
       </c>
       <c r="L101" s="10"/>
       <c r="M101" s="10"/>
@@ -3890,23 +3887,23 @@
     </row>
     <row r="103" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A103" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B103" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C103" s="11"/>
       <c r="D103" s="11"/>
       <c r="E103" s="11"/>
       <c r="F103" s="6"/>
       <c r="G103" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H103" s="11"/>
       <c r="I103" s="11"/>
       <c r="J103" s="6"/>
       <c r="K103" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L103" s="11"/>
       <c r="M103" s="11"/>
@@ -3917,10 +3914,10 @@
         <v>43</v>
       </c>
       <c r="B104" s="1">
-        <v>9.8849999999999997E-3</v>
+        <v>8.5730000000000008E-3</v>
       </c>
       <c r="C104" s="11">
-        <v>9.8849999999999997E-3</v>
+        <v>8.5730000000000008E-3</v>
       </c>
       <c r="D104" s="11"/>
       <c r="E104" s="11"/>
@@ -3945,10 +3942,10 @@
         <v>44</v>
       </c>
       <c r="B105" s="1">
-        <v>9.8849999999999997E-3</v>
+        <v>8.5730000000000008E-3</v>
       </c>
       <c r="C105" s="11">
-        <v>9.8849999999999997E-3</v>
+        <v>8.5730000000000008E-3</v>
       </c>
       <c r="D105" s="11"/>
       <c r="E105" s="11"/>
@@ -4082,10 +4079,10 @@
         <v>49</v>
       </c>
       <c r="B110" s="1">
-        <v>7.9901150000000003</v>
+        <v>7.9914269999999998</v>
       </c>
       <c r="C110" s="11">
-        <v>7.9901150000000003</v>
+        <v>7.9914269999999998</v>
       </c>
       <c r="D110" s="11"/>
       <c r="E110" s="11"/>
@@ -4191,13 +4188,13 @@
     </row>
     <row r="114" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A114" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B114" s="1">
-        <v>3105</v>
+        <v>2891</v>
       </c>
       <c r="C114" s="11">
-        <v>3105</v>
+        <v>2891</v>
       </c>
       <c r="D114" s="11"/>
       <c r="E114" s="11"/>
@@ -4222,10 +4219,10 @@
         <v>53</v>
       </c>
       <c r="B115" s="5">
-        <v>0.99011479999999996</v>
+        <v>0.99142660999999999</v>
       </c>
       <c r="C115" s="10">
-        <v>0.99011479999999996</v>
+        <v>0.99142660999999999</v>
       </c>
       <c r="D115" s="10"/>
       <c r="E115" s="10"/>
@@ -4263,23 +4260,23 @@
     </row>
     <row r="117" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A117" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B117" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C117" s="11"/>
       <c r="D117" s="11"/>
       <c r="E117" s="11"/>
       <c r="F117" s="6"/>
       <c r="G117" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H117" s="11"/>
       <c r="I117" s="11"/>
       <c r="J117" s="6"/>
       <c r="K117" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L117" s="11"/>
       <c r="M117" s="11"/>
@@ -4291,25 +4288,25 @@
       </c>
       <c r="B118" s="1">
         <f>AVERAGE(B62,B34,B90)</f>
-        <v>57.957057999999996</v>
+        <v>57.966963999999997</v>
       </c>
       <c r="C118" s="11">
         <f>AVERAGE(C62,C34,C90)</f>
-        <v>56.115327333333333</v>
+        <v>56.115340666666668</v>
       </c>
       <c r="D118" s="11"/>
       <c r="E118" s="11"/>
       <c r="F118" s="6"/>
       <c r="G118" s="11">
         <f t="shared" ref="G118:G129" si="19">C118-B118</f>
-        <v>-1.8417306666666633</v>
+        <v>-1.851623333333329</v>
       </c>
       <c r="H118" s="11"/>
       <c r="I118" s="11"/>
       <c r="J118" s="6"/>
       <c r="K118" s="10">
         <f>G118/B118</f>
-        <v>-3.17775044182999E-2</v>
+        <v>-3.1942734370793147E-2</v>
       </c>
       <c r="L118" s="10"/>
       <c r="M118" s="10"/>
@@ -4321,25 +4318,25 @@
       </c>
       <c r="B119" s="1">
         <f t="shared" ref="B119:B128" si="20">AVERAGE(B63,B35,B91)</f>
-        <v>5.2387329999999999</v>
+        <v>5.2401690000000007</v>
       </c>
       <c r="C119" s="11">
         <f t="shared" ref="C119:C129" si="21">AVERAGE(C63,C35,C91)</f>
-        <v>5.1716623333333329</v>
+        <v>5.173182333333334</v>
       </c>
       <c r="D119" s="11"/>
       <c r="E119" s="11"/>
       <c r="F119" s="6"/>
       <c r="G119" s="11">
         <f t="shared" si="19"/>
-        <v>-6.7070666666666945E-2</v>
+        <v>-6.698666666666675E-2</v>
       </c>
       <c r="H119" s="11"/>
       <c r="I119" s="11"/>
       <c r="J119" s="6"/>
       <c r="K119" s="10">
         <f>G119/B119</f>
-        <v>-1.2802841195889722E-2</v>
+        <v>-1.2783302726814105E-2</v>
       </c>
       <c r="L119" s="10"/>
       <c r="M119" s="10"/>
@@ -4427,8 +4424,8 @@
       <c r="H122" s="11"/>
       <c r="I122" s="11"/>
       <c r="J122" s="6"/>
-      <c r="K122" s="10" t="s">
-        <v>54</v>
+      <c r="K122" s="10">
+        <v>0</v>
       </c>
       <c r="L122" s="10"/>
       <c r="M122" s="10"/>
@@ -4470,25 +4467,25 @@
       </c>
       <c r="B124" s="1">
         <f t="shared" si="20"/>
-        <v>6.4259139999999997</v>
+        <v>6.4252399999999996</v>
       </c>
       <c r="C124" s="11">
         <f t="shared" si="21"/>
-        <v>6.4202806666666667</v>
+        <v>6.4194099999999992</v>
       </c>
       <c r="D124" s="11"/>
       <c r="E124" s="11"/>
       <c r="F124" s="6"/>
       <c r="G124" s="11">
         <f t="shared" si="19"/>
-        <v>-5.633333333332935E-3</v>
+        <v>-5.8300000000004459E-3</v>
       </c>
       <c r="H124" s="11"/>
       <c r="I124" s="11"/>
       <c r="J124" s="6"/>
       <c r="K124" s="10">
         <f t="shared" si="22"/>
-        <v>-8.7665868751634951E-4</v>
+        <v>-9.0735910253942991E-4</v>
       </c>
       <c r="L124" s="10"/>
       <c r="M124" s="10"/>
@@ -4586,29 +4583,29 @@
     </row>
     <row r="128" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A128" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B128" s="1">
         <f t="shared" si="20"/>
-        <v>235</v>
+        <v>215</v>
       </c>
       <c r="C128" s="11">
         <f t="shared" si="21"/>
-        <v>224</v>
+        <v>204.33333333333334</v>
       </c>
       <c r="D128" s="11"/>
       <c r="E128" s="11"/>
       <c r="F128" s="6"/>
       <c r="G128" s="11">
         <f t="shared" si="19"/>
-        <v>-11</v>
+        <v>-10.666666666666657</v>
       </c>
       <c r="H128" s="11"/>
       <c r="I128" s="11"/>
       <c r="J128" s="6"/>
       <c r="K128" s="10">
         <f t="shared" si="22"/>
-        <v>-4.6808510638297871E-2</v>
+        <v>-4.9612403100775151E-2</v>
       </c>
       <c r="L128" s="10"/>
       <c r="M128" s="10"/>
@@ -4620,25 +4617,25 @@
       </c>
       <c r="B129" s="5">
         <f>AVERAGE(B73,B45,B101)</f>
-        <v>7.4936223333333329E-2</v>
-      </c>
-      <c r="C129" s="14">
+        <v>7.3731136666666655E-2</v>
+      </c>
+      <c r="C129" s="13">
         <f t="shared" si="21"/>
-        <v>7.1428570000000011E-2</v>
+        <v>7.0073159999999995E-2</v>
       </c>
       <c r="D129" s="11"/>
       <c r="E129" s="11"/>
       <c r="F129" s="6"/>
       <c r="G129" s="11">
         <f t="shared" si="19"/>
-        <v>-3.5076533333333187E-3</v>
+        <v>-3.6579766666666597E-3</v>
       </c>
       <c r="H129" s="11"/>
       <c r="I129" s="11"/>
       <c r="J129" s="6"/>
       <c r="K129" s="10">
         <f t="shared" si="22"/>
-        <v>-4.6808514991881572E-2</v>
+        <v>-4.9612373171515282E-2</v>
       </c>
       <c r="L129" s="10"/>
       <c r="M129" s="10"/>
@@ -4662,23 +4659,23 @@
     </row>
     <row r="131" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A131" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B131" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C131" s="11"/>
       <c r="D131" s="11"/>
       <c r="E131" s="11"/>
       <c r="F131" s="6"/>
       <c r="G131" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H131" s="11"/>
       <c r="I131" s="11"/>
       <c r="J131" s="6"/>
       <c r="K131" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L131" s="11"/>
       <c r="M131" s="11"/>
@@ -4690,25 +4687,25 @@
       </c>
       <c r="B132" s="1">
         <f>AVERAGE(B76,B48,B104)</f>
-        <v>1.1305270000000001</v>
+        <v>1.1210560000000001</v>
       </c>
       <c r="C132" s="11">
         <f>AVERAGE(C76,C48,C104)</f>
-        <v>1.1316963333333334</v>
+        <v>1.1223136666666667</v>
       </c>
       <c r="D132" s="11"/>
       <c r="E132" s="11"/>
       <c r="F132" s="6"/>
       <c r="G132" s="11">
         <f t="shared" ref="G132:G143" si="23">C132-B132</f>
-        <v>1.1693333333333555E-3</v>
+        <v>1.2576666666666014E-3</v>
       </c>
       <c r="H132" s="11"/>
       <c r="I132" s="11"/>
       <c r="J132" s="6"/>
       <c r="K132" s="10">
         <f t="shared" ref="K132:K143" si="24">G132/B132</f>
-        <v>1.0343258792875848E-3</v>
+        <v>1.1218589139762878E-3</v>
       </c>
       <c r="L132" s="10"/>
       <c r="M132" s="10"/>
@@ -4720,25 +4717,25 @@
       </c>
       <c r="B133" s="1">
         <f t="shared" ref="B133:B142" si="25">AVERAGE(B77,B49,B105)</f>
-        <v>0.59204933333333332</v>
+        <v>0.58927733333333332</v>
       </c>
       <c r="C133" s="11">
         <f t="shared" ref="C133:C143" si="26">AVERAGE(C77,C49,C105)</f>
-        <v>0.59258066666666664</v>
+        <v>0.58984899999999996</v>
       </c>
       <c r="D133" s="11"/>
       <c r="E133" s="11"/>
       <c r="F133" s="6"/>
       <c r="G133" s="11">
         <f t="shared" si="23"/>
-        <v>5.3133333333332811E-4</v>
+        <v>5.7166666666663701E-4</v>
       </c>
       <c r="H133" s="11"/>
       <c r="I133" s="11"/>
       <c r="J133" s="6"/>
       <c r="K133" s="10">
         <f t="shared" si="24"/>
-        <v>8.9744773521124616E-4</v>
+        <v>9.7011480728933011E-4</v>
       </c>
       <c r="L133" s="10"/>
       <c r="M133" s="10"/>
@@ -4870,25 +4867,25 @@
       </c>
       <c r="B138" s="1">
         <f t="shared" si="25"/>
-        <v>7.5946003333333332</v>
+        <v>7.5959076666666663</v>
       </c>
       <c r="C138" s="11">
         <f t="shared" si="26"/>
-        <v>7.5944940000000001</v>
+        <v>7.595793333333333</v>
       </c>
       <c r="D138" s="11"/>
       <c r="E138" s="11"/>
       <c r="F138" s="6"/>
       <c r="G138" s="11">
         <f t="shared" si="23"/>
-        <v>-1.0633333333309736E-4</v>
+        <v>-1.143333333333274E-4</v>
       </c>
       <c r="H138" s="11"/>
       <c r="I138" s="11"/>
       <c r="J138" s="6"/>
       <c r="K138" s="10">
         <f t="shared" si="24"/>
-        <v>-1.4001175659816029E-5</v>
+        <v>-1.5051964603922131E-5</v>
       </c>
       <c r="L138" s="10"/>
       <c r="M138" s="10"/>
@@ -4986,29 +4983,29 @@
     </row>
     <row r="142" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A142" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B142" s="1">
         <f t="shared" si="25"/>
-        <v>2100.6666666666665</v>
+        <v>1954.3333333333333</v>
       </c>
       <c r="C142" s="11">
         <f>AVERAGE(C86,C58,C114)</f>
-        <v>2100.3333333333335</v>
+        <v>1954</v>
       </c>
       <c r="D142" s="11"/>
       <c r="E142" s="11"/>
       <c r="F142" s="6"/>
       <c r="G142" s="11">
         <f t="shared" si="23"/>
-        <v>-0.33333333333303017</v>
+        <v>-0.33333333333325754</v>
       </c>
       <c r="H142" s="11"/>
       <c r="I142" s="11"/>
       <c r="J142" s="6"/>
       <c r="K142" s="10">
         <f t="shared" si="24"/>
-        <v>-1.5867978419534918E-4</v>
+        <v>-1.7056114617086348E-4</v>
       </c>
       <c r="L142" s="10"/>
       <c r="M142" s="10"/>
@@ -5020,25 +5017,25 @@
       </c>
       <c r="B143" s="5">
         <f>AVERAGE(B87,B59,B115)</f>
-        <v>0.66985544333333336</v>
-      </c>
-      <c r="C143" s="14">
+        <v>0.67021033333333335</v>
+      </c>
+      <c r="C143" s="13">
         <f t="shared" si="26"/>
-        <v>0.66974915000000002</v>
+        <v>0.6700960199999999</v>
       </c>
       <c r="D143" s="11"/>
       <c r="E143" s="11"/>
       <c r="F143" s="6"/>
       <c r="G143" s="11">
         <f t="shared" si="23"/>
-        <v>-1.0629333333334046E-4</v>
+        <v>-1.1431333333344895E-4</v>
       </c>
       <c r="H143" s="11"/>
       <c r="I143" s="11"/>
       <c r="J143" s="6"/>
       <c r="K143" s="10">
         <f t="shared" si="24"/>
-        <v>-1.5868100258229414E-4</v>
+        <v>-1.7056337040478677E-4</v>
       </c>
       <c r="L143" s="10"/>
       <c r="M143" s="10"/>
@@ -5062,10 +5059,10 @@
     </row>
     <row r="145" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A145" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B145" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C145" s="11"/>
       <c r="D145" s="11"/>
@@ -5077,16 +5074,16 @@
       <c r="H145" s="11"/>
       <c r="I145" s="11"/>
       <c r="J145" s="6"/>
-      <c r="K145" s="13">
-        <v>0</v>
-      </c>
-      <c r="L145" s="13"/>
-      <c r="M145" s="13"/>
+      <c r="K145" s="15">
+        <v>0</v>
+      </c>
+      <c r="L145" s="15"/>
+      <c r="M145" s="15"/>
       <c r="N145" s="6"/>
     </row>
     <row r="146" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A146" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B146" s="11">
         <v>1</v>
@@ -5111,7 +5108,7 @@
     </row>
     <row r="147" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A147" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B147" s="11">
         <v>69633</v>
@@ -5136,7 +5133,7 @@
     </row>
     <row r="148" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A148" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B148" s="11">
         <v>70352</v>
@@ -5161,7 +5158,7 @@
     </row>
     <row r="149" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A149" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B149" s="11">
         <v>73927</v>
@@ -5186,7 +5183,7 @@
     </row>
     <row r="150" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A150" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B150" s="11">
         <f>B149-B146</f>
@@ -5212,7 +5209,7 @@
     </row>
     <row r="151" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A151" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B151" s="11">
         <f>B150/(B3*10^3)</f>
@@ -5246,7 +5243,7 @@
     </row>
     <row r="152" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A152" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B152" s="11">
         <f>B149-B147</f>
@@ -5272,7 +5269,7 @@
     </row>
     <row r="153" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A153" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B153" s="11">
         <f>B152/B3</f>
@@ -5306,7 +5303,7 @@
     </row>
     <row r="154" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A154" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B154" s="1">
         <f>B12*B151</f>
@@ -5354,7 +5351,7 @@
     </row>
     <row r="155" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A155" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B155" s="11">
         <f>1/(B151/1000)</f>
@@ -5404,63 +5401,285 @@
     </row>
   </sheetData>
   <mergeCells count="360">
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="G59:I59"/>
-    <mergeCell ref="K59:M59"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="G56:I56"/>
-    <mergeCell ref="K56:M56"/>
-    <mergeCell ref="C57:E57"/>
-    <mergeCell ref="G57:I57"/>
-    <mergeCell ref="K57:M57"/>
-    <mergeCell ref="C58:E58"/>
-    <mergeCell ref="G58:I58"/>
-    <mergeCell ref="K58:M58"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="G53:I53"/>
-    <mergeCell ref="K53:M53"/>
-    <mergeCell ref="C54:E54"/>
-    <mergeCell ref="G54:I54"/>
-    <mergeCell ref="K54:M54"/>
-    <mergeCell ref="C55:E55"/>
-    <mergeCell ref="G55:I55"/>
-    <mergeCell ref="K55:M55"/>
-    <mergeCell ref="C50:E50"/>
-    <mergeCell ref="G50:I50"/>
-    <mergeCell ref="K50:M50"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="G51:I51"/>
-    <mergeCell ref="K51:M51"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="G52:I52"/>
-    <mergeCell ref="K52:M52"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="G47:I47"/>
-    <mergeCell ref="K47:M47"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="G48:I48"/>
-    <mergeCell ref="K48:M48"/>
-    <mergeCell ref="C49:E49"/>
-    <mergeCell ref="G49:I49"/>
-    <mergeCell ref="K49:M49"/>
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="G43:I43"/>
-    <mergeCell ref="K43:M43"/>
-    <mergeCell ref="C44:E44"/>
-    <mergeCell ref="G44:I44"/>
-    <mergeCell ref="K44:M44"/>
-    <mergeCell ref="C45:E45"/>
-    <mergeCell ref="G45:I45"/>
-    <mergeCell ref="K45:M45"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="G40:I40"/>
-    <mergeCell ref="K40:M40"/>
-    <mergeCell ref="C41:E41"/>
-    <mergeCell ref="G41:I41"/>
-    <mergeCell ref="K41:M41"/>
-    <mergeCell ref="C42:E42"/>
-    <mergeCell ref="G42:I42"/>
-    <mergeCell ref="K42:M42"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="G153:H153"/>
+    <mergeCell ref="G155:H155"/>
+    <mergeCell ref="G151:H151"/>
+    <mergeCell ref="K151:L151"/>
+    <mergeCell ref="K153:L153"/>
+    <mergeCell ref="K155:L155"/>
+    <mergeCell ref="K146:M146"/>
+    <mergeCell ref="K152:M152"/>
+    <mergeCell ref="K150:M150"/>
+    <mergeCell ref="K149:M149"/>
+    <mergeCell ref="K148:M148"/>
+    <mergeCell ref="K147:M147"/>
+    <mergeCell ref="K134:M134"/>
+    <mergeCell ref="K140:M140"/>
+    <mergeCell ref="K141:M141"/>
+    <mergeCell ref="K142:M142"/>
+    <mergeCell ref="K118:M118"/>
+    <mergeCell ref="K119:M119"/>
+    <mergeCell ref="K120:M120"/>
+    <mergeCell ref="K121:M121"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="B153:D153"/>
+    <mergeCell ref="B155:D155"/>
+    <mergeCell ref="B151:D151"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="G127:I127"/>
+    <mergeCell ref="G128:I128"/>
+    <mergeCell ref="B152:E152"/>
+    <mergeCell ref="G145:I145"/>
+    <mergeCell ref="G146:I146"/>
+    <mergeCell ref="G147:I147"/>
+    <mergeCell ref="G148:I148"/>
+    <mergeCell ref="G149:I149"/>
+    <mergeCell ref="G150:I150"/>
+    <mergeCell ref="G152:I152"/>
+    <mergeCell ref="B146:E146"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="B145:E145"/>
+    <mergeCell ref="G118:I118"/>
+    <mergeCell ref="G119:I119"/>
+    <mergeCell ref="G120:I120"/>
+    <mergeCell ref="G121:I121"/>
+    <mergeCell ref="G122:I122"/>
+    <mergeCell ref="G123:I123"/>
+    <mergeCell ref="G124:I124"/>
+    <mergeCell ref="G125:I125"/>
+    <mergeCell ref="G126:I126"/>
+    <mergeCell ref="K145:M145"/>
+    <mergeCell ref="C118:E118"/>
+    <mergeCell ref="C119:E119"/>
+    <mergeCell ref="C120:E120"/>
+    <mergeCell ref="C121:E121"/>
+    <mergeCell ref="C122:E122"/>
+    <mergeCell ref="C123:E123"/>
+    <mergeCell ref="C124:E124"/>
+    <mergeCell ref="C125:E125"/>
+    <mergeCell ref="C126:E126"/>
+    <mergeCell ref="B147:E147"/>
+    <mergeCell ref="B148:E148"/>
+    <mergeCell ref="B149:E149"/>
+    <mergeCell ref="B150:E150"/>
+    <mergeCell ref="C138:E138"/>
+    <mergeCell ref="C139:E139"/>
+    <mergeCell ref="C140:E140"/>
+    <mergeCell ref="G129:I129"/>
+    <mergeCell ref="C132:E132"/>
+    <mergeCell ref="C133:E133"/>
+    <mergeCell ref="C134:E134"/>
+    <mergeCell ref="C135:E135"/>
+    <mergeCell ref="C128:E128"/>
+    <mergeCell ref="C129:E129"/>
+    <mergeCell ref="C137:E137"/>
+    <mergeCell ref="C141:E141"/>
+    <mergeCell ref="C142:E142"/>
+    <mergeCell ref="C143:E143"/>
+    <mergeCell ref="G132:I132"/>
+    <mergeCell ref="G133:I133"/>
+    <mergeCell ref="G134:I134"/>
+    <mergeCell ref="G135:I135"/>
+    <mergeCell ref="G136:I136"/>
+    <mergeCell ref="G137:I137"/>
+    <mergeCell ref="G138:I138"/>
+    <mergeCell ref="G139:I139"/>
+    <mergeCell ref="G140:I140"/>
+    <mergeCell ref="G141:I141"/>
+    <mergeCell ref="G142:I142"/>
+    <mergeCell ref="G143:I143"/>
+    <mergeCell ref="C136:E136"/>
+    <mergeCell ref="K133:M133"/>
+    <mergeCell ref="K143:M143"/>
+    <mergeCell ref="K135:M135"/>
+    <mergeCell ref="K136:M136"/>
+    <mergeCell ref="K137:M137"/>
+    <mergeCell ref="K138:M138"/>
+    <mergeCell ref="K139:M139"/>
+    <mergeCell ref="K117:M117"/>
+    <mergeCell ref="G117:I117"/>
+    <mergeCell ref="K122:M122"/>
+    <mergeCell ref="K123:M123"/>
+    <mergeCell ref="K124:M124"/>
+    <mergeCell ref="K125:M125"/>
+    <mergeCell ref="K126:M126"/>
+    <mergeCell ref="K127:M127"/>
+    <mergeCell ref="K128:M128"/>
+    <mergeCell ref="K129:M129"/>
+    <mergeCell ref="K132:M132"/>
+    <mergeCell ref="B117:E117"/>
+    <mergeCell ref="B131:E131"/>
+    <mergeCell ref="G131:I131"/>
+    <mergeCell ref="K131:M131"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="G89:I89"/>
+    <mergeCell ref="K89:M89"/>
+    <mergeCell ref="C90:E90"/>
+    <mergeCell ref="G90:I90"/>
+    <mergeCell ref="K90:M90"/>
+    <mergeCell ref="C91:E91"/>
+    <mergeCell ref="G91:I91"/>
+    <mergeCell ref="K91:M91"/>
+    <mergeCell ref="C92:E92"/>
+    <mergeCell ref="G92:I92"/>
+    <mergeCell ref="K92:M92"/>
+    <mergeCell ref="C93:E93"/>
+    <mergeCell ref="G93:I93"/>
+    <mergeCell ref="K93:M93"/>
+    <mergeCell ref="C94:E94"/>
+    <mergeCell ref="G94:I94"/>
+    <mergeCell ref="K94:M94"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="C127:E127"/>
+    <mergeCell ref="G95:I95"/>
+    <mergeCell ref="K95:M95"/>
+    <mergeCell ref="C96:E96"/>
+    <mergeCell ref="G96:I96"/>
+    <mergeCell ref="K96:M96"/>
+    <mergeCell ref="C97:E97"/>
+    <mergeCell ref="G97:I97"/>
+    <mergeCell ref="K97:M97"/>
+    <mergeCell ref="C98:E98"/>
+    <mergeCell ref="G98:I98"/>
+    <mergeCell ref="K98:M98"/>
+    <mergeCell ref="C99:E99"/>
+    <mergeCell ref="G99:I99"/>
+    <mergeCell ref="K99:M99"/>
+    <mergeCell ref="C100:E100"/>
+    <mergeCell ref="G100:I100"/>
+    <mergeCell ref="K100:M100"/>
+    <mergeCell ref="C101:E101"/>
+    <mergeCell ref="G101:I101"/>
+    <mergeCell ref="K101:M101"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="G103:I103"/>
+    <mergeCell ref="K103:M103"/>
+    <mergeCell ref="C104:E104"/>
+    <mergeCell ref="G104:I104"/>
+    <mergeCell ref="K104:M104"/>
+    <mergeCell ref="C105:E105"/>
+    <mergeCell ref="G105:I105"/>
+    <mergeCell ref="K105:M105"/>
+    <mergeCell ref="C106:E106"/>
+    <mergeCell ref="G106:I106"/>
+    <mergeCell ref="K106:M106"/>
+    <mergeCell ref="C107:E107"/>
+    <mergeCell ref="G107:I107"/>
+    <mergeCell ref="K107:M107"/>
+    <mergeCell ref="C108:E108"/>
+    <mergeCell ref="G108:I108"/>
+    <mergeCell ref="K108:M108"/>
+    <mergeCell ref="C109:E109"/>
+    <mergeCell ref="G109:I109"/>
+    <mergeCell ref="K109:M109"/>
+    <mergeCell ref="C110:E110"/>
+    <mergeCell ref="G110:I110"/>
+    <mergeCell ref="K110:M110"/>
+    <mergeCell ref="C111:E111"/>
+    <mergeCell ref="G111:I111"/>
+    <mergeCell ref="K111:M111"/>
+    <mergeCell ref="C112:E112"/>
+    <mergeCell ref="G112:I112"/>
+    <mergeCell ref="K112:M112"/>
+    <mergeCell ref="C113:E113"/>
+    <mergeCell ref="G113:I113"/>
+    <mergeCell ref="K113:M113"/>
+    <mergeCell ref="C114:E114"/>
+    <mergeCell ref="G114:I114"/>
+    <mergeCell ref="K114:M114"/>
+    <mergeCell ref="C115:E115"/>
+    <mergeCell ref="G115:I115"/>
+    <mergeCell ref="K115:M115"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="G61:I61"/>
+    <mergeCell ref="K61:M61"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="G62:I62"/>
+    <mergeCell ref="K62:M62"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="G63:I63"/>
+    <mergeCell ref="K63:M63"/>
+    <mergeCell ref="C64:E64"/>
+    <mergeCell ref="G64:I64"/>
+    <mergeCell ref="K64:M64"/>
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="G65:I65"/>
+    <mergeCell ref="K65:M65"/>
+    <mergeCell ref="C66:E66"/>
+    <mergeCell ref="G66:I66"/>
+    <mergeCell ref="K66:M66"/>
+    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="G67:I67"/>
+    <mergeCell ref="K67:M67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="G68:I68"/>
+    <mergeCell ref="K68:M68"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="G69:I69"/>
+    <mergeCell ref="K69:M69"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="G70:I70"/>
+    <mergeCell ref="K70:M70"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="G71:I71"/>
+    <mergeCell ref="K71:M71"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="G72:I72"/>
+    <mergeCell ref="K72:M72"/>
+    <mergeCell ref="C73:E73"/>
+    <mergeCell ref="G73:I73"/>
+    <mergeCell ref="K73:M73"/>
+    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="G75:I75"/>
+    <mergeCell ref="K75:M75"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="G76:I76"/>
+    <mergeCell ref="K76:M76"/>
+    <mergeCell ref="C77:E77"/>
+    <mergeCell ref="G77:I77"/>
+    <mergeCell ref="K77:M77"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="G78:I78"/>
+    <mergeCell ref="K78:M78"/>
+    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="G79:I79"/>
+    <mergeCell ref="K79:M79"/>
+    <mergeCell ref="C80:E80"/>
+    <mergeCell ref="G80:I80"/>
+    <mergeCell ref="K80:M80"/>
+    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="G81:I81"/>
+    <mergeCell ref="K81:M81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="G82:I82"/>
+    <mergeCell ref="K82:M82"/>
+    <mergeCell ref="C83:E83"/>
+    <mergeCell ref="G83:I83"/>
+    <mergeCell ref="K83:M83"/>
+    <mergeCell ref="C84:E84"/>
+    <mergeCell ref="G84:I84"/>
+    <mergeCell ref="K84:M84"/>
+    <mergeCell ref="C85:E85"/>
+    <mergeCell ref="G85:I85"/>
+    <mergeCell ref="K85:M85"/>
+    <mergeCell ref="C86:E86"/>
+    <mergeCell ref="G86:I86"/>
+    <mergeCell ref="K86:M86"/>
     <mergeCell ref="C87:E87"/>
     <mergeCell ref="G87:I87"/>
     <mergeCell ref="K87:M87"/>
@@ -5485,285 +5704,63 @@
     <mergeCell ref="C39:E39"/>
     <mergeCell ref="G39:I39"/>
     <mergeCell ref="K39:M39"/>
-    <mergeCell ref="C84:E84"/>
-    <mergeCell ref="G84:I84"/>
-    <mergeCell ref="K84:M84"/>
-    <mergeCell ref="C85:E85"/>
-    <mergeCell ref="G85:I85"/>
-    <mergeCell ref="K85:M85"/>
-    <mergeCell ref="C86:E86"/>
-    <mergeCell ref="G86:I86"/>
-    <mergeCell ref="K86:M86"/>
-    <mergeCell ref="C81:E81"/>
-    <mergeCell ref="G81:I81"/>
-    <mergeCell ref="K81:M81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="G82:I82"/>
-    <mergeCell ref="K82:M82"/>
-    <mergeCell ref="C83:E83"/>
-    <mergeCell ref="G83:I83"/>
-    <mergeCell ref="K83:M83"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="G78:I78"/>
-    <mergeCell ref="K78:M78"/>
-    <mergeCell ref="C79:E79"/>
-    <mergeCell ref="G79:I79"/>
-    <mergeCell ref="K79:M79"/>
-    <mergeCell ref="C80:E80"/>
-    <mergeCell ref="G80:I80"/>
-    <mergeCell ref="K80:M80"/>
-    <mergeCell ref="B75:E75"/>
-    <mergeCell ref="G75:I75"/>
-    <mergeCell ref="K75:M75"/>
-    <mergeCell ref="C76:E76"/>
-    <mergeCell ref="G76:I76"/>
-    <mergeCell ref="K76:M76"/>
-    <mergeCell ref="C77:E77"/>
-    <mergeCell ref="G77:I77"/>
-    <mergeCell ref="K77:M77"/>
-    <mergeCell ref="C71:E71"/>
-    <mergeCell ref="G71:I71"/>
-    <mergeCell ref="K71:M71"/>
-    <mergeCell ref="C72:E72"/>
-    <mergeCell ref="G72:I72"/>
-    <mergeCell ref="K72:M72"/>
-    <mergeCell ref="C73:E73"/>
-    <mergeCell ref="G73:I73"/>
-    <mergeCell ref="K73:M73"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="G68:I68"/>
-    <mergeCell ref="K68:M68"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="G69:I69"/>
-    <mergeCell ref="K69:M69"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="G70:I70"/>
-    <mergeCell ref="K70:M70"/>
-    <mergeCell ref="C115:E115"/>
-    <mergeCell ref="G115:I115"/>
-    <mergeCell ref="K115:M115"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="G61:I61"/>
-    <mergeCell ref="K61:M61"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="G62:I62"/>
-    <mergeCell ref="K62:M62"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="G63:I63"/>
-    <mergeCell ref="K63:M63"/>
-    <mergeCell ref="C64:E64"/>
-    <mergeCell ref="G64:I64"/>
-    <mergeCell ref="K64:M64"/>
-    <mergeCell ref="C65:E65"/>
-    <mergeCell ref="G65:I65"/>
-    <mergeCell ref="K65:M65"/>
-    <mergeCell ref="C66:E66"/>
-    <mergeCell ref="G66:I66"/>
-    <mergeCell ref="K66:M66"/>
-    <mergeCell ref="C67:E67"/>
-    <mergeCell ref="G67:I67"/>
-    <mergeCell ref="K67:M67"/>
-    <mergeCell ref="C112:E112"/>
-    <mergeCell ref="G112:I112"/>
-    <mergeCell ref="K112:M112"/>
-    <mergeCell ref="C113:E113"/>
-    <mergeCell ref="G113:I113"/>
-    <mergeCell ref="K113:M113"/>
-    <mergeCell ref="C114:E114"/>
-    <mergeCell ref="G114:I114"/>
-    <mergeCell ref="K114:M114"/>
-    <mergeCell ref="C109:E109"/>
-    <mergeCell ref="G109:I109"/>
-    <mergeCell ref="K109:M109"/>
-    <mergeCell ref="C110:E110"/>
-    <mergeCell ref="G110:I110"/>
-    <mergeCell ref="K110:M110"/>
-    <mergeCell ref="C111:E111"/>
-    <mergeCell ref="G111:I111"/>
-    <mergeCell ref="K111:M111"/>
-    <mergeCell ref="C106:E106"/>
-    <mergeCell ref="G106:I106"/>
-    <mergeCell ref="K106:M106"/>
-    <mergeCell ref="C107:E107"/>
-    <mergeCell ref="G107:I107"/>
-    <mergeCell ref="K107:M107"/>
-    <mergeCell ref="C108:E108"/>
-    <mergeCell ref="G108:I108"/>
-    <mergeCell ref="K108:M108"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="G103:I103"/>
-    <mergeCell ref="K103:M103"/>
-    <mergeCell ref="C104:E104"/>
-    <mergeCell ref="G104:I104"/>
-    <mergeCell ref="K104:M104"/>
-    <mergeCell ref="C105:E105"/>
-    <mergeCell ref="G105:I105"/>
-    <mergeCell ref="K105:M105"/>
-    <mergeCell ref="C99:E99"/>
-    <mergeCell ref="G99:I99"/>
-    <mergeCell ref="K99:M99"/>
-    <mergeCell ref="C100:E100"/>
-    <mergeCell ref="G100:I100"/>
-    <mergeCell ref="K100:M100"/>
-    <mergeCell ref="C101:E101"/>
-    <mergeCell ref="G101:I101"/>
-    <mergeCell ref="K101:M101"/>
-    <mergeCell ref="G95:I95"/>
-    <mergeCell ref="K95:M95"/>
-    <mergeCell ref="C96:E96"/>
-    <mergeCell ref="G96:I96"/>
-    <mergeCell ref="K96:M96"/>
-    <mergeCell ref="C97:E97"/>
-    <mergeCell ref="G97:I97"/>
-    <mergeCell ref="K97:M97"/>
-    <mergeCell ref="C98:E98"/>
-    <mergeCell ref="G98:I98"/>
-    <mergeCell ref="K98:M98"/>
-    <mergeCell ref="B117:E117"/>
-    <mergeCell ref="B131:E131"/>
-    <mergeCell ref="G131:I131"/>
-    <mergeCell ref="K131:M131"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="G89:I89"/>
-    <mergeCell ref="K89:M89"/>
-    <mergeCell ref="C90:E90"/>
-    <mergeCell ref="G90:I90"/>
-    <mergeCell ref="K90:M90"/>
-    <mergeCell ref="C91:E91"/>
-    <mergeCell ref="G91:I91"/>
-    <mergeCell ref="K91:M91"/>
-    <mergeCell ref="C92:E92"/>
-    <mergeCell ref="G92:I92"/>
-    <mergeCell ref="K92:M92"/>
-    <mergeCell ref="C93:E93"/>
-    <mergeCell ref="G93:I93"/>
-    <mergeCell ref="K93:M93"/>
-    <mergeCell ref="C94:E94"/>
-    <mergeCell ref="G94:I94"/>
-    <mergeCell ref="K94:M94"/>
-    <mergeCell ref="C95:E95"/>
-    <mergeCell ref="C127:E127"/>
-    <mergeCell ref="K133:M133"/>
-    <mergeCell ref="K143:M143"/>
-    <mergeCell ref="K135:M135"/>
-    <mergeCell ref="K136:M136"/>
-    <mergeCell ref="K137:M137"/>
-    <mergeCell ref="K138:M138"/>
-    <mergeCell ref="K139:M139"/>
-    <mergeCell ref="K117:M117"/>
-    <mergeCell ref="G117:I117"/>
-    <mergeCell ref="K122:M122"/>
-    <mergeCell ref="K123:M123"/>
-    <mergeCell ref="K124:M124"/>
-    <mergeCell ref="K125:M125"/>
-    <mergeCell ref="K126:M126"/>
-    <mergeCell ref="K127:M127"/>
-    <mergeCell ref="K128:M128"/>
-    <mergeCell ref="K129:M129"/>
-    <mergeCell ref="K132:M132"/>
-    <mergeCell ref="C128:E128"/>
-    <mergeCell ref="C129:E129"/>
-    <mergeCell ref="C137:E137"/>
-    <mergeCell ref="C141:E141"/>
-    <mergeCell ref="C142:E142"/>
-    <mergeCell ref="C143:E143"/>
-    <mergeCell ref="G132:I132"/>
-    <mergeCell ref="G133:I133"/>
-    <mergeCell ref="G134:I134"/>
-    <mergeCell ref="G135:I135"/>
-    <mergeCell ref="G136:I136"/>
-    <mergeCell ref="G137:I137"/>
-    <mergeCell ref="G138:I138"/>
-    <mergeCell ref="G139:I139"/>
-    <mergeCell ref="G140:I140"/>
-    <mergeCell ref="G141:I141"/>
-    <mergeCell ref="G142:I142"/>
-    <mergeCell ref="G143:I143"/>
-    <mergeCell ref="C136:E136"/>
-    <mergeCell ref="B147:E147"/>
-    <mergeCell ref="B148:E148"/>
-    <mergeCell ref="B149:E149"/>
-    <mergeCell ref="B150:E150"/>
-    <mergeCell ref="C138:E138"/>
-    <mergeCell ref="C139:E139"/>
-    <mergeCell ref="C140:E140"/>
-    <mergeCell ref="G129:I129"/>
-    <mergeCell ref="C132:E132"/>
-    <mergeCell ref="C133:E133"/>
-    <mergeCell ref="C134:E134"/>
-    <mergeCell ref="C135:E135"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="B145:E145"/>
-    <mergeCell ref="G118:I118"/>
-    <mergeCell ref="G119:I119"/>
-    <mergeCell ref="G120:I120"/>
-    <mergeCell ref="G121:I121"/>
-    <mergeCell ref="G122:I122"/>
-    <mergeCell ref="G123:I123"/>
-    <mergeCell ref="G124:I124"/>
-    <mergeCell ref="G125:I125"/>
-    <mergeCell ref="G126:I126"/>
-    <mergeCell ref="K145:M145"/>
-    <mergeCell ref="C118:E118"/>
-    <mergeCell ref="C119:E119"/>
-    <mergeCell ref="C120:E120"/>
-    <mergeCell ref="C121:E121"/>
-    <mergeCell ref="C122:E122"/>
-    <mergeCell ref="C123:E123"/>
-    <mergeCell ref="C124:E124"/>
-    <mergeCell ref="C125:E125"/>
-    <mergeCell ref="C126:E126"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="B153:D153"/>
-    <mergeCell ref="B155:D155"/>
-    <mergeCell ref="B151:D151"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="G127:I127"/>
-    <mergeCell ref="G128:I128"/>
-    <mergeCell ref="B152:E152"/>
-    <mergeCell ref="G145:I145"/>
-    <mergeCell ref="G146:I146"/>
-    <mergeCell ref="G147:I147"/>
-    <mergeCell ref="G148:I148"/>
-    <mergeCell ref="G149:I149"/>
-    <mergeCell ref="G150:I150"/>
-    <mergeCell ref="G152:I152"/>
-    <mergeCell ref="B146:E146"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="G153:H153"/>
-    <mergeCell ref="G155:H155"/>
-    <mergeCell ref="G151:H151"/>
-    <mergeCell ref="K151:L151"/>
-    <mergeCell ref="K153:L153"/>
-    <mergeCell ref="K155:L155"/>
-    <mergeCell ref="K146:M146"/>
-    <mergeCell ref="K152:M152"/>
-    <mergeCell ref="K150:M150"/>
-    <mergeCell ref="K149:M149"/>
-    <mergeCell ref="K148:M148"/>
-    <mergeCell ref="K147:M147"/>
-    <mergeCell ref="K134:M134"/>
-    <mergeCell ref="K140:M140"/>
-    <mergeCell ref="K141:M141"/>
-    <mergeCell ref="K142:M142"/>
-    <mergeCell ref="K118:M118"/>
-    <mergeCell ref="K119:M119"/>
-    <mergeCell ref="K120:M120"/>
-    <mergeCell ref="K121:M121"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="G40:I40"/>
+    <mergeCell ref="K40:M40"/>
+    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="G41:I41"/>
+    <mergeCell ref="K41:M41"/>
+    <mergeCell ref="C42:E42"/>
+    <mergeCell ref="G42:I42"/>
+    <mergeCell ref="K42:M42"/>
+    <mergeCell ref="C43:E43"/>
+    <mergeCell ref="G43:I43"/>
+    <mergeCell ref="K43:M43"/>
+    <mergeCell ref="C44:E44"/>
+    <mergeCell ref="G44:I44"/>
+    <mergeCell ref="K44:M44"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="G45:I45"/>
+    <mergeCell ref="K45:M45"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="G47:I47"/>
+    <mergeCell ref="K47:M47"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="G48:I48"/>
+    <mergeCell ref="K48:M48"/>
+    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="G49:I49"/>
+    <mergeCell ref="K49:M49"/>
+    <mergeCell ref="C50:E50"/>
+    <mergeCell ref="G50:I50"/>
+    <mergeCell ref="K50:M50"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="G51:I51"/>
+    <mergeCell ref="K51:M51"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="G52:I52"/>
+    <mergeCell ref="K52:M52"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="G53:I53"/>
+    <mergeCell ref="K53:M53"/>
+    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="G54:I54"/>
+    <mergeCell ref="K54:M54"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="G55:I55"/>
+    <mergeCell ref="K55:M55"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="G59:I59"/>
+    <mergeCell ref="K59:M59"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="G56:I56"/>
+    <mergeCell ref="K56:M56"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="G57:I57"/>
+    <mergeCell ref="K57:M57"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="G58:I58"/>
+    <mergeCell ref="K58:M58"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
MISC: Hold this and look into python and FPGA pipeline design changes.
</commit_message>
<xml_diff>
--- a/FPGA_Performance_Comparison_RGB.xlsx
+++ b/FPGA_Performance_Comparison_RGB.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/DanielBiswas/Desktop/Documents/University/Year 5/Semester 1/AMME4112/Code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4C74CC7-1F88-564D-B9C2-80C8011B9B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0488B765-EB5F-D34C-A16B-0C99B83F0755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="24660" windowHeight="26820" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="24660" windowHeight="17740" xr2:uid="{49DEC02E-5D37-064F-A7E8-1E1DC7B5FEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="81">
   <si>
     <t>FPGA Implementation</t>
   </si>
@@ -267,6 +267,18 @@
   </si>
   <si>
     <t>Disparity Exact Match Pixels (Out Of 2916)</t>
+  </si>
+  <si>
+    <t>Confidence Exact Match Pixels (Out Of 8748)</t>
+  </si>
+  <si>
+    <t>Disparity Exact Match Pixels (Out Of 8748)</t>
+  </si>
+  <si>
+    <t>Disparity Exact Match Percentage</t>
+  </si>
+  <si>
+    <t>Confidence Exact Match Percentage</t>
   </si>
 </sst>
 </file>
@@ -362,17 +374,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -719,15 +731,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
+      <c r="B1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
       <c r="F1" s="6"/>
       <c r="G1" s="11" t="s">
         <v>54</v>
@@ -743,7 +755,7 @@
       <c r="N1" s="6"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A2" s="14"/>
+      <c r="A2" s="12"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2352,11 +2364,11 @@
       <c r="B45" s="5">
         <v>0.15534978999999999</v>
       </c>
-      <c r="C45" s="12">
+      <c r="C45" s="15">
         <v>0.14986283</v>
       </c>
-      <c r="D45" s="12"/>
-      <c r="E45" s="12"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15"/>
       <c r="F45" s="6"/>
       <c r="G45" s="11">
         <f t="shared" si="7"/>
@@ -3103,11 +3115,11 @@
       <c r="B73" s="5">
         <v>5.14403E-3</v>
       </c>
-      <c r="C73" s="12">
+      <c r="C73" s="15">
         <v>5.14403E-3</v>
       </c>
-      <c r="D73" s="12"/>
-      <c r="E73" s="12"/>
+      <c r="D73" s="15"/>
+      <c r="E73" s="15"/>
       <c r="F73" s="6"/>
       <c r="G73" s="11">
         <f t="shared" si="11"/>
@@ -3848,11 +3860,11 @@
       <c r="B101" s="5">
         <v>6.0699589999999998E-2</v>
       </c>
-      <c r="C101" s="12">
+      <c r="C101" s="15">
         <v>5.5212619999999997E-2</v>
       </c>
-      <c r="D101" s="12"/>
-      <c r="E101" s="12"/>
+      <c r="D101" s="15"/>
+      <c r="E101" s="15"/>
       <c r="F101" s="6"/>
       <c r="G101" s="11">
         <f t="shared" si="15"/>
@@ -4347,15 +4359,21 @@
         <v>34</v>
       </c>
       <c r="B120" s="1">
-        <f t="shared" si="20"/>
-        <v>4</v>
+        <f>MEDIAN(B64,B36,B92)</f>
+        <v>2</v>
       </c>
       <c r="C120" s="11">
-        <f t="shared" si="21"/>
-        <v>4</v>
-      </c>
-      <c r="D120" s="11"/>
-      <c r="E120" s="11"/>
+        <f t="shared" ref="C120:E120" si="22">MEDIAN(C64,C36,C92)</f>
+        <v>2</v>
+      </c>
+      <c r="D120" s="11" t="e">
+        <f t="shared" si="22"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E120" s="11" t="e">
+        <f t="shared" si="22"/>
+        <v>#NUM!</v>
+      </c>
       <c r="F120" s="6"/>
       <c r="G120" s="11">
         <f t="shared" si="19"/>
@@ -4377,15 +4395,21 @@
         <v>35</v>
       </c>
       <c r="B121" s="1">
-        <f t="shared" si="20"/>
-        <v>4</v>
+        <f>MEDIAN(B65,B37,B93)</f>
+        <v>2</v>
       </c>
       <c r="C121" s="11">
-        <f t="shared" si="21"/>
-        <v>4</v>
-      </c>
-      <c r="D121" s="11"/>
-      <c r="E121" s="11"/>
+        <f t="shared" ref="C121:E121" si="23">MEDIAN(C65,C37,C93)</f>
+        <v>2</v>
+      </c>
+      <c r="D121" s="11" t="e">
+        <f t="shared" si="23"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E121" s="11" t="e">
+        <f t="shared" si="23"/>
+        <v>#NUM!</v>
+      </c>
       <c r="F121" s="6"/>
       <c r="G121" s="11">
         <f t="shared" si="19"/>
@@ -4407,11 +4431,11 @@
         <v>36</v>
       </c>
       <c r="B122" s="1">
-        <f t="shared" si="20"/>
+        <f>MIN(B66,B38,B94)</f>
         <v>0</v>
       </c>
       <c r="C122" s="11">
-        <f t="shared" si="21"/>
+        <f>MIN(C66,C38,C94)</f>
         <v>0</v>
       </c>
       <c r="D122" s="11"/>
@@ -4436,26 +4460,26 @@
         <v>37</v>
       </c>
       <c r="B123" s="1">
-        <f t="shared" si="20"/>
-        <v>25</v>
+        <f>MAX(B67,B39,B95)</f>
+        <v>40</v>
       </c>
       <c r="C123" s="11">
-        <f t="shared" si="21"/>
-        <v>24.666666666666668</v>
+        <f>MAX(C67,C39,C95)</f>
+        <v>39</v>
       </c>
       <c r="D123" s="11"/>
       <c r="E123" s="11"/>
       <c r="F123" s="6"/>
       <c r="G123" s="11">
         <f t="shared" si="19"/>
-        <v>-0.33333333333333215</v>
+        <v>-1</v>
       </c>
       <c r="H123" s="11"/>
       <c r="I123" s="11"/>
       <c r="J123" s="6"/>
       <c r="K123" s="10">
-        <f t="shared" ref="K123:K129" si="22">G123/B123</f>
-        <v>-1.3333333333333286E-2</v>
+        <f t="shared" ref="K123:K129" si="24">G123/B123</f>
+        <v>-2.5000000000000001E-2</v>
       </c>
       <c r="L123" s="10"/>
       <c r="M123" s="10"/>
@@ -4466,7 +4490,7 @@
         <v>38</v>
       </c>
       <c r="B124" s="1">
-        <f t="shared" si="20"/>
+        <f>AVERAGE(B68,B40,B96)</f>
         <v>6.4252399999999996</v>
       </c>
       <c r="C124" s="11">
@@ -4484,7 +4508,7 @@
       <c r="I124" s="11"/>
       <c r="J124" s="6"/>
       <c r="K124" s="10">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>-9.0735910253942991E-4</v>
       </c>
       <c r="L124" s="10"/>
@@ -4496,12 +4520,12 @@
         <v>39</v>
       </c>
       <c r="B125" s="1">
-        <f t="shared" si="20"/>
-        <v>6.666666666666667</v>
+        <f>MEDIAN(B69,B41,B97)</f>
+        <v>7</v>
       </c>
       <c r="C125" s="11">
-        <f t="shared" si="21"/>
-        <v>6.666666666666667</v>
+        <f>MEDIAN(C69,C41,C97)</f>
+        <v>7</v>
       </c>
       <c r="D125" s="11"/>
       <c r="E125" s="11"/>
@@ -4514,7 +4538,7 @@
       <c r="I125" s="11"/>
       <c r="J125" s="6"/>
       <c r="K125" s="10">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="L125" s="10"/>
@@ -4526,11 +4550,11 @@
         <v>40</v>
       </c>
       <c r="B126" s="1">
-        <f t="shared" si="20"/>
+        <f>MAX(B70,B42,B98)</f>
         <v>8</v>
       </c>
       <c r="C126" s="11">
-        <f t="shared" si="21"/>
+        <f>MAX(C70,C42,C98)</f>
         <v>8</v>
       </c>
       <c r="D126" s="11"/>
@@ -4544,7 +4568,7 @@
       <c r="I126" s="11"/>
       <c r="J126" s="6"/>
       <c r="K126" s="10">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="L126" s="10"/>
@@ -4556,12 +4580,12 @@
         <v>41</v>
       </c>
       <c r="B127" s="1">
-        <f t="shared" si="20"/>
-        <v>3.3333333333333335</v>
+        <f>MIN(B71,B43,B99)</f>
+        <v>3</v>
       </c>
       <c r="C127" s="11">
-        <f t="shared" si="21"/>
-        <v>3.3333333333333335</v>
+        <f>MIN(C71,C43,C99)</f>
+        <v>3</v>
       </c>
       <c r="D127" s="11"/>
       <c r="E127" s="11"/>
@@ -4574,7 +4598,7 @@
       <c r="I127" s="11"/>
       <c r="J127" s="6"/>
       <c r="K127" s="10">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="L127" s="10"/>
@@ -4583,29 +4607,29 @@
     </row>
     <row r="128" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A128" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B128" s="1">
-        <f t="shared" si="20"/>
-        <v>215</v>
+        <f>SUM(B72,B44,B100)</f>
+        <v>645</v>
       </c>
       <c r="C128" s="11">
-        <f t="shared" si="21"/>
-        <v>204.33333333333334</v>
+        <f>SUM(C72,C44,C100)</f>
+        <v>613</v>
       </c>
       <c r="D128" s="11"/>
       <c r="E128" s="11"/>
       <c r="F128" s="6"/>
       <c r="G128" s="11">
         <f t="shared" si="19"/>
-        <v>-10.666666666666657</v>
+        <v>-32</v>
       </c>
       <c r="H128" s="11"/>
       <c r="I128" s="11"/>
       <c r="J128" s="6"/>
       <c r="K128" s="10">
-        <f t="shared" si="22"/>
-        <v>-4.9612403100775151E-2</v>
+        <f t="shared" si="24"/>
+        <v>-4.9612403100775193E-2</v>
       </c>
       <c r="L128" s="10"/>
       <c r="M128" s="10"/>
@@ -4613,29 +4637,29 @@
     </row>
     <row r="129" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A129" s="3" t="s">
-        <v>42</v>
+        <v>80</v>
       </c>
       <c r="B129" s="5">
-        <f>AVERAGE(B73,B45,B101)</f>
-        <v>7.3731136666666655E-2</v>
-      </c>
-      <c r="C129" s="13">
-        <f t="shared" si="21"/>
-        <v>7.0073159999999995E-2</v>
+        <f>B128/8748</f>
+        <v>7.3731138545953367E-2</v>
+      </c>
+      <c r="C129" s="14">
+        <f>C128/8748</f>
+        <v>7.0073159579332425E-2</v>
       </c>
       <c r="D129" s="11"/>
       <c r="E129" s="11"/>
       <c r="F129" s="6"/>
       <c r="G129" s="11">
         <f t="shared" si="19"/>
-        <v>-3.6579766666666597E-3</v>
+        <v>-3.6579789666209422E-3</v>
       </c>
       <c r="H129" s="11"/>
       <c r="I129" s="11"/>
       <c r="J129" s="6"/>
       <c r="K129" s="10">
-        <f t="shared" si="22"/>
-        <v>-4.9612373171515282E-2</v>
+        <f t="shared" si="24"/>
+        <v>-4.9612403100775193E-2</v>
       </c>
       <c r="L129" s="10"/>
       <c r="M129" s="10"/>
@@ -4697,14 +4721,14 @@
       <c r="E132" s="11"/>
       <c r="F132" s="6"/>
       <c r="G132" s="11">
-        <f t="shared" ref="G132:G143" si="23">C132-B132</f>
+        <f t="shared" ref="G132:G143" si="25">C132-B132</f>
         <v>1.2576666666666014E-3</v>
       </c>
       <c r="H132" s="11"/>
       <c r="I132" s="11"/>
       <c r="J132" s="6"/>
       <c r="K132" s="10">
-        <f t="shared" ref="K132:K143" si="24">G132/B132</f>
+        <f t="shared" ref="K132:K143" si="26">G132/B132</f>
         <v>1.1218589139762878E-3</v>
       </c>
       <c r="L132" s="10"/>
@@ -4716,25 +4740,25 @@
         <v>44</v>
       </c>
       <c r="B133" s="1">
-        <f t="shared" ref="B133:B142" si="25">AVERAGE(B77,B49,B105)</f>
+        <f t="shared" ref="B133:B142" si="27">AVERAGE(B77,B49,B105)</f>
         <v>0.58927733333333332</v>
       </c>
       <c r="C133" s="11">
-        <f t="shared" ref="C133:C143" si="26">AVERAGE(C77,C49,C105)</f>
+        <f t="shared" ref="C133:C143" si="28">AVERAGE(C77,C49,C105)</f>
         <v>0.58984899999999996</v>
       </c>
       <c r="D133" s="11"/>
       <c r="E133" s="11"/>
       <c r="F133" s="6"/>
       <c r="G133" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>5.7166666666663701E-4</v>
       </c>
       <c r="H133" s="11"/>
       <c r="I133" s="11"/>
       <c r="J133" s="6"/>
       <c r="K133" s="10">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>9.7011480728933011E-4</v>
       </c>
       <c r="L133" s="10"/>
@@ -4746,26 +4770,26 @@
         <v>45</v>
       </c>
       <c r="B134" s="1">
-        <f t="shared" si="25"/>
-        <v>0.66666666666666663</v>
+        <f>MEDIAN(B78,B50,B106)</f>
+        <v>0</v>
       </c>
       <c r="C134" s="11">
-        <f t="shared" si="26"/>
-        <v>0.66666666666666663</v>
+        <f>MEDIAN(C78,C50,C106)</f>
+        <v>0</v>
       </c>
       <c r="D134" s="11"/>
       <c r="E134" s="11"/>
       <c r="F134" s="6"/>
       <c r="G134" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="H134" s="11"/>
       <c r="I134" s="11"/>
       <c r="J134" s="6"/>
-      <c r="K134" s="10">
-        <f t="shared" si="24"/>
-        <v>0</v>
+      <c r="K134" s="10" t="e">
+        <f t="shared" si="26"/>
+        <v>#DIV/0!</v>
       </c>
       <c r="L134" s="10"/>
       <c r="M134" s="10"/>
@@ -4776,26 +4800,26 @@
         <v>46</v>
       </c>
       <c r="B135" s="1">
-        <f t="shared" si="25"/>
-        <v>-0.66666666666666663</v>
+        <f>MEDIAN(B79,B51,B107)</f>
+        <v>0</v>
       </c>
       <c r="C135" s="11">
-        <f t="shared" si="26"/>
-        <v>-0.66666666666666663</v>
+        <f>MEDIAN(C79,C51,C107)</f>
+        <v>0</v>
       </c>
       <c r="D135" s="11"/>
       <c r="E135" s="11"/>
       <c r="F135" s="6"/>
       <c r="G135" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="H135" s="11"/>
       <c r="I135" s="11"/>
       <c r="J135" s="6"/>
-      <c r="K135" s="10">
-        <f t="shared" si="24"/>
-        <v>0</v>
+      <c r="K135" s="10" t="e">
+        <f t="shared" si="26"/>
+        <v>#DIV/0!</v>
       </c>
       <c r="L135" s="10"/>
       <c r="M135" s="10"/>
@@ -4806,25 +4830,25 @@
         <v>47</v>
       </c>
       <c r="B136" s="1">
-        <f t="shared" si="25"/>
-        <v>-1.3333333333333333</v>
+        <f>MIN(B80,B52,B108)</f>
+        <v>-3</v>
       </c>
       <c r="C136" s="11">
-        <f t="shared" si="26"/>
-        <v>-1.3333333333333333</v>
+        <f>MIN(C80,C52,C108)</f>
+        <v>-3</v>
       </c>
       <c r="D136" s="11"/>
       <c r="E136" s="11"/>
       <c r="F136" s="6"/>
       <c r="G136" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="H136" s="11"/>
       <c r="I136" s="11"/>
       <c r="J136" s="6"/>
       <c r="K136" s="10">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="L136" s="10"/>
@@ -4836,25 +4860,25 @@
         <v>48</v>
       </c>
       <c r="B137" s="1">
-        <f t="shared" si="25"/>
-        <v>0.66666666666666663</v>
+        <f>MAX(B81,B53,B109)</f>
+        <v>2</v>
       </c>
       <c r="C137" s="11">
-        <f t="shared" si="26"/>
-        <v>0.66666666666666663</v>
+        <f>MAX(C81,C53,C109)</f>
+        <v>2</v>
       </c>
       <c r="D137" s="11"/>
       <c r="E137" s="11"/>
       <c r="F137" s="6"/>
       <c r="G137" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="H137" s="11"/>
       <c r="I137" s="11"/>
       <c r="J137" s="6"/>
       <c r="K137" s="10">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="L137" s="10"/>
@@ -4866,25 +4890,25 @@
         <v>49</v>
       </c>
       <c r="B138" s="1">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>7.5959076666666663</v>
       </c>
       <c r="C138" s="11">
-        <f t="shared" si="26"/>
+        <f t="shared" si="28"/>
         <v>7.595793333333333</v>
       </c>
       <c r="D138" s="11"/>
       <c r="E138" s="11"/>
       <c r="F138" s="6"/>
       <c r="G138" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>-1.143333333333274E-4</v>
       </c>
       <c r="H138" s="11"/>
       <c r="I138" s="11"/>
       <c r="J138" s="6"/>
       <c r="K138" s="10">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>-1.5051964603922131E-5</v>
       </c>
       <c r="L138" s="10"/>
@@ -4896,25 +4920,25 @@
         <v>50</v>
       </c>
       <c r="B139" s="1">
-        <f t="shared" si="25"/>
-        <v>7.666666666666667</v>
+        <f>MEDIAN(B83,B55,B111)</f>
+        <v>8</v>
       </c>
       <c r="C139" s="11">
-        <f t="shared" si="26"/>
-        <v>7.666666666666667</v>
+        <f>MEDIAN(C83,C55,C111)</f>
+        <v>8</v>
       </c>
       <c r="D139" s="11"/>
       <c r="E139" s="11"/>
       <c r="F139" s="6"/>
       <c r="G139" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="H139" s="11"/>
       <c r="I139" s="11"/>
       <c r="J139" s="6"/>
       <c r="K139" s="10">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="L139" s="10"/>
@@ -4926,25 +4950,25 @@
         <v>51</v>
       </c>
       <c r="B140" s="1">
-        <f t="shared" si="25"/>
+        <f>MAX(B84,B56,B112)</f>
         <v>8</v>
       </c>
       <c r="C140" s="11">
-        <f t="shared" si="26"/>
+        <f>MAX(C84,C56,C112)</f>
         <v>8</v>
       </c>
       <c r="D140" s="11"/>
       <c r="E140" s="11"/>
       <c r="F140" s="6"/>
       <c r="G140" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="H140" s="11"/>
       <c r="I140" s="11"/>
       <c r="J140" s="6"/>
       <c r="K140" s="10">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="L140" s="10"/>
@@ -4956,25 +4980,25 @@
         <v>52</v>
       </c>
       <c r="B141" s="1">
-        <f t="shared" si="25"/>
-        <v>6.666666666666667</v>
+        <f>MIN(B85,B57,B113)</f>
+        <v>5</v>
       </c>
       <c r="C141" s="11">
-        <f t="shared" si="26"/>
-        <v>6.666666666666667</v>
+        <f>MIN(C85,C57,C113)</f>
+        <v>5</v>
       </c>
       <c r="D141" s="11"/>
       <c r="E141" s="11"/>
       <c r="F141" s="6"/>
       <c r="G141" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="H141" s="11"/>
       <c r="I141" s="11"/>
       <c r="J141" s="6"/>
       <c r="K141" s="10">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="L141" s="10"/>
@@ -4983,29 +5007,29 @@
     </row>
     <row r="142" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A142" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B142" s="1">
-        <f t="shared" si="25"/>
-        <v>1954.3333333333333</v>
+        <f>SUM(B86,B58,B114)</f>
+        <v>5863</v>
       </c>
       <c r="C142" s="11">
-        <f>AVERAGE(C86,C58,C114)</f>
-        <v>1954</v>
+        <f>SUM(C86,C58,C114)</f>
+        <v>5862</v>
       </c>
       <c r="D142" s="11"/>
       <c r="E142" s="11"/>
       <c r="F142" s="6"/>
       <c r="G142" s="11">
-        <f t="shared" si="23"/>
-        <v>-0.33333333333325754</v>
+        <f t="shared" si="25"/>
+        <v>-1</v>
       </c>
       <c r="H142" s="11"/>
       <c r="I142" s="11"/>
       <c r="J142" s="6"/>
       <c r="K142" s="10">
-        <f t="shared" si="24"/>
-        <v>-1.7056114617086348E-4</v>
+        <f t="shared" si="26"/>
+        <v>-1.7056114617090227E-4</v>
       </c>
       <c r="L142" s="10"/>
       <c r="M142" s="10"/>
@@ -5013,29 +5037,29 @@
     </row>
     <row r="143" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A143" s="3" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="B143" s="5">
-        <f>AVERAGE(B87,B59,B115)</f>
-        <v>0.67021033333333335</v>
-      </c>
-      <c r="C143" s="13">
-        <f t="shared" si="26"/>
-        <v>0.6700960199999999</v>
+        <f>B142/8748</f>
+        <v>0.6702103337905807</v>
+      </c>
+      <c r="C143" s="14">
+        <f>C142/8748</f>
+        <v>0.67009602194787377</v>
       </c>
       <c r="D143" s="11"/>
       <c r="E143" s="11"/>
       <c r="F143" s="6"/>
       <c r="G143" s="11">
-        <f t="shared" si="23"/>
-        <v>-1.1431333333344895E-4</v>
+        <f t="shared" si="25"/>
+        <v>-1.1431184270693784E-4</v>
       </c>
       <c r="H143" s="11"/>
       <c r="I143" s="11"/>
       <c r="J143" s="6"/>
       <c r="K143" s="10">
-        <f t="shared" si="24"/>
-        <v>-1.7056337040478677E-4</v>
+        <f t="shared" si="26"/>
+        <v>-1.7056114617095211E-4</v>
       </c>
       <c r="L143" s="10"/>
       <c r="M143" s="10"/>
@@ -5074,11 +5098,11 @@
       <c r="H145" s="11"/>
       <c r="I145" s="11"/>
       <c r="J145" s="6"/>
-      <c r="K145" s="15">
-        <v>0</v>
-      </c>
-      <c r="L145" s="15"/>
-      <c r="M145" s="15"/>
+      <c r="K145" s="13">
+        <v>0</v>
+      </c>
+      <c r="L145" s="13"/>
+      <c r="M145" s="13"/>
       <c r="N145" s="6"/>
     </row>
     <row r="146" spans="1:14" x14ac:dyDescent="0.2">
@@ -5327,7 +5351,7 @@
         <v>-8.0530056000001196</v>
       </c>
       <c r="H154" s="1">
-        <f t="shared" ref="H154" si="27">D154-B154</f>
+        <f t="shared" ref="H154" si="29">D154-B154</f>
         <v>33.1681319999999</v>
       </c>
       <c r="I154" s="1">
@@ -5340,7 +5364,7 @@
         <v>-8.4326779171183582E-3</v>
       </c>
       <c r="L154" s="5">
-        <f t="shared" ref="L154" si="28">H154/B154</f>
+        <f t="shared" ref="L154" si="30">H154/B154</f>
         <v>3.4731898642720645E-2</v>
       </c>
       <c r="M154" s="5">
@@ -5401,6 +5425,342 @@
     </row>
   </sheetData>
   <mergeCells count="360">
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="G59:I59"/>
+    <mergeCell ref="K59:M59"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="G56:I56"/>
+    <mergeCell ref="K56:M56"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="G57:I57"/>
+    <mergeCell ref="K57:M57"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="G58:I58"/>
+    <mergeCell ref="K58:M58"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="G53:I53"/>
+    <mergeCell ref="K53:M53"/>
+    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="G54:I54"/>
+    <mergeCell ref="K54:M54"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="G55:I55"/>
+    <mergeCell ref="K55:M55"/>
+    <mergeCell ref="C50:E50"/>
+    <mergeCell ref="G50:I50"/>
+    <mergeCell ref="K50:M50"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="G51:I51"/>
+    <mergeCell ref="K51:M51"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="G52:I52"/>
+    <mergeCell ref="K52:M52"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="G47:I47"/>
+    <mergeCell ref="K47:M47"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="G48:I48"/>
+    <mergeCell ref="K48:M48"/>
+    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="G49:I49"/>
+    <mergeCell ref="K49:M49"/>
+    <mergeCell ref="C43:E43"/>
+    <mergeCell ref="G43:I43"/>
+    <mergeCell ref="K43:M43"/>
+    <mergeCell ref="C44:E44"/>
+    <mergeCell ref="G44:I44"/>
+    <mergeCell ref="K44:M44"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="G45:I45"/>
+    <mergeCell ref="K45:M45"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="G40:I40"/>
+    <mergeCell ref="K40:M40"/>
+    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="G41:I41"/>
+    <mergeCell ref="K41:M41"/>
+    <mergeCell ref="C42:E42"/>
+    <mergeCell ref="G42:I42"/>
+    <mergeCell ref="K42:M42"/>
+    <mergeCell ref="C87:E87"/>
+    <mergeCell ref="G87:I87"/>
+    <mergeCell ref="K87:M87"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="K33:M33"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="K34:M34"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="K35:M35"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="G36:I36"/>
+    <mergeCell ref="K36:M36"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="G37:I37"/>
+    <mergeCell ref="K37:M37"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="G38:I38"/>
+    <mergeCell ref="K38:M38"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="G39:I39"/>
+    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="C84:E84"/>
+    <mergeCell ref="G84:I84"/>
+    <mergeCell ref="K84:M84"/>
+    <mergeCell ref="C85:E85"/>
+    <mergeCell ref="G85:I85"/>
+    <mergeCell ref="K85:M85"/>
+    <mergeCell ref="C86:E86"/>
+    <mergeCell ref="G86:I86"/>
+    <mergeCell ref="K86:M86"/>
+    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="G81:I81"/>
+    <mergeCell ref="K81:M81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="G82:I82"/>
+    <mergeCell ref="K82:M82"/>
+    <mergeCell ref="C83:E83"/>
+    <mergeCell ref="G83:I83"/>
+    <mergeCell ref="K83:M83"/>
+    <mergeCell ref="C78:E78"/>
+    <mergeCell ref="G78:I78"/>
+    <mergeCell ref="K78:M78"/>
+    <mergeCell ref="C79:E79"/>
+    <mergeCell ref="G79:I79"/>
+    <mergeCell ref="K79:M79"/>
+    <mergeCell ref="C80:E80"/>
+    <mergeCell ref="G80:I80"/>
+    <mergeCell ref="K80:M80"/>
+    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="G75:I75"/>
+    <mergeCell ref="K75:M75"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="G76:I76"/>
+    <mergeCell ref="K76:M76"/>
+    <mergeCell ref="C77:E77"/>
+    <mergeCell ref="G77:I77"/>
+    <mergeCell ref="K77:M77"/>
+    <mergeCell ref="C71:E71"/>
+    <mergeCell ref="G71:I71"/>
+    <mergeCell ref="K71:M71"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="G72:I72"/>
+    <mergeCell ref="K72:M72"/>
+    <mergeCell ref="C73:E73"/>
+    <mergeCell ref="G73:I73"/>
+    <mergeCell ref="K73:M73"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="G68:I68"/>
+    <mergeCell ref="K68:M68"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="G69:I69"/>
+    <mergeCell ref="K69:M69"/>
+    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="G70:I70"/>
+    <mergeCell ref="K70:M70"/>
+    <mergeCell ref="C115:E115"/>
+    <mergeCell ref="G115:I115"/>
+    <mergeCell ref="K115:M115"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="G61:I61"/>
+    <mergeCell ref="K61:M61"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="G62:I62"/>
+    <mergeCell ref="K62:M62"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="G63:I63"/>
+    <mergeCell ref="K63:M63"/>
+    <mergeCell ref="C64:E64"/>
+    <mergeCell ref="G64:I64"/>
+    <mergeCell ref="K64:M64"/>
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="G65:I65"/>
+    <mergeCell ref="K65:M65"/>
+    <mergeCell ref="C66:E66"/>
+    <mergeCell ref="G66:I66"/>
+    <mergeCell ref="K66:M66"/>
+    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="G67:I67"/>
+    <mergeCell ref="K67:M67"/>
+    <mergeCell ref="C112:E112"/>
+    <mergeCell ref="G112:I112"/>
+    <mergeCell ref="K112:M112"/>
+    <mergeCell ref="C113:E113"/>
+    <mergeCell ref="G113:I113"/>
+    <mergeCell ref="K113:M113"/>
+    <mergeCell ref="C114:E114"/>
+    <mergeCell ref="G114:I114"/>
+    <mergeCell ref="K114:M114"/>
+    <mergeCell ref="C109:E109"/>
+    <mergeCell ref="G109:I109"/>
+    <mergeCell ref="K109:M109"/>
+    <mergeCell ref="C110:E110"/>
+    <mergeCell ref="G110:I110"/>
+    <mergeCell ref="K110:M110"/>
+    <mergeCell ref="C111:E111"/>
+    <mergeCell ref="G111:I111"/>
+    <mergeCell ref="K111:M111"/>
+    <mergeCell ref="C106:E106"/>
+    <mergeCell ref="G106:I106"/>
+    <mergeCell ref="K106:M106"/>
+    <mergeCell ref="C107:E107"/>
+    <mergeCell ref="G107:I107"/>
+    <mergeCell ref="K107:M107"/>
+    <mergeCell ref="C108:E108"/>
+    <mergeCell ref="G108:I108"/>
+    <mergeCell ref="K108:M108"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="G103:I103"/>
+    <mergeCell ref="K103:M103"/>
+    <mergeCell ref="C104:E104"/>
+    <mergeCell ref="G104:I104"/>
+    <mergeCell ref="K104:M104"/>
+    <mergeCell ref="C105:E105"/>
+    <mergeCell ref="G105:I105"/>
+    <mergeCell ref="K105:M105"/>
+    <mergeCell ref="C99:E99"/>
+    <mergeCell ref="G99:I99"/>
+    <mergeCell ref="K99:M99"/>
+    <mergeCell ref="C100:E100"/>
+    <mergeCell ref="G100:I100"/>
+    <mergeCell ref="K100:M100"/>
+    <mergeCell ref="C101:E101"/>
+    <mergeCell ref="G101:I101"/>
+    <mergeCell ref="K101:M101"/>
+    <mergeCell ref="G95:I95"/>
+    <mergeCell ref="K95:M95"/>
+    <mergeCell ref="C96:E96"/>
+    <mergeCell ref="G96:I96"/>
+    <mergeCell ref="K96:M96"/>
+    <mergeCell ref="C97:E97"/>
+    <mergeCell ref="G97:I97"/>
+    <mergeCell ref="K97:M97"/>
+    <mergeCell ref="C98:E98"/>
+    <mergeCell ref="G98:I98"/>
+    <mergeCell ref="K98:M98"/>
+    <mergeCell ref="B117:E117"/>
+    <mergeCell ref="B131:E131"/>
+    <mergeCell ref="G131:I131"/>
+    <mergeCell ref="K131:M131"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="G89:I89"/>
+    <mergeCell ref="K89:M89"/>
+    <mergeCell ref="C90:E90"/>
+    <mergeCell ref="G90:I90"/>
+    <mergeCell ref="K90:M90"/>
+    <mergeCell ref="C91:E91"/>
+    <mergeCell ref="G91:I91"/>
+    <mergeCell ref="K91:M91"/>
+    <mergeCell ref="C92:E92"/>
+    <mergeCell ref="G92:I92"/>
+    <mergeCell ref="K92:M92"/>
+    <mergeCell ref="C93:E93"/>
+    <mergeCell ref="G93:I93"/>
+    <mergeCell ref="K93:M93"/>
+    <mergeCell ref="C94:E94"/>
+    <mergeCell ref="G94:I94"/>
+    <mergeCell ref="K94:M94"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="C127:E127"/>
+    <mergeCell ref="K133:M133"/>
+    <mergeCell ref="K143:M143"/>
+    <mergeCell ref="K135:M135"/>
+    <mergeCell ref="K136:M136"/>
+    <mergeCell ref="K137:M137"/>
+    <mergeCell ref="K138:M138"/>
+    <mergeCell ref="K139:M139"/>
+    <mergeCell ref="K117:M117"/>
+    <mergeCell ref="G117:I117"/>
+    <mergeCell ref="K122:M122"/>
+    <mergeCell ref="K123:M123"/>
+    <mergeCell ref="K124:M124"/>
+    <mergeCell ref="K125:M125"/>
+    <mergeCell ref="K126:M126"/>
+    <mergeCell ref="K127:M127"/>
+    <mergeCell ref="K128:M128"/>
+    <mergeCell ref="K129:M129"/>
+    <mergeCell ref="K132:M132"/>
+    <mergeCell ref="C128:E128"/>
+    <mergeCell ref="C129:E129"/>
+    <mergeCell ref="C137:E137"/>
+    <mergeCell ref="C141:E141"/>
+    <mergeCell ref="C142:E142"/>
+    <mergeCell ref="C143:E143"/>
+    <mergeCell ref="G132:I132"/>
+    <mergeCell ref="G133:I133"/>
+    <mergeCell ref="G134:I134"/>
+    <mergeCell ref="G135:I135"/>
+    <mergeCell ref="G136:I136"/>
+    <mergeCell ref="G137:I137"/>
+    <mergeCell ref="G138:I138"/>
+    <mergeCell ref="G139:I139"/>
+    <mergeCell ref="G140:I140"/>
+    <mergeCell ref="G141:I141"/>
+    <mergeCell ref="G142:I142"/>
+    <mergeCell ref="G143:I143"/>
+    <mergeCell ref="C136:E136"/>
+    <mergeCell ref="B147:E147"/>
+    <mergeCell ref="B148:E148"/>
+    <mergeCell ref="B149:E149"/>
+    <mergeCell ref="B150:E150"/>
+    <mergeCell ref="C138:E138"/>
+    <mergeCell ref="C139:E139"/>
+    <mergeCell ref="C140:E140"/>
+    <mergeCell ref="G129:I129"/>
+    <mergeCell ref="C132:E132"/>
+    <mergeCell ref="C133:E133"/>
+    <mergeCell ref="C134:E134"/>
+    <mergeCell ref="C135:E135"/>
+    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="B145:E145"/>
+    <mergeCell ref="G118:I118"/>
+    <mergeCell ref="G119:I119"/>
+    <mergeCell ref="G120:I120"/>
+    <mergeCell ref="G121:I121"/>
+    <mergeCell ref="G122:I122"/>
+    <mergeCell ref="G123:I123"/>
+    <mergeCell ref="G124:I124"/>
+    <mergeCell ref="G125:I125"/>
+    <mergeCell ref="G126:I126"/>
+    <mergeCell ref="K145:M145"/>
+    <mergeCell ref="C118:E118"/>
+    <mergeCell ref="C119:E119"/>
+    <mergeCell ref="C120:E120"/>
+    <mergeCell ref="C121:E121"/>
+    <mergeCell ref="C122:E122"/>
+    <mergeCell ref="C123:E123"/>
+    <mergeCell ref="C124:E124"/>
+    <mergeCell ref="C125:E125"/>
+    <mergeCell ref="C126:E126"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="B153:D153"/>
+    <mergeCell ref="B155:D155"/>
+    <mergeCell ref="B151:D151"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="G127:I127"/>
+    <mergeCell ref="G128:I128"/>
+    <mergeCell ref="B152:E152"/>
+    <mergeCell ref="G145:I145"/>
+    <mergeCell ref="G146:I146"/>
+    <mergeCell ref="G147:I147"/>
+    <mergeCell ref="G148:I148"/>
+    <mergeCell ref="G149:I149"/>
+    <mergeCell ref="G150:I150"/>
+    <mergeCell ref="G152:I152"/>
+    <mergeCell ref="B146:E146"/>
     <mergeCell ref="L7:M7"/>
     <mergeCell ref="L8:M8"/>
     <mergeCell ref="L9:M9"/>
@@ -5425,342 +5785,6 @@
     <mergeCell ref="K119:M119"/>
     <mergeCell ref="K120:M120"/>
     <mergeCell ref="K121:M121"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="B153:D153"/>
-    <mergeCell ref="B155:D155"/>
-    <mergeCell ref="B151:D151"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="G127:I127"/>
-    <mergeCell ref="G128:I128"/>
-    <mergeCell ref="B152:E152"/>
-    <mergeCell ref="G145:I145"/>
-    <mergeCell ref="G146:I146"/>
-    <mergeCell ref="G147:I147"/>
-    <mergeCell ref="G148:I148"/>
-    <mergeCell ref="G149:I149"/>
-    <mergeCell ref="G150:I150"/>
-    <mergeCell ref="G152:I152"/>
-    <mergeCell ref="B146:E146"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="B145:E145"/>
-    <mergeCell ref="G118:I118"/>
-    <mergeCell ref="G119:I119"/>
-    <mergeCell ref="G120:I120"/>
-    <mergeCell ref="G121:I121"/>
-    <mergeCell ref="G122:I122"/>
-    <mergeCell ref="G123:I123"/>
-    <mergeCell ref="G124:I124"/>
-    <mergeCell ref="G125:I125"/>
-    <mergeCell ref="G126:I126"/>
-    <mergeCell ref="K145:M145"/>
-    <mergeCell ref="C118:E118"/>
-    <mergeCell ref="C119:E119"/>
-    <mergeCell ref="C120:E120"/>
-    <mergeCell ref="C121:E121"/>
-    <mergeCell ref="C122:E122"/>
-    <mergeCell ref="C123:E123"/>
-    <mergeCell ref="C124:E124"/>
-    <mergeCell ref="C125:E125"/>
-    <mergeCell ref="C126:E126"/>
-    <mergeCell ref="B147:E147"/>
-    <mergeCell ref="B148:E148"/>
-    <mergeCell ref="B149:E149"/>
-    <mergeCell ref="B150:E150"/>
-    <mergeCell ref="C138:E138"/>
-    <mergeCell ref="C139:E139"/>
-    <mergeCell ref="C140:E140"/>
-    <mergeCell ref="G129:I129"/>
-    <mergeCell ref="C132:E132"/>
-    <mergeCell ref="C133:E133"/>
-    <mergeCell ref="C134:E134"/>
-    <mergeCell ref="C135:E135"/>
-    <mergeCell ref="C128:E128"/>
-    <mergeCell ref="C129:E129"/>
-    <mergeCell ref="C137:E137"/>
-    <mergeCell ref="C141:E141"/>
-    <mergeCell ref="C142:E142"/>
-    <mergeCell ref="C143:E143"/>
-    <mergeCell ref="G132:I132"/>
-    <mergeCell ref="G133:I133"/>
-    <mergeCell ref="G134:I134"/>
-    <mergeCell ref="G135:I135"/>
-    <mergeCell ref="G136:I136"/>
-    <mergeCell ref="G137:I137"/>
-    <mergeCell ref="G138:I138"/>
-    <mergeCell ref="G139:I139"/>
-    <mergeCell ref="G140:I140"/>
-    <mergeCell ref="G141:I141"/>
-    <mergeCell ref="G142:I142"/>
-    <mergeCell ref="G143:I143"/>
-    <mergeCell ref="C136:E136"/>
-    <mergeCell ref="K133:M133"/>
-    <mergeCell ref="K143:M143"/>
-    <mergeCell ref="K135:M135"/>
-    <mergeCell ref="K136:M136"/>
-    <mergeCell ref="K137:M137"/>
-    <mergeCell ref="K138:M138"/>
-    <mergeCell ref="K139:M139"/>
-    <mergeCell ref="K117:M117"/>
-    <mergeCell ref="G117:I117"/>
-    <mergeCell ref="K122:M122"/>
-    <mergeCell ref="K123:M123"/>
-    <mergeCell ref="K124:M124"/>
-    <mergeCell ref="K125:M125"/>
-    <mergeCell ref="K126:M126"/>
-    <mergeCell ref="K127:M127"/>
-    <mergeCell ref="K128:M128"/>
-    <mergeCell ref="K129:M129"/>
-    <mergeCell ref="K132:M132"/>
-    <mergeCell ref="B117:E117"/>
-    <mergeCell ref="B131:E131"/>
-    <mergeCell ref="G131:I131"/>
-    <mergeCell ref="K131:M131"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="G89:I89"/>
-    <mergeCell ref="K89:M89"/>
-    <mergeCell ref="C90:E90"/>
-    <mergeCell ref="G90:I90"/>
-    <mergeCell ref="K90:M90"/>
-    <mergeCell ref="C91:E91"/>
-    <mergeCell ref="G91:I91"/>
-    <mergeCell ref="K91:M91"/>
-    <mergeCell ref="C92:E92"/>
-    <mergeCell ref="G92:I92"/>
-    <mergeCell ref="K92:M92"/>
-    <mergeCell ref="C93:E93"/>
-    <mergeCell ref="G93:I93"/>
-    <mergeCell ref="K93:M93"/>
-    <mergeCell ref="C94:E94"/>
-    <mergeCell ref="G94:I94"/>
-    <mergeCell ref="K94:M94"/>
-    <mergeCell ref="C95:E95"/>
-    <mergeCell ref="C127:E127"/>
-    <mergeCell ref="G95:I95"/>
-    <mergeCell ref="K95:M95"/>
-    <mergeCell ref="C96:E96"/>
-    <mergeCell ref="G96:I96"/>
-    <mergeCell ref="K96:M96"/>
-    <mergeCell ref="C97:E97"/>
-    <mergeCell ref="G97:I97"/>
-    <mergeCell ref="K97:M97"/>
-    <mergeCell ref="C98:E98"/>
-    <mergeCell ref="G98:I98"/>
-    <mergeCell ref="K98:M98"/>
-    <mergeCell ref="C99:E99"/>
-    <mergeCell ref="G99:I99"/>
-    <mergeCell ref="K99:M99"/>
-    <mergeCell ref="C100:E100"/>
-    <mergeCell ref="G100:I100"/>
-    <mergeCell ref="K100:M100"/>
-    <mergeCell ref="C101:E101"/>
-    <mergeCell ref="G101:I101"/>
-    <mergeCell ref="K101:M101"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="G103:I103"/>
-    <mergeCell ref="K103:M103"/>
-    <mergeCell ref="C104:E104"/>
-    <mergeCell ref="G104:I104"/>
-    <mergeCell ref="K104:M104"/>
-    <mergeCell ref="C105:E105"/>
-    <mergeCell ref="G105:I105"/>
-    <mergeCell ref="K105:M105"/>
-    <mergeCell ref="C106:E106"/>
-    <mergeCell ref="G106:I106"/>
-    <mergeCell ref="K106:M106"/>
-    <mergeCell ref="C107:E107"/>
-    <mergeCell ref="G107:I107"/>
-    <mergeCell ref="K107:M107"/>
-    <mergeCell ref="C108:E108"/>
-    <mergeCell ref="G108:I108"/>
-    <mergeCell ref="K108:M108"/>
-    <mergeCell ref="C109:E109"/>
-    <mergeCell ref="G109:I109"/>
-    <mergeCell ref="K109:M109"/>
-    <mergeCell ref="C110:E110"/>
-    <mergeCell ref="G110:I110"/>
-    <mergeCell ref="K110:M110"/>
-    <mergeCell ref="C111:E111"/>
-    <mergeCell ref="G111:I111"/>
-    <mergeCell ref="K111:M111"/>
-    <mergeCell ref="C112:E112"/>
-    <mergeCell ref="G112:I112"/>
-    <mergeCell ref="K112:M112"/>
-    <mergeCell ref="C113:E113"/>
-    <mergeCell ref="G113:I113"/>
-    <mergeCell ref="K113:M113"/>
-    <mergeCell ref="C114:E114"/>
-    <mergeCell ref="G114:I114"/>
-    <mergeCell ref="K114:M114"/>
-    <mergeCell ref="C115:E115"/>
-    <mergeCell ref="G115:I115"/>
-    <mergeCell ref="K115:M115"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="G61:I61"/>
-    <mergeCell ref="K61:M61"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="G62:I62"/>
-    <mergeCell ref="K62:M62"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="G63:I63"/>
-    <mergeCell ref="K63:M63"/>
-    <mergeCell ref="C64:E64"/>
-    <mergeCell ref="G64:I64"/>
-    <mergeCell ref="K64:M64"/>
-    <mergeCell ref="C65:E65"/>
-    <mergeCell ref="G65:I65"/>
-    <mergeCell ref="K65:M65"/>
-    <mergeCell ref="C66:E66"/>
-    <mergeCell ref="G66:I66"/>
-    <mergeCell ref="K66:M66"/>
-    <mergeCell ref="C67:E67"/>
-    <mergeCell ref="G67:I67"/>
-    <mergeCell ref="K67:M67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="G68:I68"/>
-    <mergeCell ref="K68:M68"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="G69:I69"/>
-    <mergeCell ref="K69:M69"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="G70:I70"/>
-    <mergeCell ref="K70:M70"/>
-    <mergeCell ref="C71:E71"/>
-    <mergeCell ref="G71:I71"/>
-    <mergeCell ref="K71:M71"/>
-    <mergeCell ref="C72:E72"/>
-    <mergeCell ref="G72:I72"/>
-    <mergeCell ref="K72:M72"/>
-    <mergeCell ref="C73:E73"/>
-    <mergeCell ref="G73:I73"/>
-    <mergeCell ref="K73:M73"/>
-    <mergeCell ref="B75:E75"/>
-    <mergeCell ref="G75:I75"/>
-    <mergeCell ref="K75:M75"/>
-    <mergeCell ref="C76:E76"/>
-    <mergeCell ref="G76:I76"/>
-    <mergeCell ref="K76:M76"/>
-    <mergeCell ref="C77:E77"/>
-    <mergeCell ref="G77:I77"/>
-    <mergeCell ref="K77:M77"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="G78:I78"/>
-    <mergeCell ref="K78:M78"/>
-    <mergeCell ref="C79:E79"/>
-    <mergeCell ref="G79:I79"/>
-    <mergeCell ref="K79:M79"/>
-    <mergeCell ref="C80:E80"/>
-    <mergeCell ref="G80:I80"/>
-    <mergeCell ref="K80:M80"/>
-    <mergeCell ref="C81:E81"/>
-    <mergeCell ref="G81:I81"/>
-    <mergeCell ref="K81:M81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="G82:I82"/>
-    <mergeCell ref="K82:M82"/>
-    <mergeCell ref="C83:E83"/>
-    <mergeCell ref="G83:I83"/>
-    <mergeCell ref="K83:M83"/>
-    <mergeCell ref="C84:E84"/>
-    <mergeCell ref="G84:I84"/>
-    <mergeCell ref="K84:M84"/>
-    <mergeCell ref="C85:E85"/>
-    <mergeCell ref="G85:I85"/>
-    <mergeCell ref="K85:M85"/>
-    <mergeCell ref="C86:E86"/>
-    <mergeCell ref="G86:I86"/>
-    <mergeCell ref="K86:M86"/>
-    <mergeCell ref="C87:E87"/>
-    <mergeCell ref="G87:I87"/>
-    <mergeCell ref="K87:M87"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="K33:M33"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="K34:M34"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="K35:M35"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="G36:I36"/>
-    <mergeCell ref="K36:M36"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="G37:I37"/>
-    <mergeCell ref="K37:M37"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="G38:I38"/>
-    <mergeCell ref="K38:M38"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="G39:I39"/>
-    <mergeCell ref="K39:M39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="G40:I40"/>
-    <mergeCell ref="K40:M40"/>
-    <mergeCell ref="C41:E41"/>
-    <mergeCell ref="G41:I41"/>
-    <mergeCell ref="K41:M41"/>
-    <mergeCell ref="C42:E42"/>
-    <mergeCell ref="G42:I42"/>
-    <mergeCell ref="K42:M42"/>
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="G43:I43"/>
-    <mergeCell ref="K43:M43"/>
-    <mergeCell ref="C44:E44"/>
-    <mergeCell ref="G44:I44"/>
-    <mergeCell ref="K44:M44"/>
-    <mergeCell ref="C45:E45"/>
-    <mergeCell ref="G45:I45"/>
-    <mergeCell ref="K45:M45"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="G47:I47"/>
-    <mergeCell ref="K47:M47"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="G48:I48"/>
-    <mergeCell ref="K48:M48"/>
-    <mergeCell ref="C49:E49"/>
-    <mergeCell ref="G49:I49"/>
-    <mergeCell ref="K49:M49"/>
-    <mergeCell ref="C50:E50"/>
-    <mergeCell ref="G50:I50"/>
-    <mergeCell ref="K50:M50"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="G51:I51"/>
-    <mergeCell ref="K51:M51"/>
-    <mergeCell ref="C52:E52"/>
-    <mergeCell ref="G52:I52"/>
-    <mergeCell ref="K52:M52"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="G53:I53"/>
-    <mergeCell ref="K53:M53"/>
-    <mergeCell ref="C54:E54"/>
-    <mergeCell ref="G54:I54"/>
-    <mergeCell ref="K54:M54"/>
-    <mergeCell ref="C55:E55"/>
-    <mergeCell ref="G55:I55"/>
-    <mergeCell ref="K55:M55"/>
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="G59:I59"/>
-    <mergeCell ref="K59:M59"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="G56:I56"/>
-    <mergeCell ref="K56:M56"/>
-    <mergeCell ref="C57:E57"/>
-    <mergeCell ref="G57:I57"/>
-    <mergeCell ref="K57:M57"/>
-    <mergeCell ref="C58:E58"/>
-    <mergeCell ref="G58:I58"/>
-    <mergeCell ref="K58:M58"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>